<commit_message>
Nueva estética de La Reina de la Queja y accesos directos a las secciones
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014cQS814DmisHJYTJthjhHq
</commit_message>
<xml_diff>
--- a/Finanzas_Proyecto.xlsx
+++ b/Finanzas_Proyecto.xlsx
@@ -79,7 +79,7 @@
     <t xml:space="preserve">RIFA DEL PESO</t>
   </si>
   <si>
-    <t xml:space="preserve">Celdas celestes = para completar. Anotá cada recaudo (o un solo total) en una fila. La fila 5 es un ejemplo: reemplazala.</t>
+    <t xml:space="preserve">Celdas rosas = para completar. Anotá cada recaudo (o un solo total) en una fila. La fila 5 es un ejemplo: reemplazala.</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha</t>
@@ -100,7 +100,7 @@
     <t xml:space="preserve">VENTA DE REMERAS</t>
   </si>
   <si>
-    <t xml:space="preserve">Celdas celestes = para completar. Una fila por venta o tanda. La fila 5 es un ejemplo: reemplazala.</t>
+    <t xml:space="preserve">Celdas rosas = para completar. Una fila por venta o tanda. La fila 5 es un ejemplo: reemplazala.</t>
   </si>
   <si>
     <t xml:space="preserve">Detalle (talle, comprador, etc.)</t>
@@ -124,7 +124,7 @@
     <t xml:space="preserve">Precio promedio</t>
   </si>
   <si>
-    <t xml:space="preserve">Celdas celestes = para completar. Elegí la categoría del menú desplegable. La fila 5 es un ejemplo: reemplazala.</t>
+    <t xml:space="preserve">Celdas rosas = para completar. Elegí la categoría del menú desplegable. La fila 5 es un ejemplo: reemplazala.</t>
   </si>
   <si>
     <t xml:space="preserve">Categoría</t>
@@ -255,13 +255,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE4F1"/>
-        <bgColor rgb="FFE9DDF7"/>
+        <bgColor rgb="FFFFE9F5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE3F4FC"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <fgColor rgb="FFFFE9F5"/>
+        <bgColor rgb="FFFCE4F1"/>
       </patternFill>
     </fill>
   </fills>
@@ -432,8 +432,8 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FFC2185B"/>
+      <rgbColor rgb="FFFFE9F5"/>
       <rgbColor rgb="FFFCE4F1"/>
-      <rgbColor rgb="FFE3F4FC"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFE04F9A"/>
       <rgbColor rgb="FF0066CC"/>

</xml_diff>

<commit_message>
Más estrellas, frutillitas en los botones, columna Componente y categoría Comida
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014cQS814DmisHJYTJthjhHq
</commit_message>
<xml_diff>
--- a/Finanzas_Proyecto.xlsx
+++ b/Finanzas_Proyecto.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="42">
   <si>
     <t xml:space="preserve">FINANZAS DEL PROYECTO</t>
   </si>
@@ -67,6 +67,9 @@
     <t xml:space="preserve">Audio</t>
   </si>
   <si>
+    <t xml:space="preserve">Comida</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTAL GASTOS</t>
   </si>
   <si>
@@ -79,10 +82,13 @@
     <t xml:space="preserve">RIFA DEL PESO</t>
   </si>
   <si>
-    <t xml:space="preserve">Celdas rosas = para completar. Anotá cada recaudo (o un solo total) en una fila. La fila 5 es un ejemplo: reemplazala.</t>
+    <t xml:space="preserve">Celdas rosas = para completar. Una fila por recaudo; elegí el componente del menú. La fila 5 es un ejemplo: reemplazala.</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Componente</t>
   </si>
   <si>
     <t xml:space="preserve">Detalle</t>
@@ -94,13 +100,16 @@
     <t xml:space="preserve">TOTAL RIFA</t>
   </si>
   <si>
+    <t xml:space="preserve">Cami</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ejemplo: recaudo rifa del peso</t>
   </si>
   <si>
     <t xml:space="preserve">VENTA DE REMERAS</t>
   </si>
   <si>
-    <t xml:space="preserve">Celdas rosas = para completar. Una fila por venta o tanda. La fila 5 es un ejemplo: reemplazala.</t>
+    <t xml:space="preserve">Celdas rosas = para completar. Una fila por venta o tanda; elegí el componente del menú. La fila 5 es un ejemplo: reemplazala.</t>
   </si>
   <si>
     <t xml:space="preserve">Detalle (talle, comprador, etc.)</t>
@@ -113,6 +122,9 @@
   </si>
   <si>
     <t xml:space="preserve">TOTAL UNIDADES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luci</t>
   </si>
   <si>
     <t xml:space="preserve">Ejemplo: 3 remeras talle M</t>
@@ -655,7 +667,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -683,7 +695,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="n">
-        <f aca="false">'Rifa del Peso'!F4</f>
+        <f aca="false">'Rifa del Peso'!G4</f>
         <v>25000</v>
       </c>
     </row>
@@ -692,7 +704,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="n">
-        <f aca="false">Remeras!G5</f>
+        <f aca="false">Remeras!H5</f>
         <v>30000</v>
       </c>
     </row>
@@ -701,7 +713,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="6" t="n">
-        <f aca="false">Remeras!G4</f>
+        <f aca="false">Remeras!H4</f>
         <v>3</v>
       </c>
     </row>
@@ -775,26 +787,35 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="s">
+      <c r="A17" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="8" t="n">
-        <f aca="false">SUM(B11:B16)</f>
+      <c r="B17" s="5" t="n">
+        <f aca="false">Gastos!G11</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" s="8" t="n">
+        <f aca="false">SUM(B11:B17)</f>
         <v>12000</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B19" s="3"/>
-    </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
+      <c r="A20" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="10" t="n">
-        <f aca="false">B8-B17</f>
+      <c r="B20" s="3"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="10" t="n">
+        <f aca="false">B8-B18</f>
         <v>43000</v>
       </c>
     </row>
@@ -814,41 +835,45 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F204"/>
+  <dimension ref="A1:G204"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="F4" s="13" t="n">
-        <f aca="false">SUM(C5:C204)</f>
+      <c r="D4" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="13" t="n">
+        <f aca="false">SUM(D5:D204)</f>
         <v>25000</v>
       </c>
     </row>
@@ -857,1008 +882,1216 @@
         <v>46310</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="16" t="n">
         <v>25000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14"/>
       <c r="B6" s="15"/>
-      <c r="C6" s="16"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="16"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14"/>
       <c r="B7" s="15"/>
-      <c r="C7" s="16"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="16"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14"/>
       <c r="B8" s="15"/>
-      <c r="C8" s="16"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14"/>
       <c r="B9" s="15"/>
-      <c r="C9" s="16"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="16"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14"/>
       <c r="B10" s="15"/>
-      <c r="C10" s="16"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="16"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14"/>
       <c r="B11" s="15"/>
-      <c r="C11" s="16"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="16"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14"/>
       <c r="B12" s="15"/>
-      <c r="C12" s="16"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="16"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14"/>
       <c r="B13" s="15"/>
-      <c r="C13" s="16"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="16"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14"/>
       <c r="B14" s="15"/>
-      <c r="C14" s="16"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="16"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14"/>
       <c r="B15" s="15"/>
-      <c r="C15" s="16"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="16"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14"/>
       <c r="B16" s="15"/>
-      <c r="C16" s="16"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="16"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14"/>
       <c r="B17" s="15"/>
-      <c r="C17" s="16"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="16"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14"/>
       <c r="B18" s="15"/>
-      <c r="C18" s="16"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="16"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14"/>
       <c r="B19" s="15"/>
-      <c r="C19" s="16"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="16"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14"/>
       <c r="B20" s="15"/>
-      <c r="C20" s="16"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="16"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14"/>
       <c r="B21" s="15"/>
-      <c r="C21" s="16"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="16"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14"/>
       <c r="B22" s="15"/>
-      <c r="C22" s="16"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="16"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14"/>
       <c r="B23" s="15"/>
-      <c r="C23" s="16"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="16"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14"/>
       <c r="B24" s="15"/>
-      <c r="C24" s="16"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="16"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14"/>
       <c r="B25" s="15"/>
-      <c r="C25" s="16"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="16"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14"/>
       <c r="B26" s="15"/>
-      <c r="C26" s="16"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="16"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14"/>
       <c r="B27" s="15"/>
-      <c r="C27" s="16"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="16"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14"/>
       <c r="B28" s="15"/>
-      <c r="C28" s="16"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="16"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14"/>
       <c r="B29" s="15"/>
-      <c r="C29" s="16"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="16"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14"/>
       <c r="B30" s="15"/>
-      <c r="C30" s="16"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="16"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14"/>
       <c r="B31" s="15"/>
-      <c r="C31" s="16"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="16"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14"/>
       <c r="B32" s="15"/>
-      <c r="C32" s="16"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="16"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14"/>
       <c r="B33" s="15"/>
-      <c r="C33" s="16"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="16"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14"/>
       <c r="B34" s="15"/>
-      <c r="C34" s="16"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="16"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="14"/>
       <c r="B35" s="15"/>
-      <c r="C35" s="16"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="16"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="14"/>
       <c r="B36" s="15"/>
-      <c r="C36" s="16"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="16"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14"/>
       <c r="B37" s="15"/>
-      <c r="C37" s="16"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="16"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14"/>
       <c r="B38" s="15"/>
-      <c r="C38" s="16"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="16"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="14"/>
       <c r="B39" s="15"/>
-      <c r="C39" s="16"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="16"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="14"/>
       <c r="B40" s="15"/>
-      <c r="C40" s="16"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="16"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="14"/>
       <c r="B41" s="15"/>
-      <c r="C41" s="16"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="16"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14"/>
       <c r="B42" s="15"/>
-      <c r="C42" s="16"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="16"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="14"/>
       <c r="B43" s="15"/>
-      <c r="C43" s="16"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="16"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="14"/>
       <c r="B44" s="15"/>
-      <c r="C44" s="16"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="16"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="14"/>
       <c r="B45" s="15"/>
-      <c r="C45" s="16"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="16"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="14"/>
       <c r="B46" s="15"/>
-      <c r="C46" s="16"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="16"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="14"/>
       <c r="B47" s="15"/>
-      <c r="C47" s="16"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="16"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="14"/>
       <c r="B48" s="15"/>
-      <c r="C48" s="16"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="16"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="14"/>
       <c r="B49" s="15"/>
-      <c r="C49" s="16"/>
+      <c r="C49" s="15"/>
+      <c r="D49" s="16"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="14"/>
       <c r="B50" s="15"/>
-      <c r="C50" s="16"/>
+      <c r="C50" s="15"/>
+      <c r="D50" s="16"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="14"/>
       <c r="B51" s="15"/>
-      <c r="C51" s="16"/>
+      <c r="C51" s="15"/>
+      <c r="D51" s="16"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="14"/>
       <c r="B52" s="15"/>
-      <c r="C52" s="16"/>
+      <c r="C52" s="15"/>
+      <c r="D52" s="16"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="14"/>
       <c r="B53" s="15"/>
-      <c r="C53" s="16"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="16"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="14"/>
       <c r="B54" s="15"/>
-      <c r="C54" s="16"/>
+      <c r="C54" s="15"/>
+      <c r="D54" s="16"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="14"/>
       <c r="B55" s="15"/>
-      <c r="C55" s="16"/>
+      <c r="C55" s="15"/>
+      <c r="D55" s="16"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="14"/>
       <c r="B56" s="15"/>
-      <c r="C56" s="16"/>
+      <c r="C56" s="15"/>
+      <c r="D56" s="16"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="14"/>
       <c r="B57" s="15"/>
-      <c r="C57" s="16"/>
+      <c r="C57" s="15"/>
+      <c r="D57" s="16"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="14"/>
       <c r="B58" s="15"/>
-      <c r="C58" s="16"/>
+      <c r="C58" s="15"/>
+      <c r="D58" s="16"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="14"/>
       <c r="B59" s="15"/>
-      <c r="C59" s="16"/>
+      <c r="C59" s="15"/>
+      <c r="D59" s="16"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="14"/>
       <c r="B60" s="15"/>
-      <c r="C60" s="16"/>
+      <c r="C60" s="15"/>
+      <c r="D60" s="16"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="14"/>
       <c r="B61" s="15"/>
-      <c r="C61" s="16"/>
+      <c r="C61" s="15"/>
+      <c r="D61" s="16"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="14"/>
       <c r="B62" s="15"/>
-      <c r="C62" s="16"/>
+      <c r="C62" s="15"/>
+      <c r="D62" s="16"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="14"/>
       <c r="B63" s="15"/>
-      <c r="C63" s="16"/>
+      <c r="C63" s="15"/>
+      <c r="D63" s="16"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="14"/>
       <c r="B64" s="15"/>
-      <c r="C64" s="16"/>
+      <c r="C64" s="15"/>
+      <c r="D64" s="16"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="14"/>
       <c r="B65" s="15"/>
-      <c r="C65" s="16"/>
+      <c r="C65" s="15"/>
+      <c r="D65" s="16"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="14"/>
       <c r="B66" s="15"/>
-      <c r="C66" s="16"/>
+      <c r="C66" s="15"/>
+      <c r="D66" s="16"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="14"/>
       <c r="B67" s="15"/>
-      <c r="C67" s="16"/>
+      <c r="C67" s="15"/>
+      <c r="D67" s="16"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="14"/>
       <c r="B68" s="15"/>
-      <c r="C68" s="16"/>
+      <c r="C68" s="15"/>
+      <c r="D68" s="16"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="14"/>
       <c r="B69" s="15"/>
-      <c r="C69" s="16"/>
+      <c r="C69" s="15"/>
+      <c r="D69" s="16"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="14"/>
       <c r="B70" s="15"/>
-      <c r="C70" s="16"/>
+      <c r="C70" s="15"/>
+      <c r="D70" s="16"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="14"/>
       <c r="B71" s="15"/>
-      <c r="C71" s="16"/>
+      <c r="C71" s="15"/>
+      <c r="D71" s="16"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="14"/>
       <c r="B72" s="15"/>
-      <c r="C72" s="16"/>
+      <c r="C72" s="15"/>
+      <c r="D72" s="16"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="14"/>
       <c r="B73" s="15"/>
-      <c r="C73" s="16"/>
+      <c r="C73" s="15"/>
+      <c r="D73" s="16"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="14"/>
       <c r="B74" s="15"/>
-      <c r="C74" s="16"/>
+      <c r="C74" s="15"/>
+      <c r="D74" s="16"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="14"/>
       <c r="B75" s="15"/>
-      <c r="C75" s="16"/>
+      <c r="C75" s="15"/>
+      <c r="D75" s="16"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="14"/>
       <c r="B76" s="15"/>
-      <c r="C76" s="16"/>
+      <c r="C76" s="15"/>
+      <c r="D76" s="16"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="14"/>
       <c r="B77" s="15"/>
-      <c r="C77" s="16"/>
+      <c r="C77" s="15"/>
+      <c r="D77" s="16"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="14"/>
       <c r="B78" s="15"/>
-      <c r="C78" s="16"/>
+      <c r="C78" s="15"/>
+      <c r="D78" s="16"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="14"/>
       <c r="B79" s="15"/>
-      <c r="C79" s="16"/>
+      <c r="C79" s="15"/>
+      <c r="D79" s="16"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="14"/>
       <c r="B80" s="15"/>
-      <c r="C80" s="16"/>
+      <c r="C80" s="15"/>
+      <c r="D80" s="16"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="14"/>
       <c r="B81" s="15"/>
-      <c r="C81" s="16"/>
+      <c r="C81" s="15"/>
+      <c r="D81" s="16"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="14"/>
       <c r="B82" s="15"/>
-      <c r="C82" s="16"/>
+      <c r="C82" s="15"/>
+      <c r="D82" s="16"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="14"/>
       <c r="B83" s="15"/>
-      <c r="C83" s="16"/>
+      <c r="C83" s="15"/>
+      <c r="D83" s="16"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="14"/>
       <c r="B84" s="15"/>
-      <c r="C84" s="16"/>
+      <c r="C84" s="15"/>
+      <c r="D84" s="16"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="14"/>
       <c r="B85" s="15"/>
-      <c r="C85" s="16"/>
+      <c r="C85" s="15"/>
+      <c r="D85" s="16"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="14"/>
       <c r="B86" s="15"/>
-      <c r="C86" s="16"/>
+      <c r="C86" s="15"/>
+      <c r="D86" s="16"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="14"/>
       <c r="B87" s="15"/>
-      <c r="C87" s="16"/>
+      <c r="C87" s="15"/>
+      <c r="D87" s="16"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="14"/>
       <c r="B88" s="15"/>
-      <c r="C88" s="16"/>
+      <c r="C88" s="15"/>
+      <c r="D88" s="16"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="14"/>
       <c r="B89" s="15"/>
-      <c r="C89" s="16"/>
+      <c r="C89" s="15"/>
+      <c r="D89" s="16"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="14"/>
       <c r="B90" s="15"/>
-      <c r="C90" s="16"/>
+      <c r="C90" s="15"/>
+      <c r="D90" s="16"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="14"/>
       <c r="B91" s="15"/>
-      <c r="C91" s="16"/>
+      <c r="C91" s="15"/>
+      <c r="D91" s="16"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="14"/>
       <c r="B92" s="15"/>
-      <c r="C92" s="16"/>
+      <c r="C92" s="15"/>
+      <c r="D92" s="16"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="14"/>
       <c r="B93" s="15"/>
-      <c r="C93" s="16"/>
+      <c r="C93" s="15"/>
+      <c r="D93" s="16"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="14"/>
       <c r="B94" s="15"/>
-      <c r="C94" s="16"/>
+      <c r="C94" s="15"/>
+      <c r="D94" s="16"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="14"/>
       <c r="B95" s="15"/>
-      <c r="C95" s="16"/>
+      <c r="C95" s="15"/>
+      <c r="D95" s="16"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="14"/>
       <c r="B96" s="15"/>
-      <c r="C96" s="16"/>
+      <c r="C96" s="15"/>
+      <c r="D96" s="16"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="14"/>
       <c r="B97" s="15"/>
-      <c r="C97" s="16"/>
+      <c r="C97" s="15"/>
+      <c r="D97" s="16"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="14"/>
       <c r="B98" s="15"/>
-      <c r="C98" s="16"/>
+      <c r="C98" s="15"/>
+      <c r="D98" s="16"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="14"/>
       <c r="B99" s="15"/>
-      <c r="C99" s="16"/>
+      <c r="C99" s="15"/>
+      <c r="D99" s="16"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="14"/>
       <c r="B100" s="15"/>
-      <c r="C100" s="16"/>
+      <c r="C100" s="15"/>
+      <c r="D100" s="16"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="14"/>
       <c r="B101" s="15"/>
-      <c r="C101" s="16"/>
+      <c r="C101" s="15"/>
+      <c r="D101" s="16"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="14"/>
       <c r="B102" s="15"/>
-      <c r="C102" s="16"/>
+      <c r="C102" s="15"/>
+      <c r="D102" s="16"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="14"/>
       <c r="B103" s="15"/>
-      <c r="C103" s="16"/>
+      <c r="C103" s="15"/>
+      <c r="D103" s="16"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="14"/>
       <c r="B104" s="15"/>
-      <c r="C104" s="16"/>
+      <c r="C104" s="15"/>
+      <c r="D104" s="16"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="14"/>
       <c r="B105" s="15"/>
-      <c r="C105" s="16"/>
+      <c r="C105" s="15"/>
+      <c r="D105" s="16"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="14"/>
       <c r="B106" s="15"/>
-      <c r="C106" s="16"/>
+      <c r="C106" s="15"/>
+      <c r="D106" s="16"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="14"/>
       <c r="B107" s="15"/>
-      <c r="C107" s="16"/>
+      <c r="C107" s="15"/>
+      <c r="D107" s="16"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="14"/>
       <c r="B108" s="15"/>
-      <c r="C108" s="16"/>
+      <c r="C108" s="15"/>
+      <c r="D108" s="16"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="14"/>
       <c r="B109" s="15"/>
-      <c r="C109" s="16"/>
+      <c r="C109" s="15"/>
+      <c r="D109" s="16"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="14"/>
       <c r="B110" s="15"/>
-      <c r="C110" s="16"/>
+      <c r="C110" s="15"/>
+      <c r="D110" s="16"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="14"/>
       <c r="B111" s="15"/>
-      <c r="C111" s="16"/>
+      <c r="C111" s="15"/>
+      <c r="D111" s="16"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="14"/>
       <c r="B112" s="15"/>
-      <c r="C112" s="16"/>
+      <c r="C112" s="15"/>
+      <c r="D112" s="16"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="14"/>
       <c r="B113" s="15"/>
-      <c r="C113" s="16"/>
+      <c r="C113" s="15"/>
+      <c r="D113" s="16"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="14"/>
       <c r="B114" s="15"/>
-      <c r="C114" s="16"/>
+      <c r="C114" s="15"/>
+      <c r="D114" s="16"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="14"/>
       <c r="B115" s="15"/>
-      <c r="C115" s="16"/>
+      <c r="C115" s="15"/>
+      <c r="D115" s="16"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="14"/>
       <c r="B116" s="15"/>
-      <c r="C116" s="16"/>
+      <c r="C116" s="15"/>
+      <c r="D116" s="16"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="14"/>
       <c r="B117" s="15"/>
-      <c r="C117" s="16"/>
+      <c r="C117" s="15"/>
+      <c r="D117" s="16"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="14"/>
       <c r="B118" s="15"/>
-      <c r="C118" s="16"/>
+      <c r="C118" s="15"/>
+      <c r="D118" s="16"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="14"/>
       <c r="B119" s="15"/>
-      <c r="C119" s="16"/>
+      <c r="C119" s="15"/>
+      <c r="D119" s="16"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="14"/>
       <c r="B120" s="15"/>
-      <c r="C120" s="16"/>
+      <c r="C120" s="15"/>
+      <c r="D120" s="16"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="14"/>
       <c r="B121" s="15"/>
-      <c r="C121" s="16"/>
+      <c r="C121" s="15"/>
+      <c r="D121" s="16"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="14"/>
       <c r="B122" s="15"/>
-      <c r="C122" s="16"/>
+      <c r="C122" s="15"/>
+      <c r="D122" s="16"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="14"/>
       <c r="B123" s="15"/>
-      <c r="C123" s="16"/>
+      <c r="C123" s="15"/>
+      <c r="D123" s="16"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="14"/>
       <c r="B124" s="15"/>
-      <c r="C124" s="16"/>
+      <c r="C124" s="15"/>
+      <c r="D124" s="16"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="14"/>
       <c r="B125" s="15"/>
-      <c r="C125" s="16"/>
+      <c r="C125" s="15"/>
+      <c r="D125" s="16"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="14"/>
       <c r="B126" s="15"/>
-      <c r="C126" s="16"/>
+      <c r="C126" s="15"/>
+      <c r="D126" s="16"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="14"/>
       <c r="B127" s="15"/>
-      <c r="C127" s="16"/>
+      <c r="C127" s="15"/>
+      <c r="D127" s="16"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="14"/>
       <c r="B128" s="15"/>
-      <c r="C128" s="16"/>
+      <c r="C128" s="15"/>
+      <c r="D128" s="16"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="14"/>
       <c r="B129" s="15"/>
-      <c r="C129" s="16"/>
+      <c r="C129" s="15"/>
+      <c r="D129" s="16"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="14"/>
       <c r="B130" s="15"/>
-      <c r="C130" s="16"/>
+      <c r="C130" s="15"/>
+      <c r="D130" s="16"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="14"/>
       <c r="B131" s="15"/>
-      <c r="C131" s="16"/>
+      <c r="C131" s="15"/>
+      <c r="D131" s="16"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="14"/>
       <c r="B132" s="15"/>
-      <c r="C132" s="16"/>
+      <c r="C132" s="15"/>
+      <c r="D132" s="16"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="14"/>
       <c r="B133" s="15"/>
-      <c r="C133" s="16"/>
+      <c r="C133" s="15"/>
+      <c r="D133" s="16"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="14"/>
       <c r="B134" s="15"/>
-      <c r="C134" s="16"/>
+      <c r="C134" s="15"/>
+      <c r="D134" s="16"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="14"/>
       <c r="B135" s="15"/>
-      <c r="C135" s="16"/>
+      <c r="C135" s="15"/>
+      <c r="D135" s="16"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="14"/>
       <c r="B136" s="15"/>
-      <c r="C136" s="16"/>
+      <c r="C136" s="15"/>
+      <c r="D136" s="16"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="14"/>
       <c r="B137" s="15"/>
-      <c r="C137" s="16"/>
+      <c r="C137" s="15"/>
+      <c r="D137" s="16"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="14"/>
       <c r="B138" s="15"/>
-      <c r="C138" s="16"/>
+      <c r="C138" s="15"/>
+      <c r="D138" s="16"/>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="14"/>
       <c r="B139" s="15"/>
-      <c r="C139" s="16"/>
+      <c r="C139" s="15"/>
+      <c r="D139" s="16"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="14"/>
       <c r="B140" s="15"/>
-      <c r="C140" s="16"/>
+      <c r="C140" s="15"/>
+      <c r="D140" s="16"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="14"/>
       <c r="B141" s="15"/>
-      <c r="C141" s="16"/>
+      <c r="C141" s="15"/>
+      <c r="D141" s="16"/>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="14"/>
       <c r="B142" s="15"/>
-      <c r="C142" s="16"/>
+      <c r="C142" s="15"/>
+      <c r="D142" s="16"/>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="14"/>
       <c r="B143" s="15"/>
-      <c r="C143" s="16"/>
+      <c r="C143" s="15"/>
+      <c r="D143" s="16"/>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="14"/>
       <c r="B144" s="15"/>
-      <c r="C144" s="16"/>
+      <c r="C144" s="15"/>
+      <c r="D144" s="16"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="14"/>
       <c r="B145" s="15"/>
-      <c r="C145" s="16"/>
+      <c r="C145" s="15"/>
+      <c r="D145" s="16"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="14"/>
       <c r="B146" s="15"/>
-      <c r="C146" s="16"/>
+      <c r="C146" s="15"/>
+      <c r="D146" s="16"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="14"/>
       <c r="B147" s="15"/>
-      <c r="C147" s="16"/>
+      <c r="C147" s="15"/>
+      <c r="D147" s="16"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="14"/>
       <c r="B148" s="15"/>
-      <c r="C148" s="16"/>
+      <c r="C148" s="15"/>
+      <c r="D148" s="16"/>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="14"/>
       <c r="B149" s="15"/>
-      <c r="C149" s="16"/>
+      <c r="C149" s="15"/>
+      <c r="D149" s="16"/>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="14"/>
       <c r="B150" s="15"/>
-      <c r="C150" s="16"/>
+      <c r="C150" s="15"/>
+      <c r="D150" s="16"/>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="14"/>
       <c r="B151" s="15"/>
-      <c r="C151" s="16"/>
+      <c r="C151" s="15"/>
+      <c r="D151" s="16"/>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="14"/>
       <c r="B152" s="15"/>
-      <c r="C152" s="16"/>
+      <c r="C152" s="15"/>
+      <c r="D152" s="16"/>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="14"/>
       <c r="B153" s="15"/>
-      <c r="C153" s="16"/>
+      <c r="C153" s="15"/>
+      <c r="D153" s="16"/>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="14"/>
       <c r="B154" s="15"/>
-      <c r="C154" s="16"/>
+      <c r="C154" s="15"/>
+      <c r="D154" s="16"/>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="14"/>
       <c r="B155" s="15"/>
-      <c r="C155" s="16"/>
+      <c r="C155" s="15"/>
+      <c r="D155" s="16"/>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="14"/>
       <c r="B156" s="15"/>
-      <c r="C156" s="16"/>
+      <c r="C156" s="15"/>
+      <c r="D156" s="16"/>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="14"/>
       <c r="B157" s="15"/>
-      <c r="C157" s="16"/>
+      <c r="C157" s="15"/>
+      <c r="D157" s="16"/>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="14"/>
       <c r="B158" s="15"/>
-      <c r="C158" s="16"/>
+      <c r="C158" s="15"/>
+      <c r="D158" s="16"/>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="14"/>
       <c r="B159" s="15"/>
-      <c r="C159" s="16"/>
+      <c r="C159" s="15"/>
+      <c r="D159" s="16"/>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="14"/>
       <c r="B160" s="15"/>
-      <c r="C160" s="16"/>
+      <c r="C160" s="15"/>
+      <c r="D160" s="16"/>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="14"/>
       <c r="B161" s="15"/>
-      <c r="C161" s="16"/>
+      <c r="C161" s="15"/>
+      <c r="D161" s="16"/>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="14"/>
       <c r="B162" s="15"/>
-      <c r="C162" s="16"/>
+      <c r="C162" s="15"/>
+      <c r="D162" s="16"/>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="14"/>
       <c r="B163" s="15"/>
-      <c r="C163" s="16"/>
+      <c r="C163" s="15"/>
+      <c r="D163" s="16"/>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="14"/>
       <c r="B164" s="15"/>
-      <c r="C164" s="16"/>
+      <c r="C164" s="15"/>
+      <c r="D164" s="16"/>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="14"/>
       <c r="B165" s="15"/>
-      <c r="C165" s="16"/>
+      <c r="C165" s="15"/>
+      <c r="D165" s="16"/>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="14"/>
       <c r="B166" s="15"/>
-      <c r="C166" s="16"/>
+      <c r="C166" s="15"/>
+      <c r="D166" s="16"/>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="14"/>
       <c r="B167" s="15"/>
-      <c r="C167" s="16"/>
+      <c r="C167" s="15"/>
+      <c r="D167" s="16"/>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="14"/>
       <c r="B168" s="15"/>
-      <c r="C168" s="16"/>
+      <c r="C168" s="15"/>
+      <c r="D168" s="16"/>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="14"/>
       <c r="B169" s="15"/>
-      <c r="C169" s="16"/>
+      <c r="C169" s="15"/>
+      <c r="D169" s="16"/>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="14"/>
       <c r="B170" s="15"/>
-      <c r="C170" s="16"/>
+      <c r="C170" s="15"/>
+      <c r="D170" s="16"/>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="14"/>
       <c r="B171" s="15"/>
-      <c r="C171" s="16"/>
+      <c r="C171" s="15"/>
+      <c r="D171" s="16"/>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="14"/>
       <c r="B172" s="15"/>
-      <c r="C172" s="16"/>
+      <c r="C172" s="15"/>
+      <c r="D172" s="16"/>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="14"/>
       <c r="B173" s="15"/>
-      <c r="C173" s="16"/>
+      <c r="C173" s="15"/>
+      <c r="D173" s="16"/>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="14"/>
       <c r="B174" s="15"/>
-      <c r="C174" s="16"/>
+      <c r="C174" s="15"/>
+      <c r="D174" s="16"/>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="14"/>
       <c r="B175" s="15"/>
-      <c r="C175" s="16"/>
+      <c r="C175" s="15"/>
+      <c r="D175" s="16"/>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="14"/>
       <c r="B176" s="15"/>
-      <c r="C176" s="16"/>
+      <c r="C176" s="15"/>
+      <c r="D176" s="16"/>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="14"/>
       <c r="B177" s="15"/>
-      <c r="C177" s="16"/>
+      <c r="C177" s="15"/>
+      <c r="D177" s="16"/>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="14"/>
       <c r="B178" s="15"/>
-      <c r="C178" s="16"/>
+      <c r="C178" s="15"/>
+      <c r="D178" s="16"/>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="14"/>
       <c r="B179" s="15"/>
-      <c r="C179" s="16"/>
+      <c r="C179" s="15"/>
+      <c r="D179" s="16"/>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="14"/>
       <c r="B180" s="15"/>
-      <c r="C180" s="16"/>
+      <c r="C180" s="15"/>
+      <c r="D180" s="16"/>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="14"/>
       <c r="B181" s="15"/>
-      <c r="C181" s="16"/>
+      <c r="C181" s="15"/>
+      <c r="D181" s="16"/>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="14"/>
       <c r="B182" s="15"/>
-      <c r="C182" s="16"/>
+      <c r="C182" s="15"/>
+      <c r="D182" s="16"/>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="14"/>
       <c r="B183" s="15"/>
-      <c r="C183" s="16"/>
+      <c r="C183" s="15"/>
+      <c r="D183" s="16"/>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="14"/>
       <c r="B184" s="15"/>
-      <c r="C184" s="16"/>
+      <c r="C184" s="15"/>
+      <c r="D184" s="16"/>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="14"/>
       <c r="B185" s="15"/>
-      <c r="C185" s="16"/>
+      <c r="C185" s="15"/>
+      <c r="D185" s="16"/>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="14"/>
       <c r="B186" s="15"/>
-      <c r="C186" s="16"/>
+      <c r="C186" s="15"/>
+      <c r="D186" s="16"/>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="14"/>
       <c r="B187" s="15"/>
-      <c r="C187" s="16"/>
+      <c r="C187" s="15"/>
+      <c r="D187" s="16"/>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="14"/>
       <c r="B188" s="15"/>
-      <c r="C188" s="16"/>
+      <c r="C188" s="15"/>
+      <c r="D188" s="16"/>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="14"/>
       <c r="B189" s="15"/>
-      <c r="C189" s="16"/>
+      <c r="C189" s="15"/>
+      <c r="D189" s="16"/>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="14"/>
       <c r="B190" s="15"/>
-      <c r="C190" s="16"/>
+      <c r="C190" s="15"/>
+      <c r="D190" s="16"/>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="14"/>
       <c r="B191" s="15"/>
-      <c r="C191" s="16"/>
+      <c r="C191" s="15"/>
+      <c r="D191" s="16"/>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="14"/>
       <c r="B192" s="15"/>
-      <c r="C192" s="16"/>
+      <c r="C192" s="15"/>
+      <c r="D192" s="16"/>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="14"/>
       <c r="B193" s="15"/>
-      <c r="C193" s="16"/>
+      <c r="C193" s="15"/>
+      <c r="D193" s="16"/>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="14"/>
       <c r="B194" s="15"/>
-      <c r="C194" s="16"/>
+      <c r="C194" s="15"/>
+      <c r="D194" s="16"/>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="14"/>
       <c r="B195" s="15"/>
-      <c r="C195" s="16"/>
+      <c r="C195" s="15"/>
+      <c r="D195" s="16"/>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="14"/>
       <c r="B196" s="15"/>
-      <c r="C196" s="16"/>
+      <c r="C196" s="15"/>
+      <c r="D196" s="16"/>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="14"/>
       <c r="B197" s="15"/>
-      <c r="C197" s="16"/>
+      <c r="C197" s="15"/>
+      <c r="D197" s="16"/>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="14"/>
       <c r="B198" s="15"/>
-      <c r="C198" s="16"/>
+      <c r="C198" s="15"/>
+      <c r="D198" s="16"/>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="14"/>
       <c r="B199" s="15"/>
-      <c r="C199" s="16"/>
+      <c r="C199" s="15"/>
+      <c r="D199" s="16"/>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="14"/>
       <c r="B200" s="15"/>
-      <c r="C200" s="16"/>
+      <c r="C200" s="15"/>
+      <c r="D200" s="16"/>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="14"/>
       <c r="B201" s="15"/>
-      <c r="C201" s="16"/>
+      <c r="C201" s="15"/>
+      <c r="D201" s="16"/>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="14"/>
       <c r="B202" s="15"/>
-      <c r="C202" s="16"/>
+      <c r="C202" s="15"/>
+      <c r="D202" s="16"/>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="14"/>
       <c r="B203" s="15"/>
-      <c r="C203" s="16"/>
+      <c r="C203" s="15"/>
+      <c r="D203" s="16"/>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="14"/>
       <c r="B204" s="15"/>
-      <c r="C204" s="16"/>
+      <c r="C204" s="15"/>
+      <c r="D204" s="16"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" error="Elegí un componente de la lista." errorStyle="stop" errorTitle="Componente inválido" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B5:B204" type="list">
+      <formula1>"Agus C.,Agus M.,Boli,Cami,Flopa,Katy,Luci,Mai,María,Marti,Paz,Vicky"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1874,45 +2107,49 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G204"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G4" s="17" t="n">
-        <f aca="false">SUM(C5:C204)</f>
+        <v>30</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="H4" s="17" t="n">
+        <f aca="false">SUM(D5:D204)</f>
         <v>3</v>
       </c>
     </row>
@@ -1921,1224 +2158,1432 @@
         <v>46315</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="18" t="n">
+        <v>33</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="E5" s="16" t="n">
         <v>30000</v>
       </c>
-      <c r="F5" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="13" t="n">
-        <f aca="false">SUM(D5:D204)</f>
+      <c r="G5" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="H5" s="13" t="n">
+        <f aca="false">SUM(E5:E204)</f>
         <v>30000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14"/>
       <c r="B6" s="15"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="16"/>
-      <c r="F6" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="G6" s="13" t="n">
-        <f aca="false">IFERROR(G5/G4,0)</f>
+      <c r="C6" s="15"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="16"/>
+      <c r="G6" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="13" t="n">
+        <f aca="false">IFERROR(H5/H4,0)</f>
         <v>10000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14"/>
       <c r="B7" s="15"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="16"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="16"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14"/>
       <c r="B8" s="15"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="16"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14"/>
       <c r="B9" s="15"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="16"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="16"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14"/>
       <c r="B10" s="15"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="16"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="16"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14"/>
       <c r="B11" s="15"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="16"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="16"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14"/>
       <c r="B12" s="15"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="16"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="16"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14"/>
       <c r="B13" s="15"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="16"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="16"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14"/>
       <c r="B14" s="15"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="16"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="16"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14"/>
       <c r="B15" s="15"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="16"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="16"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14"/>
       <c r="B16" s="15"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="16"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="16"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14"/>
       <c r="B17" s="15"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="16"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="16"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14"/>
       <c r="B18" s="15"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="16"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="16"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14"/>
       <c r="B19" s="15"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="16"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="16"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14"/>
       <c r="B20" s="15"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="16"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="16"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14"/>
       <c r="B21" s="15"/>
-      <c r="C21" s="18"/>
-      <c r="D21" s="16"/>
+      <c r="C21" s="15"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="16"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14"/>
       <c r="B22" s="15"/>
-      <c r="C22" s="18"/>
-      <c r="D22" s="16"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="16"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14"/>
       <c r="B23" s="15"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="16"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="16"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14"/>
       <c r="B24" s="15"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="16"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="16"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14"/>
       <c r="B25" s="15"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="16"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="16"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14"/>
       <c r="B26" s="15"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="16"/>
+      <c r="C26" s="15"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="16"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14"/>
       <c r="B27" s="15"/>
-      <c r="C27" s="18"/>
-      <c r="D27" s="16"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="16"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14"/>
       <c r="B28" s="15"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="16"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="16"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14"/>
       <c r="B29" s="15"/>
-      <c r="C29" s="18"/>
-      <c r="D29" s="16"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="16"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14"/>
       <c r="B30" s="15"/>
-      <c r="C30" s="18"/>
-      <c r="D30" s="16"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="16"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14"/>
       <c r="B31" s="15"/>
-      <c r="C31" s="18"/>
-      <c r="D31" s="16"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="16"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14"/>
       <c r="B32" s="15"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="16"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="16"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14"/>
       <c r="B33" s="15"/>
-      <c r="C33" s="18"/>
-      <c r="D33" s="16"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="16"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14"/>
       <c r="B34" s="15"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="16"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="16"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="14"/>
       <c r="B35" s="15"/>
-      <c r="C35" s="18"/>
-      <c r="D35" s="16"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="16"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="14"/>
       <c r="B36" s="15"/>
-      <c r="C36" s="18"/>
-      <c r="D36" s="16"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="16"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14"/>
       <c r="B37" s="15"/>
-      <c r="C37" s="18"/>
-      <c r="D37" s="16"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="16"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14"/>
       <c r="B38" s="15"/>
-      <c r="C38" s="18"/>
-      <c r="D38" s="16"/>
+      <c r="C38" s="15"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="16"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="14"/>
       <c r="B39" s="15"/>
-      <c r="C39" s="18"/>
-      <c r="D39" s="16"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="16"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="14"/>
       <c r="B40" s="15"/>
-      <c r="C40" s="18"/>
-      <c r="D40" s="16"/>
+      <c r="C40" s="15"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="16"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="14"/>
       <c r="B41" s="15"/>
-      <c r="C41" s="18"/>
-      <c r="D41" s="16"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="18"/>
+      <c r="E41" s="16"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14"/>
       <c r="B42" s="15"/>
-      <c r="C42" s="18"/>
-      <c r="D42" s="16"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="18"/>
+      <c r="E42" s="16"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="14"/>
       <c r="B43" s="15"/>
-      <c r="C43" s="18"/>
-      <c r="D43" s="16"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="16"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="14"/>
       <c r="B44" s="15"/>
-      <c r="C44" s="18"/>
-      <c r="D44" s="16"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="18"/>
+      <c r="E44" s="16"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="14"/>
       <c r="B45" s="15"/>
-      <c r="C45" s="18"/>
-      <c r="D45" s="16"/>
+      <c r="C45" s="15"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="16"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="14"/>
       <c r="B46" s="15"/>
-      <c r="C46" s="18"/>
-      <c r="D46" s="16"/>
+      <c r="C46" s="15"/>
+      <c r="D46" s="18"/>
+      <c r="E46" s="16"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="14"/>
       <c r="B47" s="15"/>
-      <c r="C47" s="18"/>
-      <c r="D47" s="16"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="18"/>
+      <c r="E47" s="16"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="14"/>
       <c r="B48" s="15"/>
-      <c r="C48" s="18"/>
-      <c r="D48" s="16"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="18"/>
+      <c r="E48" s="16"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="14"/>
       <c r="B49" s="15"/>
-      <c r="C49" s="18"/>
-      <c r="D49" s="16"/>
+      <c r="C49" s="15"/>
+      <c r="D49" s="18"/>
+      <c r="E49" s="16"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="14"/>
       <c r="B50" s="15"/>
-      <c r="C50" s="18"/>
-      <c r="D50" s="16"/>
+      <c r="C50" s="15"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="16"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="14"/>
       <c r="B51" s="15"/>
-      <c r="C51" s="18"/>
-      <c r="D51" s="16"/>
+      <c r="C51" s="15"/>
+      <c r="D51" s="18"/>
+      <c r="E51" s="16"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="14"/>
       <c r="B52" s="15"/>
-      <c r="C52" s="18"/>
-      <c r="D52" s="16"/>
+      <c r="C52" s="15"/>
+      <c r="D52" s="18"/>
+      <c r="E52" s="16"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="14"/>
       <c r="B53" s="15"/>
-      <c r="C53" s="18"/>
-      <c r="D53" s="16"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="18"/>
+      <c r="E53" s="16"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="14"/>
       <c r="B54" s="15"/>
-      <c r="C54" s="18"/>
-      <c r="D54" s="16"/>
+      <c r="C54" s="15"/>
+      <c r="D54" s="18"/>
+      <c r="E54" s="16"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="14"/>
       <c r="B55" s="15"/>
-      <c r="C55" s="18"/>
-      <c r="D55" s="16"/>
+      <c r="C55" s="15"/>
+      <c r="D55" s="18"/>
+      <c r="E55" s="16"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="14"/>
       <c r="B56" s="15"/>
-      <c r="C56" s="18"/>
-      <c r="D56" s="16"/>
+      <c r="C56" s="15"/>
+      <c r="D56" s="18"/>
+      <c r="E56" s="16"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="14"/>
       <c r="B57" s="15"/>
-      <c r="C57" s="18"/>
-      <c r="D57" s="16"/>
+      <c r="C57" s="15"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="16"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="14"/>
       <c r="B58" s="15"/>
-      <c r="C58" s="18"/>
-      <c r="D58" s="16"/>
+      <c r="C58" s="15"/>
+      <c r="D58" s="18"/>
+      <c r="E58" s="16"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="14"/>
       <c r="B59" s="15"/>
-      <c r="C59" s="18"/>
-      <c r="D59" s="16"/>
+      <c r="C59" s="15"/>
+      <c r="D59" s="18"/>
+      <c r="E59" s="16"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="14"/>
       <c r="B60" s="15"/>
-      <c r="C60" s="18"/>
-      <c r="D60" s="16"/>
+      <c r="C60" s="15"/>
+      <c r="D60" s="18"/>
+      <c r="E60" s="16"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="14"/>
       <c r="B61" s="15"/>
-      <c r="C61" s="18"/>
-      <c r="D61" s="16"/>
+      <c r="C61" s="15"/>
+      <c r="D61" s="18"/>
+      <c r="E61" s="16"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="14"/>
       <c r="B62" s="15"/>
-      <c r="C62" s="18"/>
-      <c r="D62" s="16"/>
+      <c r="C62" s="15"/>
+      <c r="D62" s="18"/>
+      <c r="E62" s="16"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="14"/>
       <c r="B63" s="15"/>
-      <c r="C63" s="18"/>
-      <c r="D63" s="16"/>
+      <c r="C63" s="15"/>
+      <c r="D63" s="18"/>
+      <c r="E63" s="16"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="14"/>
       <c r="B64" s="15"/>
-      <c r="C64" s="18"/>
-      <c r="D64" s="16"/>
+      <c r="C64" s="15"/>
+      <c r="D64" s="18"/>
+      <c r="E64" s="16"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="14"/>
       <c r="B65" s="15"/>
-      <c r="C65" s="18"/>
-      <c r="D65" s="16"/>
+      <c r="C65" s="15"/>
+      <c r="D65" s="18"/>
+      <c r="E65" s="16"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="14"/>
       <c r="B66" s="15"/>
-      <c r="C66" s="18"/>
-      <c r="D66" s="16"/>
+      <c r="C66" s="15"/>
+      <c r="D66" s="18"/>
+      <c r="E66" s="16"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="14"/>
       <c r="B67" s="15"/>
-      <c r="C67" s="18"/>
-      <c r="D67" s="16"/>
+      <c r="C67" s="15"/>
+      <c r="D67" s="18"/>
+      <c r="E67" s="16"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="14"/>
       <c r="B68" s="15"/>
-      <c r="C68" s="18"/>
-      <c r="D68" s="16"/>
+      <c r="C68" s="15"/>
+      <c r="D68" s="18"/>
+      <c r="E68" s="16"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="14"/>
       <c r="B69" s="15"/>
-      <c r="C69" s="18"/>
-      <c r="D69" s="16"/>
+      <c r="C69" s="15"/>
+      <c r="D69" s="18"/>
+      <c r="E69" s="16"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="14"/>
       <c r="B70" s="15"/>
-      <c r="C70" s="18"/>
-      <c r="D70" s="16"/>
+      <c r="C70" s="15"/>
+      <c r="D70" s="18"/>
+      <c r="E70" s="16"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="14"/>
       <c r="B71" s="15"/>
-      <c r="C71" s="18"/>
-      <c r="D71" s="16"/>
+      <c r="C71" s="15"/>
+      <c r="D71" s="18"/>
+      <c r="E71" s="16"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="14"/>
       <c r="B72" s="15"/>
-      <c r="C72" s="18"/>
-      <c r="D72" s="16"/>
+      <c r="C72" s="15"/>
+      <c r="D72" s="18"/>
+      <c r="E72" s="16"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="14"/>
       <c r="B73" s="15"/>
-      <c r="C73" s="18"/>
-      <c r="D73" s="16"/>
+      <c r="C73" s="15"/>
+      <c r="D73" s="18"/>
+      <c r="E73" s="16"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="14"/>
       <c r="B74" s="15"/>
-      <c r="C74" s="18"/>
-      <c r="D74" s="16"/>
+      <c r="C74" s="15"/>
+      <c r="D74" s="18"/>
+      <c r="E74" s="16"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="14"/>
       <c r="B75" s="15"/>
-      <c r="C75" s="18"/>
-      <c r="D75" s="16"/>
+      <c r="C75" s="15"/>
+      <c r="D75" s="18"/>
+      <c r="E75" s="16"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="14"/>
       <c r="B76" s="15"/>
-      <c r="C76" s="18"/>
-      <c r="D76" s="16"/>
+      <c r="C76" s="15"/>
+      <c r="D76" s="18"/>
+      <c r="E76" s="16"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="14"/>
       <c r="B77" s="15"/>
-      <c r="C77" s="18"/>
-      <c r="D77" s="16"/>
+      <c r="C77" s="15"/>
+      <c r="D77" s="18"/>
+      <c r="E77" s="16"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="14"/>
       <c r="B78" s="15"/>
-      <c r="C78" s="18"/>
-      <c r="D78" s="16"/>
+      <c r="C78" s="15"/>
+      <c r="D78" s="18"/>
+      <c r="E78" s="16"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="14"/>
       <c r="B79" s="15"/>
-      <c r="C79" s="18"/>
-      <c r="D79" s="16"/>
+      <c r="C79" s="15"/>
+      <c r="D79" s="18"/>
+      <c r="E79" s="16"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="14"/>
       <c r="B80" s="15"/>
-      <c r="C80" s="18"/>
-      <c r="D80" s="16"/>
+      <c r="C80" s="15"/>
+      <c r="D80" s="18"/>
+      <c r="E80" s="16"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="14"/>
       <c r="B81" s="15"/>
-      <c r="C81" s="18"/>
-      <c r="D81" s="16"/>
+      <c r="C81" s="15"/>
+      <c r="D81" s="18"/>
+      <c r="E81" s="16"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="14"/>
       <c r="B82" s="15"/>
-      <c r="C82" s="18"/>
-      <c r="D82" s="16"/>
+      <c r="C82" s="15"/>
+      <c r="D82" s="18"/>
+      <c r="E82" s="16"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="14"/>
       <c r="B83" s="15"/>
-      <c r="C83" s="18"/>
-      <c r="D83" s="16"/>
+      <c r="C83" s="15"/>
+      <c r="D83" s="18"/>
+      <c r="E83" s="16"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="14"/>
       <c r="B84" s="15"/>
-      <c r="C84" s="18"/>
-      <c r="D84" s="16"/>
+      <c r="C84" s="15"/>
+      <c r="D84" s="18"/>
+      <c r="E84" s="16"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="14"/>
       <c r="B85" s="15"/>
-      <c r="C85" s="18"/>
-      <c r="D85" s="16"/>
+      <c r="C85" s="15"/>
+      <c r="D85" s="18"/>
+      <c r="E85" s="16"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="14"/>
       <c r="B86" s="15"/>
-      <c r="C86" s="18"/>
-      <c r="D86" s="16"/>
+      <c r="C86" s="15"/>
+      <c r="D86" s="18"/>
+      <c r="E86" s="16"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="14"/>
       <c r="B87" s="15"/>
-      <c r="C87" s="18"/>
-      <c r="D87" s="16"/>
+      <c r="C87" s="15"/>
+      <c r="D87" s="18"/>
+      <c r="E87" s="16"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="14"/>
       <c r="B88" s="15"/>
-      <c r="C88" s="18"/>
-      <c r="D88" s="16"/>
+      <c r="C88" s="15"/>
+      <c r="D88" s="18"/>
+      <c r="E88" s="16"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="14"/>
       <c r="B89" s="15"/>
-      <c r="C89" s="18"/>
-      <c r="D89" s="16"/>
+      <c r="C89" s="15"/>
+      <c r="D89" s="18"/>
+      <c r="E89" s="16"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="14"/>
       <c r="B90" s="15"/>
-      <c r="C90" s="18"/>
-      <c r="D90" s="16"/>
+      <c r="C90" s="15"/>
+      <c r="D90" s="18"/>
+      <c r="E90" s="16"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="14"/>
       <c r="B91" s="15"/>
-      <c r="C91" s="18"/>
-      <c r="D91" s="16"/>
+      <c r="C91" s="15"/>
+      <c r="D91" s="18"/>
+      <c r="E91" s="16"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="14"/>
       <c r="B92" s="15"/>
-      <c r="C92" s="18"/>
-      <c r="D92" s="16"/>
+      <c r="C92" s="15"/>
+      <c r="D92" s="18"/>
+      <c r="E92" s="16"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="14"/>
       <c r="B93" s="15"/>
-      <c r="C93" s="18"/>
-      <c r="D93" s="16"/>
+      <c r="C93" s="15"/>
+      <c r="D93" s="18"/>
+      <c r="E93" s="16"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="14"/>
       <c r="B94" s="15"/>
-      <c r="C94" s="18"/>
-      <c r="D94" s="16"/>
+      <c r="C94" s="15"/>
+      <c r="D94" s="18"/>
+      <c r="E94" s="16"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="14"/>
       <c r="B95" s="15"/>
-      <c r="C95" s="18"/>
-      <c r="D95" s="16"/>
+      <c r="C95" s="15"/>
+      <c r="D95" s="18"/>
+      <c r="E95" s="16"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="14"/>
       <c r="B96" s="15"/>
-      <c r="C96" s="18"/>
-      <c r="D96" s="16"/>
+      <c r="C96" s="15"/>
+      <c r="D96" s="18"/>
+      <c r="E96" s="16"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="14"/>
       <c r="B97" s="15"/>
-      <c r="C97" s="18"/>
-      <c r="D97" s="16"/>
+      <c r="C97" s="15"/>
+      <c r="D97" s="18"/>
+      <c r="E97" s="16"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="14"/>
       <c r="B98" s="15"/>
-      <c r="C98" s="18"/>
-      <c r="D98" s="16"/>
+      <c r="C98" s="15"/>
+      <c r="D98" s="18"/>
+      <c r="E98" s="16"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="14"/>
       <c r="B99" s="15"/>
-      <c r="C99" s="18"/>
-      <c r="D99" s="16"/>
+      <c r="C99" s="15"/>
+      <c r="D99" s="18"/>
+      <c r="E99" s="16"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="14"/>
       <c r="B100" s="15"/>
-      <c r="C100" s="18"/>
-      <c r="D100" s="16"/>
+      <c r="C100" s="15"/>
+      <c r="D100" s="18"/>
+      <c r="E100" s="16"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="14"/>
       <c r="B101" s="15"/>
-      <c r="C101" s="18"/>
-      <c r="D101" s="16"/>
+      <c r="C101" s="15"/>
+      <c r="D101" s="18"/>
+      <c r="E101" s="16"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="14"/>
       <c r="B102" s="15"/>
-      <c r="C102" s="18"/>
-      <c r="D102" s="16"/>
+      <c r="C102" s="15"/>
+      <c r="D102" s="18"/>
+      <c r="E102" s="16"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="14"/>
       <c r="B103" s="15"/>
-      <c r="C103" s="18"/>
-      <c r="D103" s="16"/>
+      <c r="C103" s="15"/>
+      <c r="D103" s="18"/>
+      <c r="E103" s="16"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="14"/>
       <c r="B104" s="15"/>
-      <c r="C104" s="18"/>
-      <c r="D104" s="16"/>
+      <c r="C104" s="15"/>
+      <c r="D104" s="18"/>
+      <c r="E104" s="16"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="14"/>
       <c r="B105" s="15"/>
-      <c r="C105" s="18"/>
-      <c r="D105" s="16"/>
+      <c r="C105" s="15"/>
+      <c r="D105" s="18"/>
+      <c r="E105" s="16"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="14"/>
       <c r="B106" s="15"/>
-      <c r="C106" s="18"/>
-      <c r="D106" s="16"/>
+      <c r="C106" s="15"/>
+      <c r="D106" s="18"/>
+      <c r="E106" s="16"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="14"/>
       <c r="B107" s="15"/>
-      <c r="C107" s="18"/>
-      <c r="D107" s="16"/>
+      <c r="C107" s="15"/>
+      <c r="D107" s="18"/>
+      <c r="E107" s="16"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="14"/>
       <c r="B108" s="15"/>
-      <c r="C108" s="18"/>
-      <c r="D108" s="16"/>
+      <c r="C108" s="15"/>
+      <c r="D108" s="18"/>
+      <c r="E108" s="16"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="14"/>
       <c r="B109" s="15"/>
-      <c r="C109" s="18"/>
-      <c r="D109" s="16"/>
+      <c r="C109" s="15"/>
+      <c r="D109" s="18"/>
+      <c r="E109" s="16"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="14"/>
       <c r="B110" s="15"/>
-      <c r="C110" s="18"/>
-      <c r="D110" s="16"/>
+      <c r="C110" s="15"/>
+      <c r="D110" s="18"/>
+      <c r="E110" s="16"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="14"/>
       <c r="B111" s="15"/>
-      <c r="C111" s="18"/>
-      <c r="D111" s="16"/>
+      <c r="C111" s="15"/>
+      <c r="D111" s="18"/>
+      <c r="E111" s="16"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="14"/>
       <c r="B112" s="15"/>
-      <c r="C112" s="18"/>
-      <c r="D112" s="16"/>
+      <c r="C112" s="15"/>
+      <c r="D112" s="18"/>
+      <c r="E112" s="16"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="14"/>
       <c r="B113" s="15"/>
-      <c r="C113" s="18"/>
-      <c r="D113" s="16"/>
+      <c r="C113" s="15"/>
+      <c r="D113" s="18"/>
+      <c r="E113" s="16"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="14"/>
       <c r="B114" s="15"/>
-      <c r="C114" s="18"/>
-      <c r="D114" s="16"/>
+      <c r="C114" s="15"/>
+      <c r="D114" s="18"/>
+      <c r="E114" s="16"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="14"/>
       <c r="B115" s="15"/>
-      <c r="C115" s="18"/>
-      <c r="D115" s="16"/>
+      <c r="C115" s="15"/>
+      <c r="D115" s="18"/>
+      <c r="E115" s="16"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="14"/>
       <c r="B116" s="15"/>
-      <c r="C116" s="18"/>
-      <c r="D116" s="16"/>
+      <c r="C116" s="15"/>
+      <c r="D116" s="18"/>
+      <c r="E116" s="16"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="14"/>
       <c r="B117" s="15"/>
-      <c r="C117" s="18"/>
-      <c r="D117" s="16"/>
+      <c r="C117" s="15"/>
+      <c r="D117" s="18"/>
+      <c r="E117" s="16"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="14"/>
       <c r="B118" s="15"/>
-      <c r="C118" s="18"/>
-      <c r="D118" s="16"/>
+      <c r="C118" s="15"/>
+      <c r="D118" s="18"/>
+      <c r="E118" s="16"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="14"/>
       <c r="B119" s="15"/>
-      <c r="C119" s="18"/>
-      <c r="D119" s="16"/>
+      <c r="C119" s="15"/>
+      <c r="D119" s="18"/>
+      <c r="E119" s="16"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="14"/>
       <c r="B120" s="15"/>
-      <c r="C120" s="18"/>
-      <c r="D120" s="16"/>
+      <c r="C120" s="15"/>
+      <c r="D120" s="18"/>
+      <c r="E120" s="16"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="14"/>
       <c r="B121" s="15"/>
-      <c r="C121" s="18"/>
-      <c r="D121" s="16"/>
+      <c r="C121" s="15"/>
+      <c r="D121" s="18"/>
+      <c r="E121" s="16"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="14"/>
       <c r="B122" s="15"/>
-      <c r="C122" s="18"/>
-      <c r="D122" s="16"/>
+      <c r="C122" s="15"/>
+      <c r="D122" s="18"/>
+      <c r="E122" s="16"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="14"/>
       <c r="B123" s="15"/>
-      <c r="C123" s="18"/>
-      <c r="D123" s="16"/>
+      <c r="C123" s="15"/>
+      <c r="D123" s="18"/>
+      <c r="E123" s="16"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="14"/>
       <c r="B124" s="15"/>
-      <c r="C124" s="18"/>
-      <c r="D124" s="16"/>
+      <c r="C124" s="15"/>
+      <c r="D124" s="18"/>
+      <c r="E124" s="16"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="14"/>
       <c r="B125" s="15"/>
-      <c r="C125" s="18"/>
-      <c r="D125" s="16"/>
+      <c r="C125" s="15"/>
+      <c r="D125" s="18"/>
+      <c r="E125" s="16"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="14"/>
       <c r="B126" s="15"/>
-      <c r="C126" s="18"/>
-      <c r="D126" s="16"/>
+      <c r="C126" s="15"/>
+      <c r="D126" s="18"/>
+      <c r="E126" s="16"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="14"/>
       <c r="B127" s="15"/>
-      <c r="C127" s="18"/>
-      <c r="D127" s="16"/>
+      <c r="C127" s="15"/>
+      <c r="D127" s="18"/>
+      <c r="E127" s="16"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="14"/>
       <c r="B128" s="15"/>
-      <c r="C128" s="18"/>
-      <c r="D128" s="16"/>
+      <c r="C128" s="15"/>
+      <c r="D128" s="18"/>
+      <c r="E128" s="16"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="14"/>
       <c r="B129" s="15"/>
-      <c r="C129" s="18"/>
-      <c r="D129" s="16"/>
+      <c r="C129" s="15"/>
+      <c r="D129" s="18"/>
+      <c r="E129" s="16"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="14"/>
       <c r="B130" s="15"/>
-      <c r="C130" s="18"/>
-      <c r="D130" s="16"/>
+      <c r="C130" s="15"/>
+      <c r="D130" s="18"/>
+      <c r="E130" s="16"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="14"/>
       <c r="B131" s="15"/>
-      <c r="C131" s="18"/>
-      <c r="D131" s="16"/>
+      <c r="C131" s="15"/>
+      <c r="D131" s="18"/>
+      <c r="E131" s="16"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="14"/>
       <c r="B132" s="15"/>
-      <c r="C132" s="18"/>
-      <c r="D132" s="16"/>
+      <c r="C132" s="15"/>
+      <c r="D132" s="18"/>
+      <c r="E132" s="16"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="14"/>
       <c r="B133" s="15"/>
-      <c r="C133" s="18"/>
-      <c r="D133" s="16"/>
+      <c r="C133" s="15"/>
+      <c r="D133" s="18"/>
+      <c r="E133" s="16"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="14"/>
       <c r="B134" s="15"/>
-      <c r="C134" s="18"/>
-      <c r="D134" s="16"/>
+      <c r="C134" s="15"/>
+      <c r="D134" s="18"/>
+      <c r="E134" s="16"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="14"/>
       <c r="B135" s="15"/>
-      <c r="C135" s="18"/>
-      <c r="D135" s="16"/>
+      <c r="C135" s="15"/>
+      <c r="D135" s="18"/>
+      <c r="E135" s="16"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="14"/>
       <c r="B136" s="15"/>
-      <c r="C136" s="18"/>
-      <c r="D136" s="16"/>
+      <c r="C136" s="15"/>
+      <c r="D136" s="18"/>
+      <c r="E136" s="16"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="14"/>
       <c r="B137" s="15"/>
-      <c r="C137" s="18"/>
-      <c r="D137" s="16"/>
+      <c r="C137" s="15"/>
+      <c r="D137" s="18"/>
+      <c r="E137" s="16"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="14"/>
       <c r="B138" s="15"/>
-      <c r="C138" s="18"/>
-      <c r="D138" s="16"/>
+      <c r="C138" s="15"/>
+      <c r="D138" s="18"/>
+      <c r="E138" s="16"/>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="14"/>
       <c r="B139" s="15"/>
-      <c r="C139" s="18"/>
-      <c r="D139" s="16"/>
+      <c r="C139" s="15"/>
+      <c r="D139" s="18"/>
+      <c r="E139" s="16"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="14"/>
       <c r="B140" s="15"/>
-      <c r="C140" s="18"/>
-      <c r="D140" s="16"/>
+      <c r="C140" s="15"/>
+      <c r="D140" s="18"/>
+      <c r="E140" s="16"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="14"/>
       <c r="B141" s="15"/>
-      <c r="C141" s="18"/>
-      <c r="D141" s="16"/>
+      <c r="C141" s="15"/>
+      <c r="D141" s="18"/>
+      <c r="E141" s="16"/>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="14"/>
       <c r="B142" s="15"/>
-      <c r="C142" s="18"/>
-      <c r="D142" s="16"/>
+      <c r="C142" s="15"/>
+      <c r="D142" s="18"/>
+      <c r="E142" s="16"/>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="14"/>
       <c r="B143" s="15"/>
-      <c r="C143" s="18"/>
-      <c r="D143" s="16"/>
+      <c r="C143" s="15"/>
+      <c r="D143" s="18"/>
+      <c r="E143" s="16"/>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="14"/>
       <c r="B144" s="15"/>
-      <c r="C144" s="18"/>
-      <c r="D144" s="16"/>
+      <c r="C144" s="15"/>
+      <c r="D144" s="18"/>
+      <c r="E144" s="16"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="14"/>
       <c r="B145" s="15"/>
-      <c r="C145" s="18"/>
-      <c r="D145" s="16"/>
+      <c r="C145" s="15"/>
+      <c r="D145" s="18"/>
+      <c r="E145" s="16"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="14"/>
       <c r="B146" s="15"/>
-      <c r="C146" s="18"/>
-      <c r="D146" s="16"/>
+      <c r="C146" s="15"/>
+      <c r="D146" s="18"/>
+      <c r="E146" s="16"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="14"/>
       <c r="B147" s="15"/>
-      <c r="C147" s="18"/>
-      <c r="D147" s="16"/>
+      <c r="C147" s="15"/>
+      <c r="D147" s="18"/>
+      <c r="E147" s="16"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="14"/>
       <c r="B148" s="15"/>
-      <c r="C148" s="18"/>
-      <c r="D148" s="16"/>
+      <c r="C148" s="15"/>
+      <c r="D148" s="18"/>
+      <c r="E148" s="16"/>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="14"/>
       <c r="B149" s="15"/>
-      <c r="C149" s="18"/>
-      <c r="D149" s="16"/>
+      <c r="C149" s="15"/>
+      <c r="D149" s="18"/>
+      <c r="E149" s="16"/>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="14"/>
       <c r="B150" s="15"/>
-      <c r="C150" s="18"/>
-      <c r="D150" s="16"/>
+      <c r="C150" s="15"/>
+      <c r="D150" s="18"/>
+      <c r="E150" s="16"/>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="14"/>
       <c r="B151" s="15"/>
-      <c r="C151" s="18"/>
-      <c r="D151" s="16"/>
+      <c r="C151" s="15"/>
+      <c r="D151" s="18"/>
+      <c r="E151" s="16"/>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="14"/>
       <c r="B152" s="15"/>
-      <c r="C152" s="18"/>
-      <c r="D152" s="16"/>
+      <c r="C152" s="15"/>
+      <c r="D152" s="18"/>
+      <c r="E152" s="16"/>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="14"/>
       <c r="B153" s="15"/>
-      <c r="C153" s="18"/>
-      <c r="D153" s="16"/>
+      <c r="C153" s="15"/>
+      <c r="D153" s="18"/>
+      <c r="E153" s="16"/>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="14"/>
       <c r="B154" s="15"/>
-      <c r="C154" s="18"/>
-      <c r="D154" s="16"/>
+      <c r="C154" s="15"/>
+      <c r="D154" s="18"/>
+      <c r="E154" s="16"/>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="14"/>
       <c r="B155" s="15"/>
-      <c r="C155" s="18"/>
-      <c r="D155" s="16"/>
+      <c r="C155" s="15"/>
+      <c r="D155" s="18"/>
+      <c r="E155" s="16"/>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="14"/>
       <c r="B156" s="15"/>
-      <c r="C156" s="18"/>
-      <c r="D156" s="16"/>
+      <c r="C156" s="15"/>
+      <c r="D156" s="18"/>
+      <c r="E156" s="16"/>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="14"/>
       <c r="B157" s="15"/>
-      <c r="C157" s="18"/>
-      <c r="D157" s="16"/>
+      <c r="C157" s="15"/>
+      <c r="D157" s="18"/>
+      <c r="E157" s="16"/>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="14"/>
       <c r="B158" s="15"/>
-      <c r="C158" s="18"/>
-      <c r="D158" s="16"/>
+      <c r="C158" s="15"/>
+      <c r="D158" s="18"/>
+      <c r="E158" s="16"/>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="14"/>
       <c r="B159" s="15"/>
-      <c r="C159" s="18"/>
-      <c r="D159" s="16"/>
+      <c r="C159" s="15"/>
+      <c r="D159" s="18"/>
+      <c r="E159" s="16"/>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="14"/>
       <c r="B160" s="15"/>
-      <c r="C160" s="18"/>
-      <c r="D160" s="16"/>
+      <c r="C160" s="15"/>
+      <c r="D160" s="18"/>
+      <c r="E160" s="16"/>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="14"/>
       <c r="B161" s="15"/>
-      <c r="C161" s="18"/>
-      <c r="D161" s="16"/>
+      <c r="C161" s="15"/>
+      <c r="D161" s="18"/>
+      <c r="E161" s="16"/>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="14"/>
       <c r="B162" s="15"/>
-      <c r="C162" s="18"/>
-      <c r="D162" s="16"/>
+      <c r="C162" s="15"/>
+      <c r="D162" s="18"/>
+      <c r="E162" s="16"/>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="14"/>
       <c r="B163" s="15"/>
-      <c r="C163" s="18"/>
-      <c r="D163" s="16"/>
+      <c r="C163" s="15"/>
+      <c r="D163" s="18"/>
+      <c r="E163" s="16"/>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="14"/>
       <c r="B164" s="15"/>
-      <c r="C164" s="18"/>
-      <c r="D164" s="16"/>
+      <c r="C164" s="15"/>
+      <c r="D164" s="18"/>
+      <c r="E164" s="16"/>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="14"/>
       <c r="B165" s="15"/>
-      <c r="C165" s="18"/>
-      <c r="D165" s="16"/>
+      <c r="C165" s="15"/>
+      <c r="D165" s="18"/>
+      <c r="E165" s="16"/>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="14"/>
       <c r="B166" s="15"/>
-      <c r="C166" s="18"/>
-      <c r="D166" s="16"/>
+      <c r="C166" s="15"/>
+      <c r="D166" s="18"/>
+      <c r="E166" s="16"/>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="14"/>
       <c r="B167" s="15"/>
-      <c r="C167" s="18"/>
-      <c r="D167" s="16"/>
+      <c r="C167" s="15"/>
+      <c r="D167" s="18"/>
+      <c r="E167" s="16"/>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="14"/>
       <c r="B168" s="15"/>
-      <c r="C168" s="18"/>
-      <c r="D168" s="16"/>
+      <c r="C168" s="15"/>
+      <c r="D168" s="18"/>
+      <c r="E168" s="16"/>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="14"/>
       <c r="B169" s="15"/>
-      <c r="C169" s="18"/>
-      <c r="D169" s="16"/>
+      <c r="C169" s="15"/>
+      <c r="D169" s="18"/>
+      <c r="E169" s="16"/>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="14"/>
       <c r="B170" s="15"/>
-      <c r="C170" s="18"/>
-      <c r="D170" s="16"/>
+      <c r="C170" s="15"/>
+      <c r="D170" s="18"/>
+      <c r="E170" s="16"/>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="14"/>
       <c r="B171" s="15"/>
-      <c r="C171" s="18"/>
-      <c r="D171" s="16"/>
+      <c r="C171" s="15"/>
+      <c r="D171" s="18"/>
+      <c r="E171" s="16"/>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="14"/>
       <c r="B172" s="15"/>
-      <c r="C172" s="18"/>
-      <c r="D172" s="16"/>
+      <c r="C172" s="15"/>
+      <c r="D172" s="18"/>
+      <c r="E172" s="16"/>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="14"/>
       <c r="B173" s="15"/>
-      <c r="C173" s="18"/>
-      <c r="D173" s="16"/>
+      <c r="C173" s="15"/>
+      <c r="D173" s="18"/>
+      <c r="E173" s="16"/>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="14"/>
       <c r="B174" s="15"/>
-      <c r="C174" s="18"/>
-      <c r="D174" s="16"/>
+      <c r="C174" s="15"/>
+      <c r="D174" s="18"/>
+      <c r="E174" s="16"/>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="14"/>
       <c r="B175" s="15"/>
-      <c r="C175" s="18"/>
-      <c r="D175" s="16"/>
+      <c r="C175" s="15"/>
+      <c r="D175" s="18"/>
+      <c r="E175" s="16"/>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="14"/>
       <c r="B176" s="15"/>
-      <c r="C176" s="18"/>
-      <c r="D176" s="16"/>
+      <c r="C176" s="15"/>
+      <c r="D176" s="18"/>
+      <c r="E176" s="16"/>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="14"/>
       <c r="B177" s="15"/>
-      <c r="C177" s="18"/>
-      <c r="D177" s="16"/>
+      <c r="C177" s="15"/>
+      <c r="D177" s="18"/>
+      <c r="E177" s="16"/>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="14"/>
       <c r="B178" s="15"/>
-      <c r="C178" s="18"/>
-      <c r="D178" s="16"/>
+      <c r="C178" s="15"/>
+      <c r="D178" s="18"/>
+      <c r="E178" s="16"/>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="14"/>
       <c r="B179" s="15"/>
-      <c r="C179" s="18"/>
-      <c r="D179" s="16"/>
+      <c r="C179" s="15"/>
+      <c r="D179" s="18"/>
+      <c r="E179" s="16"/>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="14"/>
       <c r="B180" s="15"/>
-      <c r="C180" s="18"/>
-      <c r="D180" s="16"/>
+      <c r="C180" s="15"/>
+      <c r="D180" s="18"/>
+      <c r="E180" s="16"/>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="14"/>
       <c r="B181" s="15"/>
-      <c r="C181" s="18"/>
-      <c r="D181" s="16"/>
+      <c r="C181" s="15"/>
+      <c r="D181" s="18"/>
+      <c r="E181" s="16"/>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="14"/>
       <c r="B182" s="15"/>
-      <c r="C182" s="18"/>
-      <c r="D182" s="16"/>
+      <c r="C182" s="15"/>
+      <c r="D182" s="18"/>
+      <c r="E182" s="16"/>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="14"/>
       <c r="B183" s="15"/>
-      <c r="C183" s="18"/>
-      <c r="D183" s="16"/>
+      <c r="C183" s="15"/>
+      <c r="D183" s="18"/>
+      <c r="E183" s="16"/>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="14"/>
       <c r="B184" s="15"/>
-      <c r="C184" s="18"/>
-      <c r="D184" s="16"/>
+      <c r="C184" s="15"/>
+      <c r="D184" s="18"/>
+      <c r="E184" s="16"/>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="14"/>
       <c r="B185" s="15"/>
-      <c r="C185" s="18"/>
-      <c r="D185" s="16"/>
+      <c r="C185" s="15"/>
+      <c r="D185" s="18"/>
+      <c r="E185" s="16"/>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="14"/>
       <c r="B186" s="15"/>
-      <c r="C186" s="18"/>
-      <c r="D186" s="16"/>
+      <c r="C186" s="15"/>
+      <c r="D186" s="18"/>
+      <c r="E186" s="16"/>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="14"/>
       <c r="B187" s="15"/>
-      <c r="C187" s="18"/>
-      <c r="D187" s="16"/>
+      <c r="C187" s="15"/>
+      <c r="D187" s="18"/>
+      <c r="E187" s="16"/>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="14"/>
       <c r="B188" s="15"/>
-      <c r="C188" s="18"/>
-      <c r="D188" s="16"/>
+      <c r="C188" s="15"/>
+      <c r="D188" s="18"/>
+      <c r="E188" s="16"/>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="14"/>
       <c r="B189" s="15"/>
-      <c r="C189" s="18"/>
-      <c r="D189" s="16"/>
+      <c r="C189" s="15"/>
+      <c r="D189" s="18"/>
+      <c r="E189" s="16"/>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="14"/>
       <c r="B190" s="15"/>
-      <c r="C190" s="18"/>
-      <c r="D190" s="16"/>
+      <c r="C190" s="15"/>
+      <c r="D190" s="18"/>
+      <c r="E190" s="16"/>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="14"/>
       <c r="B191" s="15"/>
-      <c r="C191" s="18"/>
-      <c r="D191" s="16"/>
+      <c r="C191" s="15"/>
+      <c r="D191" s="18"/>
+      <c r="E191" s="16"/>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="14"/>
       <c r="B192" s="15"/>
-      <c r="C192" s="18"/>
-      <c r="D192" s="16"/>
+      <c r="C192" s="15"/>
+      <c r="D192" s="18"/>
+      <c r="E192" s="16"/>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="14"/>
       <c r="B193" s="15"/>
-      <c r="C193" s="18"/>
-      <c r="D193" s="16"/>
+      <c r="C193" s="15"/>
+      <c r="D193" s="18"/>
+      <c r="E193" s="16"/>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="14"/>
       <c r="B194" s="15"/>
-      <c r="C194" s="18"/>
-      <c r="D194" s="16"/>
+      <c r="C194" s="15"/>
+      <c r="D194" s="18"/>
+      <c r="E194" s="16"/>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="14"/>
       <c r="B195" s="15"/>
-      <c r="C195" s="18"/>
-      <c r="D195" s="16"/>
+      <c r="C195" s="15"/>
+      <c r="D195" s="18"/>
+      <c r="E195" s="16"/>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="14"/>
       <c r="B196" s="15"/>
-      <c r="C196" s="18"/>
-      <c r="D196" s="16"/>
+      <c r="C196" s="15"/>
+      <c r="D196" s="18"/>
+      <c r="E196" s="16"/>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="14"/>
       <c r="B197" s="15"/>
-      <c r="C197" s="18"/>
-      <c r="D197" s="16"/>
+      <c r="C197" s="15"/>
+      <c r="D197" s="18"/>
+      <c r="E197" s="16"/>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="14"/>
       <c r="B198" s="15"/>
-      <c r="C198" s="18"/>
-      <c r="D198" s="16"/>
+      <c r="C198" s="15"/>
+      <c r="D198" s="18"/>
+      <c r="E198" s="16"/>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="14"/>
       <c r="B199" s="15"/>
-      <c r="C199" s="18"/>
-      <c r="D199" s="16"/>
+      <c r="C199" s="15"/>
+      <c r="D199" s="18"/>
+      <c r="E199" s="16"/>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="14"/>
       <c r="B200" s="15"/>
-      <c r="C200" s="18"/>
-      <c r="D200" s="16"/>
+      <c r="C200" s="15"/>
+      <c r="D200" s="18"/>
+      <c r="E200" s="16"/>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="14"/>
       <c r="B201" s="15"/>
-      <c r="C201" s="18"/>
-      <c r="D201" s="16"/>
+      <c r="C201" s="15"/>
+      <c r="D201" s="18"/>
+      <c r="E201" s="16"/>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="14"/>
       <c r="B202" s="15"/>
-      <c r="C202" s="18"/>
-      <c r="D202" s="16"/>
+      <c r="C202" s="15"/>
+      <c r="D202" s="18"/>
+      <c r="E202" s="16"/>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="14"/>
       <c r="B203" s="15"/>
-      <c r="C203" s="18"/>
-      <c r="D203" s="16"/>
+      <c r="C203" s="15"/>
+      <c r="D203" s="18"/>
+      <c r="E203" s="16"/>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="14"/>
       <c r="B204" s="15"/>
-      <c r="C204" s="18"/>
-      <c r="D204" s="16"/>
+      <c r="C204" s="15"/>
+      <c r="D204" s="18"/>
+      <c r="E204" s="16"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation allowBlank="true" error="Elegí un componente de la lista." errorStyle="stop" errorTitle="Componente inválido" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B5:B204" type="list">
+      <formula1>"Agus C.,Agus M.,Boli,Cami,Flopa,Katy,Luci,Mai,María,Marti,Paz,Vicky"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3172,27 +3617,27 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="F4" s="19" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3203,7 +3648,7 @@
         <v>8</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>12000</v>
@@ -3286,12 +3731,12 @@
       <c r="B11" s="15"/>
       <c r="C11" s="15"/>
       <c r="D11" s="16"/>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="21" t="n">
-        <f aca="false">SUM(G5:G10)</f>
-        <v>12000</v>
+      <c r="G11" s="20" t="n">
+        <f aca="false">SUMIF($B$5:$B$204,F11,$D$5:$D$204)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3299,6 +3744,13 @@
       <c r="B12" s="15"/>
       <c r="C12" s="15"/>
       <c r="D12" s="16"/>
+      <c r="F12" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="G12" s="21" t="n">
+        <f aca="false">SUM(G5:G11)</f>
+        <v>12000</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14"/>
@@ -4455,7 +4907,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation allowBlank="true" error="Elegí una categoría de la lista." errorStyle="stop" errorTitle="Categoría inválida" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B5:B204" type="list">
-      <formula1>"Maquillaje,Luces,Escenografía,Utilería,Vestuario,Audio"</formula1>
+      <formula1>"Maquillaje,Luces,Escenografía,Utilería,Vestuario,Audio,Comida"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Remeras a precio fijo de $490, encabezados de tablas en rosa, saca 'las finanzas de'
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014cQS814DmisHJYTJthjhHq
</commit_message>
<xml_diff>
--- a/Finanzas_Proyecto.xlsx
+++ b/Finanzas_Proyecto.xlsx
@@ -109,7 +109,7 @@
     <t xml:space="preserve">VENTA DE REMERAS</t>
   </si>
   <si>
-    <t xml:space="preserve">Celdas rosas = para completar. Una fila por venta o tanda; elegí el componente del menú. La fila 5 es un ejemplo: reemplazala.</t>
+    <t xml:space="preserve">Celdas rosas = para completar. Una fila por venta; elegí el componente y poné las unidades. El recaudo se calcula solo con el precio por unidad. La fila 5 es un ejemplo: reemplazala.</t>
   </si>
   <si>
     <t xml:space="preserve">Detalle (talle, comprador, etc.)</t>
@@ -133,7 +133,7 @@
     <t xml:space="preserve">TOTAL RECAUDO</t>
   </si>
   <si>
-    <t xml:space="preserve">Precio promedio</t>
+    <t xml:space="preserve">Precio por unidad</t>
   </si>
   <si>
     <t xml:space="preserve">Celdas rosas = para completar. Elegí la categoría del menú desplegable. La fila 5 es un ejemplo: reemplazala.</t>
@@ -162,7 +162,7 @@
     <numFmt numFmtId="167" formatCode="\$#,##0;[RED]&quot;-$&quot;#,##0;\-"/>
     <numFmt numFmtId="168" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -238,6 +238,21 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF6A3FA0"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="11"/>
       <color rgb="FF6A3FA0"/>
       <name val="Arial"/>
@@ -326,7 +341,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -400,6 +415,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -705,7 +728,7 @@
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">Remeras!H5</f>
-        <v>30000</v>
+        <v>1470</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -723,7 +746,7 @@
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">B5+B6</f>
-        <v>55000</v>
+        <v>26470</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -816,7 +839,7 @@
       </c>
       <c r="B21" s="10" t="n">
         <f aca="false">B8-B18</f>
-        <v>43000</v>
+        <v>14470</v>
       </c>
     </row>
   </sheetData>
@@ -2166,15 +2189,16 @@
       <c r="D5" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="E5" s="16" t="n">
-        <v>30000</v>
+      <c r="E5" s="19" t="n">
+        <f aca="false">IF(D5="","",D5*$H$6)</f>
+        <v>1470</v>
       </c>
       <c r="G5" s="12" t="s">
         <v>35</v>
       </c>
       <c r="H5" s="13" t="n">
         <f aca="false">SUM(E5:E204)</f>
-        <v>30000</v>
+        <v>1470</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2182,13 +2206,15 @@
       <c r="B6" s="15"/>
       <c r="C6" s="15"/>
       <c r="D6" s="18"/>
-      <c r="E6" s="16"/>
+      <c r="E6" s="19" t="str">
+        <f aca="false">IF(D6="","",D6*$H$6)</f>
+        <v/>
+      </c>
       <c r="G6" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="H6" s="13" t="n">
-        <f aca="false">IFERROR(H5/H4,0)</f>
-        <v>10000</v>
+      <c r="H6" s="20" t="n">
+        <v>490</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2196,1386 +2222,1980 @@
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="18"/>
-      <c r="E7" s="16"/>
+      <c r="E7" s="19" t="str">
+        <f aca="false">IF(D7="","",D7*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="18"/>
-      <c r="E8" s="16"/>
+      <c r="E8" s="19" t="str">
+        <f aca="false">IF(D8="","",D8*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14"/>
       <c r="B9" s="15"/>
       <c r="C9" s="15"/>
       <c r="D9" s="18"/>
-      <c r="E9" s="16"/>
+      <c r="E9" s="19" t="str">
+        <f aca="false">IF(D9="","",D9*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14"/>
       <c r="B10" s="15"/>
       <c r="C10" s="15"/>
       <c r="D10" s="18"/>
-      <c r="E10" s="16"/>
+      <c r="E10" s="19" t="str">
+        <f aca="false">IF(D10="","",D10*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14"/>
       <c r="B11" s="15"/>
       <c r="C11" s="15"/>
       <c r="D11" s="18"/>
-      <c r="E11" s="16"/>
+      <c r="E11" s="19" t="str">
+        <f aca="false">IF(D11="","",D11*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14"/>
       <c r="B12" s="15"/>
       <c r="C12" s="15"/>
       <c r="D12" s="18"/>
-      <c r="E12" s="16"/>
+      <c r="E12" s="19" t="str">
+        <f aca="false">IF(D12="","",D12*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14"/>
       <c r="B13" s="15"/>
       <c r="C13" s="15"/>
       <c r="D13" s="18"/>
-      <c r="E13" s="16"/>
+      <c r="E13" s="19" t="str">
+        <f aca="false">IF(D13="","",D13*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14"/>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
       <c r="D14" s="18"/>
-      <c r="E14" s="16"/>
+      <c r="E14" s="19" t="str">
+        <f aca="false">IF(D14="","",D14*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14"/>
       <c r="B15" s="15"/>
       <c r="C15" s="15"/>
       <c r="D15" s="18"/>
-      <c r="E15" s="16"/>
+      <c r="E15" s="19" t="str">
+        <f aca="false">IF(D15="","",D15*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14"/>
       <c r="B16" s="15"/>
       <c r="C16" s="15"/>
       <c r="D16" s="18"/>
-      <c r="E16" s="16"/>
+      <c r="E16" s="19" t="str">
+        <f aca="false">IF(D16="","",D16*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14"/>
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
       <c r="D17" s="18"/>
-      <c r="E17" s="16"/>
+      <c r="E17" s="19" t="str">
+        <f aca="false">IF(D17="","",D17*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14"/>
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
       <c r="D18" s="18"/>
-      <c r="E18" s="16"/>
+      <c r="E18" s="19" t="str">
+        <f aca="false">IF(D18="","",D18*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14"/>
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
       <c r="D19" s="18"/>
-      <c r="E19" s="16"/>
+      <c r="E19" s="19" t="str">
+        <f aca="false">IF(D19="","",D19*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14"/>
       <c r="B20" s="15"/>
       <c r="C20" s="15"/>
       <c r="D20" s="18"/>
-      <c r="E20" s="16"/>
+      <c r="E20" s="19" t="str">
+        <f aca="false">IF(D20="","",D20*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14"/>
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
       <c r="D21" s="18"/>
-      <c r="E21" s="16"/>
+      <c r="E21" s="19" t="str">
+        <f aca="false">IF(D21="","",D21*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14"/>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
       <c r="D22" s="18"/>
-      <c r="E22" s="16"/>
+      <c r="E22" s="19" t="str">
+        <f aca="false">IF(D22="","",D22*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14"/>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
       <c r="D23" s="18"/>
-      <c r="E23" s="16"/>
+      <c r="E23" s="19" t="str">
+        <f aca="false">IF(D23="","",D23*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14"/>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
       <c r="D24" s="18"/>
-      <c r="E24" s="16"/>
+      <c r="E24" s="19" t="str">
+        <f aca="false">IF(D24="","",D24*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14"/>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
       <c r="D25" s="18"/>
-      <c r="E25" s="16"/>
+      <c r="E25" s="19" t="str">
+        <f aca="false">IF(D25="","",D25*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14"/>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
       <c r="D26" s="18"/>
-      <c r="E26" s="16"/>
+      <c r="E26" s="19" t="str">
+        <f aca="false">IF(D26="","",D26*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14"/>
       <c r="B27" s="15"/>
       <c r="C27" s="15"/>
       <c r="D27" s="18"/>
-      <c r="E27" s="16"/>
+      <c r="E27" s="19" t="str">
+        <f aca="false">IF(D27="","",D27*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14"/>
       <c r="B28" s="15"/>
       <c r="C28" s="15"/>
       <c r="D28" s="18"/>
-      <c r="E28" s="16"/>
+      <c r="E28" s="19" t="str">
+        <f aca="false">IF(D28="","",D28*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14"/>
       <c r="B29" s="15"/>
       <c r="C29" s="15"/>
       <c r="D29" s="18"/>
-      <c r="E29" s="16"/>
+      <c r="E29" s="19" t="str">
+        <f aca="false">IF(D29="","",D29*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14"/>
       <c r="B30" s="15"/>
       <c r="C30" s="15"/>
       <c r="D30" s="18"/>
-      <c r="E30" s="16"/>
+      <c r="E30" s="19" t="str">
+        <f aca="false">IF(D30="","",D30*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14"/>
       <c r="B31" s="15"/>
       <c r="C31" s="15"/>
       <c r="D31" s="18"/>
-      <c r="E31" s="16"/>
+      <c r="E31" s="19" t="str">
+        <f aca="false">IF(D31="","",D31*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14"/>
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
       <c r="D32" s="18"/>
-      <c r="E32" s="16"/>
+      <c r="E32" s="19" t="str">
+        <f aca="false">IF(D32="","",D32*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14"/>
       <c r="B33" s="15"/>
       <c r="C33" s="15"/>
       <c r="D33" s="18"/>
-      <c r="E33" s="16"/>
+      <c r="E33" s="19" t="str">
+        <f aca="false">IF(D33="","",D33*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14"/>
       <c r="B34" s="15"/>
       <c r="C34" s="15"/>
       <c r="D34" s="18"/>
-      <c r="E34" s="16"/>
+      <c r="E34" s="19" t="str">
+        <f aca="false">IF(D34="","",D34*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="14"/>
       <c r="B35" s="15"/>
       <c r="C35" s="15"/>
       <c r="D35" s="18"/>
-      <c r="E35" s="16"/>
+      <c r="E35" s="19" t="str">
+        <f aca="false">IF(D35="","",D35*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="14"/>
       <c r="B36" s="15"/>
       <c r="C36" s="15"/>
       <c r="D36" s="18"/>
-      <c r="E36" s="16"/>
+      <c r="E36" s="19" t="str">
+        <f aca="false">IF(D36="","",D36*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14"/>
       <c r="B37" s="15"/>
       <c r="C37" s="15"/>
       <c r="D37" s="18"/>
-      <c r="E37" s="16"/>
+      <c r="E37" s="19" t="str">
+        <f aca="false">IF(D37="","",D37*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14"/>
       <c r="B38" s="15"/>
       <c r="C38" s="15"/>
       <c r="D38" s="18"/>
-      <c r="E38" s="16"/>
+      <c r="E38" s="19" t="str">
+        <f aca="false">IF(D38="","",D38*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="14"/>
       <c r="B39" s="15"/>
       <c r="C39" s="15"/>
       <c r="D39" s="18"/>
-      <c r="E39" s="16"/>
+      <c r="E39" s="19" t="str">
+        <f aca="false">IF(D39="","",D39*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="14"/>
       <c r="B40" s="15"/>
       <c r="C40" s="15"/>
       <c r="D40" s="18"/>
-      <c r="E40" s="16"/>
+      <c r="E40" s="19" t="str">
+        <f aca="false">IF(D40="","",D40*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="14"/>
       <c r="B41" s="15"/>
       <c r="C41" s="15"/>
       <c r="D41" s="18"/>
-      <c r="E41" s="16"/>
+      <c r="E41" s="19" t="str">
+        <f aca="false">IF(D41="","",D41*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14"/>
       <c r="B42" s="15"/>
       <c r="C42" s="15"/>
       <c r="D42" s="18"/>
-      <c r="E42" s="16"/>
+      <c r="E42" s="19" t="str">
+        <f aca="false">IF(D42="","",D42*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="14"/>
       <c r="B43" s="15"/>
       <c r="C43" s="15"/>
       <c r="D43" s="18"/>
-      <c r="E43" s="16"/>
+      <c r="E43" s="19" t="str">
+        <f aca="false">IF(D43="","",D43*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="14"/>
       <c r="B44" s="15"/>
       <c r="C44" s="15"/>
       <c r="D44" s="18"/>
-      <c r="E44" s="16"/>
+      <c r="E44" s="19" t="str">
+        <f aca="false">IF(D44="","",D44*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="14"/>
       <c r="B45" s="15"/>
       <c r="C45" s="15"/>
       <c r="D45" s="18"/>
-      <c r="E45" s="16"/>
+      <c r="E45" s="19" t="str">
+        <f aca="false">IF(D45="","",D45*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="14"/>
       <c r="B46" s="15"/>
       <c r="C46" s="15"/>
       <c r="D46" s="18"/>
-      <c r="E46" s="16"/>
+      <c r="E46" s="19" t="str">
+        <f aca="false">IF(D46="","",D46*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="14"/>
       <c r="B47" s="15"/>
       <c r="C47" s="15"/>
       <c r="D47" s="18"/>
-      <c r="E47" s="16"/>
+      <c r="E47" s="19" t="str">
+        <f aca="false">IF(D47="","",D47*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="14"/>
       <c r="B48" s="15"/>
       <c r="C48" s="15"/>
       <c r="D48" s="18"/>
-      <c r="E48" s="16"/>
+      <c r="E48" s="19" t="str">
+        <f aca="false">IF(D48="","",D48*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="14"/>
       <c r="B49" s="15"/>
       <c r="C49" s="15"/>
       <c r="D49" s="18"/>
-      <c r="E49" s="16"/>
+      <c r="E49" s="19" t="str">
+        <f aca="false">IF(D49="","",D49*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="14"/>
       <c r="B50" s="15"/>
       <c r="C50" s="15"/>
       <c r="D50" s="18"/>
-      <c r="E50" s="16"/>
+      <c r="E50" s="19" t="str">
+        <f aca="false">IF(D50="","",D50*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="14"/>
       <c r="B51" s="15"/>
       <c r="C51" s="15"/>
       <c r="D51" s="18"/>
-      <c r="E51" s="16"/>
+      <c r="E51" s="19" t="str">
+        <f aca="false">IF(D51="","",D51*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="14"/>
       <c r="B52" s="15"/>
       <c r="C52" s="15"/>
       <c r="D52" s="18"/>
-      <c r="E52" s="16"/>
+      <c r="E52" s="19" t="str">
+        <f aca="false">IF(D52="","",D52*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="14"/>
       <c r="B53" s="15"/>
       <c r="C53" s="15"/>
       <c r="D53" s="18"/>
-      <c r="E53" s="16"/>
+      <c r="E53" s="19" t="str">
+        <f aca="false">IF(D53="","",D53*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="14"/>
       <c r="B54" s="15"/>
       <c r="C54" s="15"/>
       <c r="D54" s="18"/>
-      <c r="E54" s="16"/>
+      <c r="E54" s="19" t="str">
+        <f aca="false">IF(D54="","",D54*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="14"/>
       <c r="B55" s="15"/>
       <c r="C55" s="15"/>
       <c r="D55" s="18"/>
-      <c r="E55" s="16"/>
+      <c r="E55" s="19" t="str">
+        <f aca="false">IF(D55="","",D55*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="14"/>
       <c r="B56" s="15"/>
       <c r="C56" s="15"/>
       <c r="D56" s="18"/>
-      <c r="E56" s="16"/>
+      <c r="E56" s="19" t="str">
+        <f aca="false">IF(D56="","",D56*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="14"/>
       <c r="B57" s="15"/>
       <c r="C57" s="15"/>
       <c r="D57" s="18"/>
-      <c r="E57" s="16"/>
+      <c r="E57" s="19" t="str">
+        <f aca="false">IF(D57="","",D57*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="14"/>
       <c r="B58" s="15"/>
       <c r="C58" s="15"/>
       <c r="D58" s="18"/>
-      <c r="E58" s="16"/>
+      <c r="E58" s="19" t="str">
+        <f aca="false">IF(D58="","",D58*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="14"/>
       <c r="B59" s="15"/>
       <c r="C59" s="15"/>
       <c r="D59" s="18"/>
-      <c r="E59" s="16"/>
+      <c r="E59" s="19" t="str">
+        <f aca="false">IF(D59="","",D59*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="14"/>
       <c r="B60" s="15"/>
       <c r="C60" s="15"/>
       <c r="D60" s="18"/>
-      <c r="E60" s="16"/>
+      <c r="E60" s="19" t="str">
+        <f aca="false">IF(D60="","",D60*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="14"/>
       <c r="B61" s="15"/>
       <c r="C61" s="15"/>
       <c r="D61" s="18"/>
-      <c r="E61" s="16"/>
+      <c r="E61" s="19" t="str">
+        <f aca="false">IF(D61="","",D61*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="14"/>
       <c r="B62" s="15"/>
       <c r="C62" s="15"/>
       <c r="D62" s="18"/>
-      <c r="E62" s="16"/>
+      <c r="E62" s="19" t="str">
+        <f aca="false">IF(D62="","",D62*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="14"/>
       <c r="B63" s="15"/>
       <c r="C63" s="15"/>
       <c r="D63" s="18"/>
-      <c r="E63" s="16"/>
+      <c r="E63" s="19" t="str">
+        <f aca="false">IF(D63="","",D63*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="14"/>
       <c r="B64" s="15"/>
       <c r="C64" s="15"/>
       <c r="D64" s="18"/>
-      <c r="E64" s="16"/>
+      <c r="E64" s="19" t="str">
+        <f aca="false">IF(D64="","",D64*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="14"/>
       <c r="B65" s="15"/>
       <c r="C65" s="15"/>
       <c r="D65" s="18"/>
-      <c r="E65" s="16"/>
+      <c r="E65" s="19" t="str">
+        <f aca="false">IF(D65="","",D65*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="14"/>
       <c r="B66" s="15"/>
       <c r="C66" s="15"/>
       <c r="D66" s="18"/>
-      <c r="E66" s="16"/>
+      <c r="E66" s="19" t="str">
+        <f aca="false">IF(D66="","",D66*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="14"/>
       <c r="B67" s="15"/>
       <c r="C67" s="15"/>
       <c r="D67" s="18"/>
-      <c r="E67" s="16"/>
+      <c r="E67" s="19" t="str">
+        <f aca="false">IF(D67="","",D67*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="14"/>
       <c r="B68" s="15"/>
       <c r="C68" s="15"/>
       <c r="D68" s="18"/>
-      <c r="E68" s="16"/>
+      <c r="E68" s="19" t="str">
+        <f aca="false">IF(D68="","",D68*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="14"/>
       <c r="B69" s="15"/>
       <c r="C69" s="15"/>
       <c r="D69" s="18"/>
-      <c r="E69" s="16"/>
+      <c r="E69" s="19" t="str">
+        <f aca="false">IF(D69="","",D69*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="14"/>
       <c r="B70" s="15"/>
       <c r="C70" s="15"/>
       <c r="D70" s="18"/>
-      <c r="E70" s="16"/>
+      <c r="E70" s="19" t="str">
+        <f aca="false">IF(D70="","",D70*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="14"/>
       <c r="B71" s="15"/>
       <c r="C71" s="15"/>
       <c r="D71" s="18"/>
-      <c r="E71" s="16"/>
+      <c r="E71" s="19" t="str">
+        <f aca="false">IF(D71="","",D71*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="14"/>
       <c r="B72" s="15"/>
       <c r="C72" s="15"/>
       <c r="D72" s="18"/>
-      <c r="E72" s="16"/>
+      <c r="E72" s="19" t="str">
+        <f aca="false">IF(D72="","",D72*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="14"/>
       <c r="B73" s="15"/>
       <c r="C73" s="15"/>
       <c r="D73" s="18"/>
-      <c r="E73" s="16"/>
+      <c r="E73" s="19" t="str">
+        <f aca="false">IF(D73="","",D73*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="14"/>
       <c r="B74" s="15"/>
       <c r="C74" s="15"/>
       <c r="D74" s="18"/>
-      <c r="E74" s="16"/>
+      <c r="E74" s="19" t="str">
+        <f aca="false">IF(D74="","",D74*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="14"/>
       <c r="B75" s="15"/>
       <c r="C75" s="15"/>
       <c r="D75" s="18"/>
-      <c r="E75" s="16"/>
+      <c r="E75" s="19" t="str">
+        <f aca="false">IF(D75="","",D75*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="14"/>
       <c r="B76" s="15"/>
       <c r="C76" s="15"/>
       <c r="D76" s="18"/>
-      <c r="E76" s="16"/>
+      <c r="E76" s="19" t="str">
+        <f aca="false">IF(D76="","",D76*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="14"/>
       <c r="B77" s="15"/>
       <c r="C77" s="15"/>
       <c r="D77" s="18"/>
-      <c r="E77" s="16"/>
+      <c r="E77" s="19" t="str">
+        <f aca="false">IF(D77="","",D77*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="14"/>
       <c r="B78" s="15"/>
       <c r="C78" s="15"/>
       <c r="D78" s="18"/>
-      <c r="E78" s="16"/>
+      <c r="E78" s="19" t="str">
+        <f aca="false">IF(D78="","",D78*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="14"/>
       <c r="B79" s="15"/>
       <c r="C79" s="15"/>
       <c r="D79" s="18"/>
-      <c r="E79" s="16"/>
+      <c r="E79" s="19" t="str">
+        <f aca="false">IF(D79="","",D79*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="14"/>
       <c r="B80" s="15"/>
       <c r="C80" s="15"/>
       <c r="D80" s="18"/>
-      <c r="E80" s="16"/>
+      <c r="E80" s="19" t="str">
+        <f aca="false">IF(D80="","",D80*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="14"/>
       <c r="B81" s="15"/>
       <c r="C81" s="15"/>
       <c r="D81" s="18"/>
-      <c r="E81" s="16"/>
+      <c r="E81" s="19" t="str">
+        <f aca="false">IF(D81="","",D81*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="14"/>
       <c r="B82" s="15"/>
       <c r="C82" s="15"/>
       <c r="D82" s="18"/>
-      <c r="E82" s="16"/>
+      <c r="E82" s="19" t="str">
+        <f aca="false">IF(D82="","",D82*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="14"/>
       <c r="B83" s="15"/>
       <c r="C83" s="15"/>
       <c r="D83" s="18"/>
-      <c r="E83" s="16"/>
+      <c r="E83" s="19" t="str">
+        <f aca="false">IF(D83="","",D83*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="14"/>
       <c r="B84" s="15"/>
       <c r="C84" s="15"/>
       <c r="D84" s="18"/>
-      <c r="E84" s="16"/>
+      <c r="E84" s="19" t="str">
+        <f aca="false">IF(D84="","",D84*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="14"/>
       <c r="B85" s="15"/>
       <c r="C85" s="15"/>
       <c r="D85" s="18"/>
-      <c r="E85" s="16"/>
+      <c r="E85" s="19" t="str">
+        <f aca="false">IF(D85="","",D85*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="14"/>
       <c r="B86" s="15"/>
       <c r="C86" s="15"/>
       <c r="D86" s="18"/>
-      <c r="E86" s="16"/>
+      <c r="E86" s="19" t="str">
+        <f aca="false">IF(D86="","",D86*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="14"/>
       <c r="B87" s="15"/>
       <c r="C87" s="15"/>
       <c r="D87" s="18"/>
-      <c r="E87" s="16"/>
+      <c r="E87" s="19" t="str">
+        <f aca="false">IF(D87="","",D87*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="14"/>
       <c r="B88" s="15"/>
       <c r="C88" s="15"/>
       <c r="D88" s="18"/>
-      <c r="E88" s="16"/>
+      <c r="E88" s="19" t="str">
+        <f aca="false">IF(D88="","",D88*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="14"/>
       <c r="B89" s="15"/>
       <c r="C89" s="15"/>
       <c r="D89" s="18"/>
-      <c r="E89" s="16"/>
+      <c r="E89" s="19" t="str">
+        <f aca="false">IF(D89="","",D89*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="14"/>
       <c r="B90" s="15"/>
       <c r="C90" s="15"/>
       <c r="D90" s="18"/>
-      <c r="E90" s="16"/>
+      <c r="E90" s="19" t="str">
+        <f aca="false">IF(D90="","",D90*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="14"/>
       <c r="B91" s="15"/>
       <c r="C91" s="15"/>
       <c r="D91" s="18"/>
-      <c r="E91" s="16"/>
+      <c r="E91" s="19" t="str">
+        <f aca="false">IF(D91="","",D91*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="14"/>
       <c r="B92" s="15"/>
       <c r="C92" s="15"/>
       <c r="D92" s="18"/>
-      <c r="E92" s="16"/>
+      <c r="E92" s="19" t="str">
+        <f aca="false">IF(D92="","",D92*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="14"/>
       <c r="B93" s="15"/>
       <c r="C93" s="15"/>
       <c r="D93" s="18"/>
-      <c r="E93" s="16"/>
+      <c r="E93" s="19" t="str">
+        <f aca="false">IF(D93="","",D93*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="14"/>
       <c r="B94" s="15"/>
       <c r="C94" s="15"/>
       <c r="D94" s="18"/>
-      <c r="E94" s="16"/>
+      <c r="E94" s="19" t="str">
+        <f aca="false">IF(D94="","",D94*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="14"/>
       <c r="B95" s="15"/>
       <c r="C95" s="15"/>
       <c r="D95" s="18"/>
-      <c r="E95" s="16"/>
+      <c r="E95" s="19" t="str">
+        <f aca="false">IF(D95="","",D95*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="14"/>
       <c r="B96" s="15"/>
       <c r="C96" s="15"/>
       <c r="D96" s="18"/>
-      <c r="E96" s="16"/>
+      <c r="E96" s="19" t="str">
+        <f aca="false">IF(D96="","",D96*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="14"/>
       <c r="B97" s="15"/>
       <c r="C97" s="15"/>
       <c r="D97" s="18"/>
-      <c r="E97" s="16"/>
+      <c r="E97" s="19" t="str">
+        <f aca="false">IF(D97="","",D97*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="14"/>
       <c r="B98" s="15"/>
       <c r="C98" s="15"/>
       <c r="D98" s="18"/>
-      <c r="E98" s="16"/>
+      <c r="E98" s="19" t="str">
+        <f aca="false">IF(D98="","",D98*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="14"/>
       <c r="B99" s="15"/>
       <c r="C99" s="15"/>
       <c r="D99" s="18"/>
-      <c r="E99" s="16"/>
+      <c r="E99" s="19" t="str">
+        <f aca="false">IF(D99="","",D99*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="14"/>
       <c r="B100" s="15"/>
       <c r="C100" s="15"/>
       <c r="D100" s="18"/>
-      <c r="E100" s="16"/>
+      <c r="E100" s="19" t="str">
+        <f aca="false">IF(D100="","",D100*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="14"/>
       <c r="B101" s="15"/>
       <c r="C101" s="15"/>
       <c r="D101" s="18"/>
-      <c r="E101" s="16"/>
+      <c r="E101" s="19" t="str">
+        <f aca="false">IF(D101="","",D101*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="14"/>
       <c r="B102" s="15"/>
       <c r="C102" s="15"/>
       <c r="D102" s="18"/>
-      <c r="E102" s="16"/>
+      <c r="E102" s="19" t="str">
+        <f aca="false">IF(D102="","",D102*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="14"/>
       <c r="B103" s="15"/>
       <c r="C103" s="15"/>
       <c r="D103" s="18"/>
-      <c r="E103" s="16"/>
+      <c r="E103" s="19" t="str">
+        <f aca="false">IF(D103="","",D103*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="14"/>
       <c r="B104" s="15"/>
       <c r="C104" s="15"/>
       <c r="D104" s="18"/>
-      <c r="E104" s="16"/>
+      <c r="E104" s="19" t="str">
+        <f aca="false">IF(D104="","",D104*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="14"/>
       <c r="B105" s="15"/>
       <c r="C105" s="15"/>
       <c r="D105" s="18"/>
-      <c r="E105" s="16"/>
+      <c r="E105" s="19" t="str">
+        <f aca="false">IF(D105="","",D105*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="14"/>
       <c r="B106" s="15"/>
       <c r="C106" s="15"/>
       <c r="D106" s="18"/>
-      <c r="E106" s="16"/>
+      <c r="E106" s="19" t="str">
+        <f aca="false">IF(D106="","",D106*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="14"/>
       <c r="B107" s="15"/>
       <c r="C107" s="15"/>
       <c r="D107" s="18"/>
-      <c r="E107" s="16"/>
+      <c r="E107" s="19" t="str">
+        <f aca="false">IF(D107="","",D107*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="14"/>
       <c r="B108" s="15"/>
       <c r="C108" s="15"/>
       <c r="D108" s="18"/>
-      <c r="E108" s="16"/>
+      <c r="E108" s="19" t="str">
+        <f aca="false">IF(D108="","",D108*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="14"/>
       <c r="B109" s="15"/>
       <c r="C109" s="15"/>
       <c r="D109" s="18"/>
-      <c r="E109" s="16"/>
+      <c r="E109" s="19" t="str">
+        <f aca="false">IF(D109="","",D109*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="14"/>
       <c r="B110" s="15"/>
       <c r="C110" s="15"/>
       <c r="D110" s="18"/>
-      <c r="E110" s="16"/>
+      <c r="E110" s="19" t="str">
+        <f aca="false">IF(D110="","",D110*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="14"/>
       <c r="B111" s="15"/>
       <c r="C111" s="15"/>
       <c r="D111" s="18"/>
-      <c r="E111" s="16"/>
+      <c r="E111" s="19" t="str">
+        <f aca="false">IF(D111="","",D111*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="14"/>
       <c r="B112" s="15"/>
       <c r="C112" s="15"/>
       <c r="D112" s="18"/>
-      <c r="E112" s="16"/>
+      <c r="E112" s="19" t="str">
+        <f aca="false">IF(D112="","",D112*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="14"/>
       <c r="B113" s="15"/>
       <c r="C113" s="15"/>
       <c r="D113" s="18"/>
-      <c r="E113" s="16"/>
+      <c r="E113" s="19" t="str">
+        <f aca="false">IF(D113="","",D113*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="14"/>
       <c r="B114" s="15"/>
       <c r="C114" s="15"/>
       <c r="D114" s="18"/>
-      <c r="E114" s="16"/>
+      <c r="E114" s="19" t="str">
+        <f aca="false">IF(D114="","",D114*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="14"/>
       <c r="B115" s="15"/>
       <c r="C115" s="15"/>
       <c r="D115" s="18"/>
-      <c r="E115" s="16"/>
+      <c r="E115" s="19" t="str">
+        <f aca="false">IF(D115="","",D115*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="14"/>
       <c r="B116" s="15"/>
       <c r="C116" s="15"/>
       <c r="D116" s="18"/>
-      <c r="E116" s="16"/>
+      <c r="E116" s="19" t="str">
+        <f aca="false">IF(D116="","",D116*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="14"/>
       <c r="B117" s="15"/>
       <c r="C117" s="15"/>
       <c r="D117" s="18"/>
-      <c r="E117" s="16"/>
+      <c r="E117" s="19" t="str">
+        <f aca="false">IF(D117="","",D117*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="14"/>
       <c r="B118" s="15"/>
       <c r="C118" s="15"/>
       <c r="D118" s="18"/>
-      <c r="E118" s="16"/>
+      <c r="E118" s="19" t="str">
+        <f aca="false">IF(D118="","",D118*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="14"/>
       <c r="B119" s="15"/>
       <c r="C119" s="15"/>
       <c r="D119" s="18"/>
-      <c r="E119" s="16"/>
+      <c r="E119" s="19" t="str">
+        <f aca="false">IF(D119="","",D119*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="14"/>
       <c r="B120" s="15"/>
       <c r="C120" s="15"/>
       <c r="D120" s="18"/>
-      <c r="E120" s="16"/>
+      <c r="E120" s="19" t="str">
+        <f aca="false">IF(D120="","",D120*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="14"/>
       <c r="B121" s="15"/>
       <c r="C121" s="15"/>
       <c r="D121" s="18"/>
-      <c r="E121" s="16"/>
+      <c r="E121" s="19" t="str">
+        <f aca="false">IF(D121="","",D121*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="14"/>
       <c r="B122" s="15"/>
       <c r="C122" s="15"/>
       <c r="D122" s="18"/>
-      <c r="E122" s="16"/>
+      <c r="E122" s="19" t="str">
+        <f aca="false">IF(D122="","",D122*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="14"/>
       <c r="B123" s="15"/>
       <c r="C123" s="15"/>
       <c r="D123" s="18"/>
-      <c r="E123" s="16"/>
+      <c r="E123" s="19" t="str">
+        <f aca="false">IF(D123="","",D123*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="14"/>
       <c r="B124" s="15"/>
       <c r="C124" s="15"/>
       <c r="D124" s="18"/>
-      <c r="E124" s="16"/>
+      <c r="E124" s="19" t="str">
+        <f aca="false">IF(D124="","",D124*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="14"/>
       <c r="B125" s="15"/>
       <c r="C125" s="15"/>
       <c r="D125" s="18"/>
-      <c r="E125" s="16"/>
+      <c r="E125" s="19" t="str">
+        <f aca="false">IF(D125="","",D125*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="14"/>
       <c r="B126" s="15"/>
       <c r="C126" s="15"/>
       <c r="D126" s="18"/>
-      <c r="E126" s="16"/>
+      <c r="E126" s="19" t="str">
+        <f aca="false">IF(D126="","",D126*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="14"/>
       <c r="B127" s="15"/>
       <c r="C127" s="15"/>
       <c r="D127" s="18"/>
-      <c r="E127" s="16"/>
+      <c r="E127" s="19" t="str">
+        <f aca="false">IF(D127="","",D127*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="14"/>
       <c r="B128" s="15"/>
       <c r="C128" s="15"/>
       <c r="D128" s="18"/>
-      <c r="E128" s="16"/>
+      <c r="E128" s="19" t="str">
+        <f aca="false">IF(D128="","",D128*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="14"/>
       <c r="B129" s="15"/>
       <c r="C129" s="15"/>
       <c r="D129" s="18"/>
-      <c r="E129" s="16"/>
+      <c r="E129" s="19" t="str">
+        <f aca="false">IF(D129="","",D129*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="14"/>
       <c r="B130" s="15"/>
       <c r="C130" s="15"/>
       <c r="D130" s="18"/>
-      <c r="E130" s="16"/>
+      <c r="E130" s="19" t="str">
+        <f aca="false">IF(D130="","",D130*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="14"/>
       <c r="B131" s="15"/>
       <c r="C131" s="15"/>
       <c r="D131" s="18"/>
-      <c r="E131" s="16"/>
+      <c r="E131" s="19" t="str">
+        <f aca="false">IF(D131="","",D131*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="14"/>
       <c r="B132" s="15"/>
       <c r="C132" s="15"/>
       <c r="D132" s="18"/>
-      <c r="E132" s="16"/>
+      <c r="E132" s="19" t="str">
+        <f aca="false">IF(D132="","",D132*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="14"/>
       <c r="B133" s="15"/>
       <c r="C133" s="15"/>
       <c r="D133" s="18"/>
-      <c r="E133" s="16"/>
+      <c r="E133" s="19" t="str">
+        <f aca="false">IF(D133="","",D133*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="14"/>
       <c r="B134" s="15"/>
       <c r="C134" s="15"/>
       <c r="D134" s="18"/>
-      <c r="E134" s="16"/>
+      <c r="E134" s="19" t="str">
+        <f aca="false">IF(D134="","",D134*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="14"/>
       <c r="B135" s="15"/>
       <c r="C135" s="15"/>
       <c r="D135" s="18"/>
-      <c r="E135" s="16"/>
+      <c r="E135" s="19" t="str">
+        <f aca="false">IF(D135="","",D135*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="14"/>
       <c r="B136" s="15"/>
       <c r="C136" s="15"/>
       <c r="D136" s="18"/>
-      <c r="E136" s="16"/>
+      <c r="E136" s="19" t="str">
+        <f aca="false">IF(D136="","",D136*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="14"/>
       <c r="B137" s="15"/>
       <c r="C137" s="15"/>
       <c r="D137" s="18"/>
-      <c r="E137" s="16"/>
+      <c r="E137" s="19" t="str">
+        <f aca="false">IF(D137="","",D137*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="14"/>
       <c r="B138" s="15"/>
       <c r="C138" s="15"/>
       <c r="D138" s="18"/>
-      <c r="E138" s="16"/>
+      <c r="E138" s="19" t="str">
+        <f aca="false">IF(D138="","",D138*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="14"/>
       <c r="B139" s="15"/>
       <c r="C139" s="15"/>
       <c r="D139" s="18"/>
-      <c r="E139" s="16"/>
+      <c r="E139" s="19" t="str">
+        <f aca="false">IF(D139="","",D139*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="14"/>
       <c r="B140" s="15"/>
       <c r="C140" s="15"/>
       <c r="D140" s="18"/>
-      <c r="E140" s="16"/>
+      <c r="E140" s="19" t="str">
+        <f aca="false">IF(D140="","",D140*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="14"/>
       <c r="B141" s="15"/>
       <c r="C141" s="15"/>
       <c r="D141" s="18"/>
-      <c r="E141" s="16"/>
+      <c r="E141" s="19" t="str">
+        <f aca="false">IF(D141="","",D141*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="14"/>
       <c r="B142" s="15"/>
       <c r="C142" s="15"/>
       <c r="D142" s="18"/>
-      <c r="E142" s="16"/>
+      <c r="E142" s="19" t="str">
+        <f aca="false">IF(D142="","",D142*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="14"/>
       <c r="B143" s="15"/>
       <c r="C143" s="15"/>
       <c r="D143" s="18"/>
-      <c r="E143" s="16"/>
+      <c r="E143" s="19" t="str">
+        <f aca="false">IF(D143="","",D143*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="14"/>
       <c r="B144" s="15"/>
       <c r="C144" s="15"/>
       <c r="D144" s="18"/>
-      <c r="E144" s="16"/>
+      <c r="E144" s="19" t="str">
+        <f aca="false">IF(D144="","",D144*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="14"/>
       <c r="B145" s="15"/>
       <c r="C145" s="15"/>
       <c r="D145" s="18"/>
-      <c r="E145" s="16"/>
+      <c r="E145" s="19" t="str">
+        <f aca="false">IF(D145="","",D145*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="14"/>
       <c r="B146" s="15"/>
       <c r="C146" s="15"/>
       <c r="D146" s="18"/>
-      <c r="E146" s="16"/>
+      <c r="E146" s="19" t="str">
+        <f aca="false">IF(D146="","",D146*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="14"/>
       <c r="B147" s="15"/>
       <c r="C147" s="15"/>
       <c r="D147" s="18"/>
-      <c r="E147" s="16"/>
+      <c r="E147" s="19" t="str">
+        <f aca="false">IF(D147="","",D147*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="14"/>
       <c r="B148" s="15"/>
       <c r="C148" s="15"/>
       <c r="D148" s="18"/>
-      <c r="E148" s="16"/>
+      <c r="E148" s="19" t="str">
+        <f aca="false">IF(D148="","",D148*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="14"/>
       <c r="B149" s="15"/>
       <c r="C149" s="15"/>
       <c r="D149" s="18"/>
-      <c r="E149" s="16"/>
+      <c r="E149" s="19" t="str">
+        <f aca="false">IF(D149="","",D149*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="14"/>
       <c r="B150" s="15"/>
       <c r="C150" s="15"/>
       <c r="D150" s="18"/>
-      <c r="E150" s="16"/>
+      <c r="E150" s="19" t="str">
+        <f aca="false">IF(D150="","",D150*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="14"/>
       <c r="B151" s="15"/>
       <c r="C151" s="15"/>
       <c r="D151" s="18"/>
-      <c r="E151" s="16"/>
+      <c r="E151" s="19" t="str">
+        <f aca="false">IF(D151="","",D151*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="14"/>
       <c r="B152" s="15"/>
       <c r="C152" s="15"/>
       <c r="D152" s="18"/>
-      <c r="E152" s="16"/>
+      <c r="E152" s="19" t="str">
+        <f aca="false">IF(D152="","",D152*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="14"/>
       <c r="B153" s="15"/>
       <c r="C153" s="15"/>
       <c r="D153" s="18"/>
-      <c r="E153" s="16"/>
+      <c r="E153" s="19" t="str">
+        <f aca="false">IF(D153="","",D153*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="14"/>
       <c r="B154" s="15"/>
       <c r="C154" s="15"/>
       <c r="D154" s="18"/>
-      <c r="E154" s="16"/>
+      <c r="E154" s="19" t="str">
+        <f aca="false">IF(D154="","",D154*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="14"/>
       <c r="B155" s="15"/>
       <c r="C155" s="15"/>
       <c r="D155" s="18"/>
-      <c r="E155" s="16"/>
+      <c r="E155" s="19" t="str">
+        <f aca="false">IF(D155="","",D155*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="14"/>
       <c r="B156" s="15"/>
       <c r="C156" s="15"/>
       <c r="D156" s="18"/>
-      <c r="E156" s="16"/>
+      <c r="E156" s="19" t="str">
+        <f aca="false">IF(D156="","",D156*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="14"/>
       <c r="B157" s="15"/>
       <c r="C157" s="15"/>
       <c r="D157" s="18"/>
-      <c r="E157" s="16"/>
+      <c r="E157" s="19" t="str">
+        <f aca="false">IF(D157="","",D157*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="14"/>
       <c r="B158" s="15"/>
       <c r="C158" s="15"/>
       <c r="D158" s="18"/>
-      <c r="E158" s="16"/>
+      <c r="E158" s="19" t="str">
+        <f aca="false">IF(D158="","",D158*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="14"/>
       <c r="B159" s="15"/>
       <c r="C159" s="15"/>
       <c r="D159" s="18"/>
-      <c r="E159" s="16"/>
+      <c r="E159" s="19" t="str">
+        <f aca="false">IF(D159="","",D159*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="14"/>
       <c r="B160" s="15"/>
       <c r="C160" s="15"/>
       <c r="D160" s="18"/>
-      <c r="E160" s="16"/>
+      <c r="E160" s="19" t="str">
+        <f aca="false">IF(D160="","",D160*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="14"/>
       <c r="B161" s="15"/>
       <c r="C161" s="15"/>
       <c r="D161" s="18"/>
-      <c r="E161" s="16"/>
+      <c r="E161" s="19" t="str">
+        <f aca="false">IF(D161="","",D161*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="14"/>
       <c r="B162" s="15"/>
       <c r="C162" s="15"/>
       <c r="D162" s="18"/>
-      <c r="E162" s="16"/>
+      <c r="E162" s="19" t="str">
+        <f aca="false">IF(D162="","",D162*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="14"/>
       <c r="B163" s="15"/>
       <c r="C163" s="15"/>
       <c r="D163" s="18"/>
-      <c r="E163" s="16"/>
+      <c r="E163" s="19" t="str">
+        <f aca="false">IF(D163="","",D163*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="14"/>
       <c r="B164" s="15"/>
       <c r="C164" s="15"/>
       <c r="D164" s="18"/>
-      <c r="E164" s="16"/>
+      <c r="E164" s="19" t="str">
+        <f aca="false">IF(D164="","",D164*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="14"/>
       <c r="B165" s="15"/>
       <c r="C165" s="15"/>
       <c r="D165" s="18"/>
-      <c r="E165" s="16"/>
+      <c r="E165" s="19" t="str">
+        <f aca="false">IF(D165="","",D165*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="14"/>
       <c r="B166" s="15"/>
       <c r="C166" s="15"/>
       <c r="D166" s="18"/>
-      <c r="E166" s="16"/>
+      <c r="E166" s="19" t="str">
+        <f aca="false">IF(D166="","",D166*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="14"/>
       <c r="B167" s="15"/>
       <c r="C167" s="15"/>
       <c r="D167" s="18"/>
-      <c r="E167" s="16"/>
+      <c r="E167" s="19" t="str">
+        <f aca="false">IF(D167="","",D167*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="14"/>
       <c r="B168" s="15"/>
       <c r="C168" s="15"/>
       <c r="D168" s="18"/>
-      <c r="E168" s="16"/>
+      <c r="E168" s="19" t="str">
+        <f aca="false">IF(D168="","",D168*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="14"/>
       <c r="B169" s="15"/>
       <c r="C169" s="15"/>
       <c r="D169" s="18"/>
-      <c r="E169" s="16"/>
+      <c r="E169" s="19" t="str">
+        <f aca="false">IF(D169="","",D169*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="14"/>
       <c r="B170" s="15"/>
       <c r="C170" s="15"/>
       <c r="D170" s="18"/>
-      <c r="E170" s="16"/>
+      <c r="E170" s="19" t="str">
+        <f aca="false">IF(D170="","",D170*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="14"/>
       <c r="B171" s="15"/>
       <c r="C171" s="15"/>
       <c r="D171" s="18"/>
-      <c r="E171" s="16"/>
+      <c r="E171" s="19" t="str">
+        <f aca="false">IF(D171="","",D171*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="14"/>
       <c r="B172" s="15"/>
       <c r="C172" s="15"/>
       <c r="D172" s="18"/>
-      <c r="E172" s="16"/>
+      <c r="E172" s="19" t="str">
+        <f aca="false">IF(D172="","",D172*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="14"/>
       <c r="B173" s="15"/>
       <c r="C173" s="15"/>
       <c r="D173" s="18"/>
-      <c r="E173" s="16"/>
+      <c r="E173" s="19" t="str">
+        <f aca="false">IF(D173="","",D173*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="14"/>
       <c r="B174" s="15"/>
       <c r="C174" s="15"/>
       <c r="D174" s="18"/>
-      <c r="E174" s="16"/>
+      <c r="E174" s="19" t="str">
+        <f aca="false">IF(D174="","",D174*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="14"/>
       <c r="B175" s="15"/>
       <c r="C175" s="15"/>
       <c r="D175" s="18"/>
-      <c r="E175" s="16"/>
+      <c r="E175" s="19" t="str">
+        <f aca="false">IF(D175="","",D175*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="14"/>
       <c r="B176" s="15"/>
       <c r="C176" s="15"/>
       <c r="D176" s="18"/>
-      <c r="E176" s="16"/>
+      <c r="E176" s="19" t="str">
+        <f aca="false">IF(D176="","",D176*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="14"/>
       <c r="B177" s="15"/>
       <c r="C177" s="15"/>
       <c r="D177" s="18"/>
-      <c r="E177" s="16"/>
+      <c r="E177" s="19" t="str">
+        <f aca="false">IF(D177="","",D177*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="14"/>
       <c r="B178" s="15"/>
       <c r="C178" s="15"/>
       <c r="D178" s="18"/>
-      <c r="E178" s="16"/>
+      <c r="E178" s="19" t="str">
+        <f aca="false">IF(D178="","",D178*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="14"/>
       <c r="B179" s="15"/>
       <c r="C179" s="15"/>
       <c r="D179" s="18"/>
-      <c r="E179" s="16"/>
+      <c r="E179" s="19" t="str">
+        <f aca="false">IF(D179="","",D179*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="14"/>
       <c r="B180" s="15"/>
       <c r="C180" s="15"/>
       <c r="D180" s="18"/>
-      <c r="E180" s="16"/>
+      <c r="E180" s="19" t="str">
+        <f aca="false">IF(D180="","",D180*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="14"/>
       <c r="B181" s="15"/>
       <c r="C181" s="15"/>
       <c r="D181" s="18"/>
-      <c r="E181" s="16"/>
+      <c r="E181" s="19" t="str">
+        <f aca="false">IF(D181="","",D181*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="14"/>
       <c r="B182" s="15"/>
       <c r="C182" s="15"/>
       <c r="D182" s="18"/>
-      <c r="E182" s="16"/>
+      <c r="E182" s="19" t="str">
+        <f aca="false">IF(D182="","",D182*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="14"/>
       <c r="B183" s="15"/>
       <c r="C183" s="15"/>
       <c r="D183" s="18"/>
-      <c r="E183" s="16"/>
+      <c r="E183" s="19" t="str">
+        <f aca="false">IF(D183="","",D183*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="14"/>
       <c r="B184" s="15"/>
       <c r="C184" s="15"/>
       <c r="D184" s="18"/>
-      <c r="E184" s="16"/>
+      <c r="E184" s="19" t="str">
+        <f aca="false">IF(D184="","",D184*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="14"/>
       <c r="B185" s="15"/>
       <c r="C185" s="15"/>
       <c r="D185" s="18"/>
-      <c r="E185" s="16"/>
+      <c r="E185" s="19" t="str">
+        <f aca="false">IF(D185="","",D185*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="14"/>
       <c r="B186" s="15"/>
       <c r="C186" s="15"/>
       <c r="D186" s="18"/>
-      <c r="E186" s="16"/>
+      <c r="E186" s="19" t="str">
+        <f aca="false">IF(D186="","",D186*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="14"/>
       <c r="B187" s="15"/>
       <c r="C187" s="15"/>
       <c r="D187" s="18"/>
-      <c r="E187" s="16"/>
+      <c r="E187" s="19" t="str">
+        <f aca="false">IF(D187="","",D187*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="14"/>
       <c r="B188" s="15"/>
       <c r="C188" s="15"/>
       <c r="D188" s="18"/>
-      <c r="E188" s="16"/>
+      <c r="E188" s="19" t="str">
+        <f aca="false">IF(D188="","",D188*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="14"/>
       <c r="B189" s="15"/>
       <c r="C189" s="15"/>
       <c r="D189" s="18"/>
-      <c r="E189" s="16"/>
+      <c r="E189" s="19" t="str">
+        <f aca="false">IF(D189="","",D189*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="14"/>
       <c r="B190" s="15"/>
       <c r="C190" s="15"/>
       <c r="D190" s="18"/>
-      <c r="E190" s="16"/>
+      <c r="E190" s="19" t="str">
+        <f aca="false">IF(D190="","",D190*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="14"/>
       <c r="B191" s="15"/>
       <c r="C191" s="15"/>
       <c r="D191" s="18"/>
-      <c r="E191" s="16"/>
+      <c r="E191" s="19" t="str">
+        <f aca="false">IF(D191="","",D191*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="14"/>
       <c r="B192" s="15"/>
       <c r="C192" s="15"/>
       <c r="D192" s="18"/>
-      <c r="E192" s="16"/>
+      <c r="E192" s="19" t="str">
+        <f aca="false">IF(D192="","",D192*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="14"/>
       <c r="B193" s="15"/>
       <c r="C193" s="15"/>
       <c r="D193" s="18"/>
-      <c r="E193" s="16"/>
+      <c r="E193" s="19" t="str">
+        <f aca="false">IF(D193="","",D193*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="14"/>
       <c r="B194" s="15"/>
       <c r="C194" s="15"/>
       <c r="D194" s="18"/>
-      <c r="E194" s="16"/>
+      <c r="E194" s="19" t="str">
+        <f aca="false">IF(D194="","",D194*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="14"/>
       <c r="B195" s="15"/>
       <c r="C195" s="15"/>
       <c r="D195" s="18"/>
-      <c r="E195" s="16"/>
+      <c r="E195" s="19" t="str">
+        <f aca="false">IF(D195="","",D195*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="14"/>
       <c r="B196" s="15"/>
       <c r="C196" s="15"/>
       <c r="D196" s="18"/>
-      <c r="E196" s="16"/>
+      <c r="E196" s="19" t="str">
+        <f aca="false">IF(D196="","",D196*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="14"/>
       <c r="B197" s="15"/>
       <c r="C197" s="15"/>
       <c r="D197" s="18"/>
-      <c r="E197" s="16"/>
+      <c r="E197" s="19" t="str">
+        <f aca="false">IF(D197="","",D197*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="14"/>
       <c r="B198" s="15"/>
       <c r="C198" s="15"/>
       <c r="D198" s="18"/>
-      <c r="E198" s="16"/>
+      <c r="E198" s="19" t="str">
+        <f aca="false">IF(D198="","",D198*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="14"/>
       <c r="B199" s="15"/>
       <c r="C199" s="15"/>
       <c r="D199" s="18"/>
-      <c r="E199" s="16"/>
+      <c r="E199" s="19" t="str">
+        <f aca="false">IF(D199="","",D199*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="14"/>
       <c r="B200" s="15"/>
       <c r="C200" s="15"/>
       <c r="D200" s="18"/>
-      <c r="E200" s="16"/>
+      <c r="E200" s="19" t="str">
+        <f aca="false">IF(D200="","",D200*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="14"/>
       <c r="B201" s="15"/>
       <c r="C201" s="15"/>
       <c r="D201" s="18"/>
-      <c r="E201" s="16"/>
+      <c r="E201" s="19" t="str">
+        <f aca="false">IF(D201="","",D201*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="14"/>
       <c r="B202" s="15"/>
       <c r="C202" s="15"/>
       <c r="D202" s="18"/>
-      <c r="E202" s="16"/>
+      <c r="E202" s="19" t="str">
+        <f aca="false">IF(D202="","",D202*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="14"/>
       <c r="B203" s="15"/>
       <c r="C203" s="15"/>
       <c r="D203" s="18"/>
-      <c r="E203" s="16"/>
+      <c r="E203" s="19" t="str">
+        <f aca="false">IF(D203="","",D203*$H$6)</f>
+        <v/>
+      </c>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="14"/>
       <c r="B204" s="15"/>
       <c r="C204" s="15"/>
       <c r="D204" s="18"/>
-      <c r="E204" s="16"/>
+      <c r="E204" s="19" t="str">
+        <f aca="false">IF(D204="","",D204*$H$6)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -3633,10 +4253,10 @@
       <c r="D4" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="19" t="s">
+      <c r="G4" s="21" t="s">
         <v>40</v>
       </c>
     </row>
@@ -3656,7 +4276,7 @@
       <c r="F5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="20" t="n">
+      <c r="G5" s="22" t="n">
         <f aca="false">SUMIF($B$5:$B$204,F5,$D$5:$D$204)</f>
         <v>12000</v>
       </c>
@@ -3669,7 +4289,7 @@
       <c r="F6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G6" s="20" t="n">
+      <c r="G6" s="22" t="n">
         <f aca="false">SUMIF($B$5:$B$204,F6,$D$5:$D$204)</f>
         <v>0</v>
       </c>
@@ -3682,7 +4302,7 @@
       <c r="F7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="20" t="n">
+      <c r="G7" s="22" t="n">
         <f aca="false">SUMIF($B$5:$B$204,F7,$D$5:$D$204)</f>
         <v>0</v>
       </c>
@@ -3695,7 +4315,7 @@
       <c r="F8" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="20" t="n">
+      <c r="G8" s="22" t="n">
         <f aca="false">SUMIF($B$5:$B$204,F8,$D$5:$D$204)</f>
         <v>0</v>
       </c>
@@ -3708,7 +4328,7 @@
       <c r="F9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="20" t="n">
+      <c r="G9" s="22" t="n">
         <f aca="false">SUMIF($B$5:$B$204,F9,$D$5:$D$204)</f>
         <v>0</v>
       </c>
@@ -3721,7 +4341,7 @@
       <c r="F10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="20" t="n">
+      <c r="G10" s="22" t="n">
         <f aca="false">SUMIF($B$5:$B$204,F10,$D$5:$D$204)</f>
         <v>0</v>
       </c>
@@ -3734,7 +4354,7 @@
       <c r="F11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="20" t="n">
+      <c r="G11" s="22" t="n">
         <f aca="false">SUMIF($B$5:$B$204,F11,$D$5:$D$204)</f>
         <v>0</v>
       </c>
@@ -3747,7 +4367,7 @@
       <c r="F12" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G12" s="21" t="n">
+      <c r="G12" s="23" t="n">
         <f aca="false">SUM(G5:G11)</f>
         <v>12000</v>
       </c>

</xml_diff>

<commit_message>
Textos en femenino, ¿qué reina sos? con colores, Pagado en rifa, Extra en gastos, barco animado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014cQS814DmisHJYTJthjhHq
</commit_message>
<xml_diff>
--- a/Finanzas_Proyecto.xlsx
+++ b/Finanzas_Proyecto.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="46">
   <si>
     <t xml:space="preserve">FINANZAS DEL PROYECTO</t>
   </si>
@@ -70,6 +70,9 @@
     <t xml:space="preserve">Comida</t>
   </si>
   <si>
+    <t xml:space="preserve">Extra</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTAL GASTOS</t>
   </si>
   <si>
@@ -82,7 +85,7 @@
     <t xml:space="preserve">RIFA DEL PESO</t>
   </si>
   <si>
-    <t xml:space="preserve">Celdas rosas = para completar. Una fila por recaudo; elegí el componente del menú. La fila 5 es un ejemplo: reemplazala.</t>
+    <t xml:space="preserve">Celdas rosas = para completar. Reina, detallá si transferís, pagás en efectivo o continúa pendiente. Marcá Sí en Pagado cuando esté cobrado. La fila 5 es un ejemplo: reemplazala.</t>
   </si>
   <si>
     <t xml:space="preserve">Fecha</t>
@@ -97,6 +100,9 @@
     <t xml:space="preserve">Monto recaudado</t>
   </si>
   <si>
+    <t xml:space="preserve">Pagado</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTAL RIFA</t>
   </si>
   <si>
@@ -104,6 +110,12 @@
   </si>
   <si>
     <t xml:space="preserve">Ejemplo: recaudo rifa del peso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sí</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
     <t xml:space="preserve">VENTA DE REMERAS</t>
@@ -136,7 +148,7 @@
     <t xml:space="preserve">Precio por unidad</t>
   </si>
   <si>
-    <t xml:space="preserve">Celdas rosas = para completar. Elegí la categoría del menú desplegable. La fila 5 es un ejemplo: reemplazala.</t>
+    <t xml:space="preserve">Celdas rosas = para completar. Elegí la categoría. Editable para grupo finanzas: si hiciste algún mandado, elegí la categoría Extra y especificá en el renglón. La fila 5 es un ejemplo: reemplazala.</t>
   </si>
   <si>
     <t xml:space="preserve">Categoría</t>
@@ -690,7 +702,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -718,7 +730,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="n">
-        <f aca="false">'Rifa del Peso'!G4</f>
+        <f aca="false">'Rifa del Peso'!H4</f>
         <v>25000</v>
       </c>
     </row>
@@ -819,26 +831,35 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="8" t="n">
-        <f aca="false">SUM(B11:B17)</f>
+      <c r="B18" s="5" t="n">
+        <f aca="false">Gastos!G12</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19" s="8" t="n">
+        <f aca="false">SUM(B11:B18)</f>
         <v>12000</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B20" s="3"/>
-    </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="10" t="n">
-        <f aca="false">B8-B18</f>
+      <c r="B21" s="3"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="10" t="n">
+        <f aca="false">B8-B19</f>
         <v>14470</v>
       </c>
     </row>
@@ -858,44 +879,48 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G204"/>
+  <dimension ref="A1:H204"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="G4" s="13" t="n">
+      <c r="E4" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="13" t="n">
         <f aca="false">SUM(D5:D204)</f>
         <v>25000</v>
       </c>
@@ -905,12 +930,22 @@
         <v>46310</v>
       </c>
       <c r="B5" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>25000</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="16" t="n">
+      <c r="H5" s="13" t="n">
+        <f aca="false">SUMIF(E5:E204,"Sí",D5:D204)</f>
         <v>25000</v>
       </c>
     </row>
@@ -919,1199 +954,1409 @@
       <c r="B6" s="15"/>
       <c r="C6" s="15"/>
       <c r="D6" s="16"/>
+      <c r="E6" s="15"/>
+      <c r="G6" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6" s="13" t="n">
+        <f aca="false">H4-H5</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="16"/>
+      <c r="E7" s="15"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="16"/>
+      <c r="E8" s="15"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14"/>
       <c r="B9" s="15"/>
       <c r="C9" s="15"/>
       <c r="D9" s="16"/>
+      <c r="E9" s="15"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14"/>
       <c r="B10" s="15"/>
       <c r="C10" s="15"/>
       <c r="D10" s="16"/>
+      <c r="E10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14"/>
       <c r="B11" s="15"/>
       <c r="C11" s="15"/>
       <c r="D11" s="16"/>
+      <c r="E11" s="15"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14"/>
       <c r="B12" s="15"/>
       <c r="C12" s="15"/>
       <c r="D12" s="16"/>
+      <c r="E12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14"/>
       <c r="B13" s="15"/>
       <c r="C13" s="15"/>
       <c r="D13" s="16"/>
+      <c r="E13" s="15"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14"/>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
       <c r="D14" s="16"/>
+      <c r="E14" s="15"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14"/>
       <c r="B15" s="15"/>
       <c r="C15" s="15"/>
       <c r="D15" s="16"/>
+      <c r="E15" s="15"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14"/>
       <c r="B16" s="15"/>
       <c r="C16" s="15"/>
       <c r="D16" s="16"/>
+      <c r="E16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14"/>
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
       <c r="D17" s="16"/>
+      <c r="E17" s="15"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14"/>
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
       <c r="D18" s="16"/>
+      <c r="E18" s="15"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14"/>
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
       <c r="D19" s="16"/>
+      <c r="E19" s="15"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14"/>
       <c r="B20" s="15"/>
       <c r="C20" s="15"/>
       <c r="D20" s="16"/>
+      <c r="E20" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14"/>
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
       <c r="D21" s="16"/>
+      <c r="E21" s="15"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14"/>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
       <c r="D22" s="16"/>
+      <c r="E22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14"/>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
       <c r="D23" s="16"/>
+      <c r="E23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14"/>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
       <c r="D24" s="16"/>
+      <c r="E24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14"/>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
       <c r="D25" s="16"/>
+      <c r="E25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14"/>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
       <c r="D26" s="16"/>
+      <c r="E26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14"/>
       <c r="B27" s="15"/>
       <c r="C27" s="15"/>
       <c r="D27" s="16"/>
+      <c r="E27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14"/>
       <c r="B28" s="15"/>
       <c r="C28" s="15"/>
       <c r="D28" s="16"/>
+      <c r="E28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14"/>
       <c r="B29" s="15"/>
       <c r="C29" s="15"/>
       <c r="D29" s="16"/>
+      <c r="E29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14"/>
       <c r="B30" s="15"/>
       <c r="C30" s="15"/>
       <c r="D30" s="16"/>
+      <c r="E30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14"/>
       <c r="B31" s="15"/>
       <c r="C31" s="15"/>
       <c r="D31" s="16"/>
+      <c r="E31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14"/>
       <c r="B32" s="15"/>
       <c r="C32" s="15"/>
       <c r="D32" s="16"/>
+      <c r="E32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14"/>
       <c r="B33" s="15"/>
       <c r="C33" s="15"/>
       <c r="D33" s="16"/>
+      <c r="E33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14"/>
       <c r="B34" s="15"/>
       <c r="C34" s="15"/>
       <c r="D34" s="16"/>
+      <c r="E34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="14"/>
       <c r="B35" s="15"/>
       <c r="C35" s="15"/>
       <c r="D35" s="16"/>
+      <c r="E35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="14"/>
       <c r="B36" s="15"/>
       <c r="C36" s="15"/>
       <c r="D36" s="16"/>
+      <c r="E36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14"/>
       <c r="B37" s="15"/>
       <c r="C37" s="15"/>
       <c r="D37" s="16"/>
+      <c r="E37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14"/>
       <c r="B38" s="15"/>
       <c r="C38" s="15"/>
       <c r="D38" s="16"/>
+      <c r="E38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="14"/>
       <c r="B39" s="15"/>
       <c r="C39" s="15"/>
       <c r="D39" s="16"/>
+      <c r="E39" s="15"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="14"/>
       <c r="B40" s="15"/>
       <c r="C40" s="15"/>
       <c r="D40" s="16"/>
+      <c r="E40" s="15"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="14"/>
       <c r="B41" s="15"/>
       <c r="C41" s="15"/>
       <c r="D41" s="16"/>
+      <c r="E41" s="15"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14"/>
       <c r="B42" s="15"/>
       <c r="C42" s="15"/>
       <c r="D42" s="16"/>
+      <c r="E42" s="15"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="14"/>
       <c r="B43" s="15"/>
       <c r="C43" s="15"/>
       <c r="D43" s="16"/>
+      <c r="E43" s="15"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="14"/>
       <c r="B44" s="15"/>
       <c r="C44" s="15"/>
       <c r="D44" s="16"/>
+      <c r="E44" s="15"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="14"/>
       <c r="B45" s="15"/>
       <c r="C45" s="15"/>
       <c r="D45" s="16"/>
+      <c r="E45" s="15"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="14"/>
       <c r="B46" s="15"/>
       <c r="C46" s="15"/>
       <c r="D46" s="16"/>
+      <c r="E46" s="15"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="14"/>
       <c r="B47" s="15"/>
       <c r="C47" s="15"/>
       <c r="D47" s="16"/>
+      <c r="E47" s="15"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="14"/>
       <c r="B48" s="15"/>
       <c r="C48" s="15"/>
       <c r="D48" s="16"/>
+      <c r="E48" s="15"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="14"/>
       <c r="B49" s="15"/>
       <c r="C49" s="15"/>
       <c r="D49" s="16"/>
+      <c r="E49" s="15"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="14"/>
       <c r="B50" s="15"/>
       <c r="C50" s="15"/>
       <c r="D50" s="16"/>
+      <c r="E50" s="15"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="14"/>
       <c r="B51" s="15"/>
       <c r="C51" s="15"/>
       <c r="D51" s="16"/>
+      <c r="E51" s="15"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="14"/>
       <c r="B52" s="15"/>
       <c r="C52" s="15"/>
       <c r="D52" s="16"/>
+      <c r="E52" s="15"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="14"/>
       <c r="B53" s="15"/>
       <c r="C53" s="15"/>
       <c r="D53" s="16"/>
+      <c r="E53" s="15"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="14"/>
       <c r="B54" s="15"/>
       <c r="C54" s="15"/>
       <c r="D54" s="16"/>
+      <c r="E54" s="15"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="14"/>
       <c r="B55" s="15"/>
       <c r="C55" s="15"/>
       <c r="D55" s="16"/>
+      <c r="E55" s="15"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="14"/>
       <c r="B56" s="15"/>
       <c r="C56" s="15"/>
       <c r="D56" s="16"/>
+      <c r="E56" s="15"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="14"/>
       <c r="B57" s="15"/>
       <c r="C57" s="15"/>
       <c r="D57" s="16"/>
+      <c r="E57" s="15"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="14"/>
       <c r="B58" s="15"/>
       <c r="C58" s="15"/>
       <c r="D58" s="16"/>
+      <c r="E58" s="15"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="14"/>
       <c r="B59" s="15"/>
       <c r="C59" s="15"/>
       <c r="D59" s="16"/>
+      <c r="E59" s="15"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="14"/>
       <c r="B60" s="15"/>
       <c r="C60" s="15"/>
       <c r="D60" s="16"/>
+      <c r="E60" s="15"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="14"/>
       <c r="B61" s="15"/>
       <c r="C61" s="15"/>
       <c r="D61" s="16"/>
+      <c r="E61" s="15"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="14"/>
       <c r="B62" s="15"/>
       <c r="C62" s="15"/>
       <c r="D62" s="16"/>
+      <c r="E62" s="15"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="14"/>
       <c r="B63" s="15"/>
       <c r="C63" s="15"/>
       <c r="D63" s="16"/>
+      <c r="E63" s="15"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="14"/>
       <c r="B64" s="15"/>
       <c r="C64" s="15"/>
       <c r="D64" s="16"/>
+      <c r="E64" s="15"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="14"/>
       <c r="B65" s="15"/>
       <c r="C65" s="15"/>
       <c r="D65" s="16"/>
+      <c r="E65" s="15"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="14"/>
       <c r="B66" s="15"/>
       <c r="C66" s="15"/>
       <c r="D66" s="16"/>
+      <c r="E66" s="15"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="14"/>
       <c r="B67" s="15"/>
       <c r="C67" s="15"/>
       <c r="D67" s="16"/>
+      <c r="E67" s="15"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="14"/>
       <c r="B68" s="15"/>
       <c r="C68" s="15"/>
       <c r="D68" s="16"/>
+      <c r="E68" s="15"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="14"/>
       <c r="B69" s="15"/>
       <c r="C69" s="15"/>
       <c r="D69" s="16"/>
+      <c r="E69" s="15"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="14"/>
       <c r="B70" s="15"/>
       <c r="C70" s="15"/>
       <c r="D70" s="16"/>
+      <c r="E70" s="15"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="14"/>
       <c r="B71" s="15"/>
       <c r="C71" s="15"/>
       <c r="D71" s="16"/>
+      <c r="E71" s="15"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="14"/>
       <c r="B72" s="15"/>
       <c r="C72" s="15"/>
       <c r="D72" s="16"/>
+      <c r="E72" s="15"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="14"/>
       <c r="B73" s="15"/>
       <c r="C73" s="15"/>
       <c r="D73" s="16"/>
+      <c r="E73" s="15"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="14"/>
       <c r="B74" s="15"/>
       <c r="C74" s="15"/>
       <c r="D74" s="16"/>
+      <c r="E74" s="15"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="14"/>
       <c r="B75" s="15"/>
       <c r="C75" s="15"/>
       <c r="D75" s="16"/>
+      <c r="E75" s="15"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="14"/>
       <c r="B76" s="15"/>
       <c r="C76" s="15"/>
       <c r="D76" s="16"/>
+      <c r="E76" s="15"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="14"/>
       <c r="B77" s="15"/>
       <c r="C77" s="15"/>
       <c r="D77" s="16"/>
+      <c r="E77" s="15"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="14"/>
       <c r="B78" s="15"/>
       <c r="C78" s="15"/>
       <c r="D78" s="16"/>
+      <c r="E78" s="15"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="14"/>
       <c r="B79" s="15"/>
       <c r="C79" s="15"/>
       <c r="D79" s="16"/>
+      <c r="E79" s="15"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="14"/>
       <c r="B80" s="15"/>
       <c r="C80" s="15"/>
       <c r="D80" s="16"/>
+      <c r="E80" s="15"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="14"/>
       <c r="B81" s="15"/>
       <c r="C81" s="15"/>
       <c r="D81" s="16"/>
+      <c r="E81" s="15"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="14"/>
       <c r="B82" s="15"/>
       <c r="C82" s="15"/>
       <c r="D82" s="16"/>
+      <c r="E82" s="15"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="14"/>
       <c r="B83" s="15"/>
       <c r="C83" s="15"/>
       <c r="D83" s="16"/>
+      <c r="E83" s="15"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="14"/>
       <c r="B84" s="15"/>
       <c r="C84" s="15"/>
       <c r="D84" s="16"/>
+      <c r="E84" s="15"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="14"/>
       <c r="B85" s="15"/>
       <c r="C85" s="15"/>
       <c r="D85" s="16"/>
+      <c r="E85" s="15"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="14"/>
       <c r="B86" s="15"/>
       <c r="C86" s="15"/>
       <c r="D86" s="16"/>
+      <c r="E86" s="15"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="14"/>
       <c r="B87" s="15"/>
       <c r="C87" s="15"/>
       <c r="D87" s="16"/>
+      <c r="E87" s="15"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="14"/>
       <c r="B88" s="15"/>
       <c r="C88" s="15"/>
       <c r="D88" s="16"/>
+      <c r="E88" s="15"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="14"/>
       <c r="B89" s="15"/>
       <c r="C89" s="15"/>
       <c r="D89" s="16"/>
+      <c r="E89" s="15"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="14"/>
       <c r="B90" s="15"/>
       <c r="C90" s="15"/>
       <c r="D90" s="16"/>
+      <c r="E90" s="15"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="14"/>
       <c r="B91" s="15"/>
       <c r="C91" s="15"/>
       <c r="D91" s="16"/>
+      <c r="E91" s="15"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="14"/>
       <c r="B92" s="15"/>
       <c r="C92" s="15"/>
       <c r="D92" s="16"/>
+      <c r="E92" s="15"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="14"/>
       <c r="B93" s="15"/>
       <c r="C93" s="15"/>
       <c r="D93" s="16"/>
+      <c r="E93" s="15"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="14"/>
       <c r="B94" s="15"/>
       <c r="C94" s="15"/>
       <c r="D94" s="16"/>
+      <c r="E94" s="15"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="14"/>
       <c r="B95" s="15"/>
       <c r="C95" s="15"/>
       <c r="D95" s="16"/>
+      <c r="E95" s="15"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="14"/>
       <c r="B96" s="15"/>
       <c r="C96" s="15"/>
       <c r="D96" s="16"/>
+      <c r="E96" s="15"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="14"/>
       <c r="B97" s="15"/>
       <c r="C97" s="15"/>
       <c r="D97" s="16"/>
+      <c r="E97" s="15"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="14"/>
       <c r="B98" s="15"/>
       <c r="C98" s="15"/>
       <c r="D98" s="16"/>
+      <c r="E98" s="15"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="14"/>
       <c r="B99" s="15"/>
       <c r="C99" s="15"/>
       <c r="D99" s="16"/>
+      <c r="E99" s="15"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="14"/>
       <c r="B100" s="15"/>
       <c r="C100" s="15"/>
       <c r="D100" s="16"/>
+      <c r="E100" s="15"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="14"/>
       <c r="B101" s="15"/>
       <c r="C101" s="15"/>
       <c r="D101" s="16"/>
+      <c r="E101" s="15"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="14"/>
       <c r="B102" s="15"/>
       <c r="C102" s="15"/>
       <c r="D102" s="16"/>
+      <c r="E102" s="15"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="14"/>
       <c r="B103" s="15"/>
       <c r="C103" s="15"/>
       <c r="D103" s="16"/>
+      <c r="E103" s="15"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="14"/>
       <c r="B104" s="15"/>
       <c r="C104" s="15"/>
       <c r="D104" s="16"/>
+      <c r="E104" s="15"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="14"/>
       <c r="B105" s="15"/>
       <c r="C105" s="15"/>
       <c r="D105" s="16"/>
+      <c r="E105" s="15"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="14"/>
       <c r="B106" s="15"/>
       <c r="C106" s="15"/>
       <c r="D106" s="16"/>
+      <c r="E106" s="15"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="14"/>
       <c r="B107" s="15"/>
       <c r="C107" s="15"/>
       <c r="D107" s="16"/>
+      <c r="E107" s="15"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="14"/>
       <c r="B108" s="15"/>
       <c r="C108" s="15"/>
       <c r="D108" s="16"/>
+      <c r="E108" s="15"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="14"/>
       <c r="B109" s="15"/>
       <c r="C109" s="15"/>
       <c r="D109" s="16"/>
+      <c r="E109" s="15"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="14"/>
       <c r="B110" s="15"/>
       <c r="C110" s="15"/>
       <c r="D110" s="16"/>
+      <c r="E110" s="15"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="14"/>
       <c r="B111" s="15"/>
       <c r="C111" s="15"/>
       <c r="D111" s="16"/>
+      <c r="E111" s="15"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="14"/>
       <c r="B112" s="15"/>
       <c r="C112" s="15"/>
       <c r="D112" s="16"/>
+      <c r="E112" s="15"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="14"/>
       <c r="B113" s="15"/>
       <c r="C113" s="15"/>
       <c r="D113" s="16"/>
+      <c r="E113" s="15"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="14"/>
       <c r="B114" s="15"/>
       <c r="C114" s="15"/>
       <c r="D114" s="16"/>
+      <c r="E114" s="15"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="14"/>
       <c r="B115" s="15"/>
       <c r="C115" s="15"/>
       <c r="D115" s="16"/>
+      <c r="E115" s="15"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="14"/>
       <c r="B116" s="15"/>
       <c r="C116" s="15"/>
       <c r="D116" s="16"/>
+      <c r="E116" s="15"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="14"/>
       <c r="B117" s="15"/>
       <c r="C117" s="15"/>
       <c r="D117" s="16"/>
+      <c r="E117" s="15"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="14"/>
       <c r="B118" s="15"/>
       <c r="C118" s="15"/>
       <c r="D118" s="16"/>
+      <c r="E118" s="15"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="14"/>
       <c r="B119" s="15"/>
       <c r="C119" s="15"/>
       <c r="D119" s="16"/>
+      <c r="E119" s="15"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="14"/>
       <c r="B120" s="15"/>
       <c r="C120" s="15"/>
       <c r="D120" s="16"/>
+      <c r="E120" s="15"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="14"/>
       <c r="B121" s="15"/>
       <c r="C121" s="15"/>
       <c r="D121" s="16"/>
+      <c r="E121" s="15"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="14"/>
       <c r="B122" s="15"/>
       <c r="C122" s="15"/>
       <c r="D122" s="16"/>
+      <c r="E122" s="15"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="14"/>
       <c r="B123" s="15"/>
       <c r="C123" s="15"/>
       <c r="D123" s="16"/>
+      <c r="E123" s="15"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="14"/>
       <c r="B124" s="15"/>
       <c r="C124" s="15"/>
       <c r="D124" s="16"/>
+      <c r="E124" s="15"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="14"/>
       <c r="B125" s="15"/>
       <c r="C125" s="15"/>
       <c r="D125" s="16"/>
+      <c r="E125" s="15"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="14"/>
       <c r="B126" s="15"/>
       <c r="C126" s="15"/>
       <c r="D126" s="16"/>
+      <c r="E126" s="15"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="14"/>
       <c r="B127" s="15"/>
       <c r="C127" s="15"/>
       <c r="D127" s="16"/>
+      <c r="E127" s="15"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="14"/>
       <c r="B128" s="15"/>
       <c r="C128" s="15"/>
       <c r="D128" s="16"/>
+      <c r="E128" s="15"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="14"/>
       <c r="B129" s="15"/>
       <c r="C129" s="15"/>
       <c r="D129" s="16"/>
+      <c r="E129" s="15"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="14"/>
       <c r="B130" s="15"/>
       <c r="C130" s="15"/>
       <c r="D130" s="16"/>
+      <c r="E130" s="15"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="14"/>
       <c r="B131" s="15"/>
       <c r="C131" s="15"/>
       <c r="D131" s="16"/>
+      <c r="E131" s="15"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="14"/>
       <c r="B132" s="15"/>
       <c r="C132" s="15"/>
       <c r="D132" s="16"/>
+      <c r="E132" s="15"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="14"/>
       <c r="B133" s="15"/>
       <c r="C133" s="15"/>
       <c r="D133" s="16"/>
+      <c r="E133" s="15"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="14"/>
       <c r="B134" s="15"/>
       <c r="C134" s="15"/>
       <c r="D134" s="16"/>
+      <c r="E134" s="15"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="14"/>
       <c r="B135" s="15"/>
       <c r="C135" s="15"/>
       <c r="D135" s="16"/>
+      <c r="E135" s="15"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="14"/>
       <c r="B136" s="15"/>
       <c r="C136" s="15"/>
       <c r="D136" s="16"/>
+      <c r="E136" s="15"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="14"/>
       <c r="B137" s="15"/>
       <c r="C137" s="15"/>
       <c r="D137" s="16"/>
+      <c r="E137" s="15"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="14"/>
       <c r="B138" s="15"/>
       <c r="C138" s="15"/>
       <c r="D138" s="16"/>
+      <c r="E138" s="15"/>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="14"/>
       <c r="B139" s="15"/>
       <c r="C139" s="15"/>
       <c r="D139" s="16"/>
+      <c r="E139" s="15"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="14"/>
       <c r="B140" s="15"/>
       <c r="C140" s="15"/>
       <c r="D140" s="16"/>
+      <c r="E140" s="15"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="14"/>
       <c r="B141" s="15"/>
       <c r="C141" s="15"/>
       <c r="D141" s="16"/>
+      <c r="E141" s="15"/>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="14"/>
       <c r="B142" s="15"/>
       <c r="C142" s="15"/>
       <c r="D142" s="16"/>
+      <c r="E142" s="15"/>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="14"/>
       <c r="B143" s="15"/>
       <c r="C143" s="15"/>
       <c r="D143" s="16"/>
+      <c r="E143" s="15"/>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="14"/>
       <c r="B144" s="15"/>
       <c r="C144" s="15"/>
       <c r="D144" s="16"/>
+      <c r="E144" s="15"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="14"/>
       <c r="B145" s="15"/>
       <c r="C145" s="15"/>
       <c r="D145" s="16"/>
+      <c r="E145" s="15"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="14"/>
       <c r="B146" s="15"/>
       <c r="C146" s="15"/>
       <c r="D146" s="16"/>
+      <c r="E146" s="15"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="14"/>
       <c r="B147" s="15"/>
       <c r="C147" s="15"/>
       <c r="D147" s="16"/>
+      <c r="E147" s="15"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="14"/>
       <c r="B148" s="15"/>
       <c r="C148" s="15"/>
       <c r="D148" s="16"/>
+      <c r="E148" s="15"/>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="14"/>
       <c r="B149" s="15"/>
       <c r="C149" s="15"/>
       <c r="D149" s="16"/>
+      <c r="E149" s="15"/>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="14"/>
       <c r="B150" s="15"/>
       <c r="C150" s="15"/>
       <c r="D150" s="16"/>
+      <c r="E150" s="15"/>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="14"/>
       <c r="B151" s="15"/>
       <c r="C151" s="15"/>
       <c r="D151" s="16"/>
+      <c r="E151" s="15"/>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="14"/>
       <c r="B152" s="15"/>
       <c r="C152" s="15"/>
       <c r="D152" s="16"/>
+      <c r="E152" s="15"/>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="14"/>
       <c r="B153" s="15"/>
       <c r="C153" s="15"/>
       <c r="D153" s="16"/>
+      <c r="E153" s="15"/>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="14"/>
       <c r="B154" s="15"/>
       <c r="C154" s="15"/>
       <c r="D154" s="16"/>
+      <c r="E154" s="15"/>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="14"/>
       <c r="B155" s="15"/>
       <c r="C155" s="15"/>
       <c r="D155" s="16"/>
+      <c r="E155" s="15"/>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="14"/>
       <c r="B156" s="15"/>
       <c r="C156" s="15"/>
       <c r="D156" s="16"/>
+      <c r="E156" s="15"/>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="14"/>
       <c r="B157" s="15"/>
       <c r="C157" s="15"/>
       <c r="D157" s="16"/>
+      <c r="E157" s="15"/>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="14"/>
       <c r="B158" s="15"/>
       <c r="C158" s="15"/>
       <c r="D158" s="16"/>
+      <c r="E158" s="15"/>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="14"/>
       <c r="B159" s="15"/>
       <c r="C159" s="15"/>
       <c r="D159" s="16"/>
+      <c r="E159" s="15"/>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="14"/>
       <c r="B160" s="15"/>
       <c r="C160" s="15"/>
       <c r="D160" s="16"/>
+      <c r="E160" s="15"/>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="14"/>
       <c r="B161" s="15"/>
       <c r="C161" s="15"/>
       <c r="D161" s="16"/>
+      <c r="E161" s="15"/>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="14"/>
       <c r="B162" s="15"/>
       <c r="C162" s="15"/>
       <c r="D162" s="16"/>
+      <c r="E162" s="15"/>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="14"/>
       <c r="B163" s="15"/>
       <c r="C163" s="15"/>
       <c r="D163" s="16"/>
+      <c r="E163" s="15"/>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="14"/>
       <c r="B164" s="15"/>
       <c r="C164" s="15"/>
       <c r="D164" s="16"/>
+      <c r="E164" s="15"/>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="14"/>
       <c r="B165" s="15"/>
       <c r="C165" s="15"/>
       <c r="D165" s="16"/>
+      <c r="E165" s="15"/>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="14"/>
       <c r="B166" s="15"/>
       <c r="C166" s="15"/>
       <c r="D166" s="16"/>
+      <c r="E166" s="15"/>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="14"/>
       <c r="B167" s="15"/>
       <c r="C167" s="15"/>
       <c r="D167" s="16"/>
+      <c r="E167" s="15"/>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="14"/>
       <c r="B168" s="15"/>
       <c r="C168" s="15"/>
       <c r="D168" s="16"/>
+      <c r="E168" s="15"/>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="14"/>
       <c r="B169" s="15"/>
       <c r="C169" s="15"/>
       <c r="D169" s="16"/>
+      <c r="E169" s="15"/>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="14"/>
       <c r="B170" s="15"/>
       <c r="C170" s="15"/>
       <c r="D170" s="16"/>
+      <c r="E170" s="15"/>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="14"/>
       <c r="B171" s="15"/>
       <c r="C171" s="15"/>
       <c r="D171" s="16"/>
+      <c r="E171" s="15"/>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="14"/>
       <c r="B172" s="15"/>
       <c r="C172" s="15"/>
       <c r="D172" s="16"/>
+      <c r="E172" s="15"/>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="14"/>
       <c r="B173" s="15"/>
       <c r="C173" s="15"/>
       <c r="D173" s="16"/>
+      <c r="E173" s="15"/>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="14"/>
       <c r="B174" s="15"/>
       <c r="C174" s="15"/>
       <c r="D174" s="16"/>
+      <c r="E174" s="15"/>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="14"/>
       <c r="B175" s="15"/>
       <c r="C175" s="15"/>
       <c r="D175" s="16"/>
+      <c r="E175" s="15"/>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="14"/>
       <c r="B176" s="15"/>
       <c r="C176" s="15"/>
       <c r="D176" s="16"/>
+      <c r="E176" s="15"/>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="14"/>
       <c r="B177" s="15"/>
       <c r="C177" s="15"/>
       <c r="D177" s="16"/>
+      <c r="E177" s="15"/>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="14"/>
       <c r="B178" s="15"/>
       <c r="C178" s="15"/>
       <c r="D178" s="16"/>
+      <c r="E178" s="15"/>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="14"/>
       <c r="B179" s="15"/>
       <c r="C179" s="15"/>
       <c r="D179" s="16"/>
+      <c r="E179" s="15"/>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="14"/>
       <c r="B180" s="15"/>
       <c r="C180" s="15"/>
       <c r="D180" s="16"/>
+      <c r="E180" s="15"/>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="14"/>
       <c r="B181" s="15"/>
       <c r="C181" s="15"/>
       <c r="D181" s="16"/>
+      <c r="E181" s="15"/>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="14"/>
       <c r="B182" s="15"/>
       <c r="C182" s="15"/>
       <c r="D182" s="16"/>
+      <c r="E182" s="15"/>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="14"/>
       <c r="B183" s="15"/>
       <c r="C183" s="15"/>
       <c r="D183" s="16"/>
+      <c r="E183" s="15"/>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="14"/>
       <c r="B184" s="15"/>
       <c r="C184" s="15"/>
       <c r="D184" s="16"/>
+      <c r="E184" s="15"/>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="14"/>
       <c r="B185" s="15"/>
       <c r="C185" s="15"/>
       <c r="D185" s="16"/>
+      <c r="E185" s="15"/>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="14"/>
       <c r="B186" s="15"/>
       <c r="C186" s="15"/>
       <c r="D186" s="16"/>
+      <c r="E186" s="15"/>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="14"/>
       <c r="B187" s="15"/>
       <c r="C187" s="15"/>
       <c r="D187" s="16"/>
+      <c r="E187" s="15"/>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="14"/>
       <c r="B188" s="15"/>
       <c r="C188" s="15"/>
       <c r="D188" s="16"/>
+      <c r="E188" s="15"/>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="14"/>
       <c r="B189" s="15"/>
       <c r="C189" s="15"/>
       <c r="D189" s="16"/>
+      <c r="E189" s="15"/>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="14"/>
       <c r="B190" s="15"/>
       <c r="C190" s="15"/>
       <c r="D190" s="16"/>
+      <c r="E190" s="15"/>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="14"/>
       <c r="B191" s="15"/>
       <c r="C191" s="15"/>
       <c r="D191" s="16"/>
+      <c r="E191" s="15"/>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="14"/>
       <c r="B192" s="15"/>
       <c r="C192" s="15"/>
       <c r="D192" s="16"/>
+      <c r="E192" s="15"/>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="14"/>
       <c r="B193" s="15"/>
       <c r="C193" s="15"/>
       <c r="D193" s="16"/>
+      <c r="E193" s="15"/>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="14"/>
       <c r="B194" s="15"/>
       <c r="C194" s="15"/>
       <c r="D194" s="16"/>
+      <c r="E194" s="15"/>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="14"/>
       <c r="B195" s="15"/>
       <c r="C195" s="15"/>
       <c r="D195" s="16"/>
+      <c r="E195" s="15"/>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="14"/>
       <c r="B196" s="15"/>
       <c r="C196" s="15"/>
       <c r="D196" s="16"/>
+      <c r="E196" s="15"/>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="14"/>
       <c r="B197" s="15"/>
       <c r="C197" s="15"/>
       <c r="D197" s="16"/>
+      <c r="E197" s="15"/>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="14"/>
       <c r="B198" s="15"/>
       <c r="C198" s="15"/>
       <c r="D198" s="16"/>
+      <c r="E198" s="15"/>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="14"/>
       <c r="B199" s="15"/>
       <c r="C199" s="15"/>
       <c r="D199" s="16"/>
+      <c r="E199" s="15"/>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="14"/>
       <c r="B200" s="15"/>
       <c r="C200" s="15"/>
       <c r="D200" s="16"/>
+      <c r="E200" s="15"/>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="14"/>
       <c r="B201" s="15"/>
       <c r="C201" s="15"/>
       <c r="D201" s="16"/>
+      <c r="E201" s="15"/>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="14"/>
       <c r="B202" s="15"/>
       <c r="C202" s="15"/>
       <c r="D202" s="16"/>
+      <c r="E202" s="15"/>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="14"/>
       <c r="B203" s="15"/>
       <c r="C203" s="15"/>
       <c r="D203" s="16"/>
+      <c r="E203" s="15"/>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="14"/>
       <c r="B204" s="15"/>
       <c r="C204" s="15"/>
       <c r="D204" s="16"/>
+      <c r="E204" s="15"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation allowBlank="true" error="Elegí un componente de la lista." errorStyle="stop" errorTitle="Componente inválido" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B5:B204" type="list">
       <formula1>"Agus C.,Agus M.,Boli,Cami,Flopa,Katy,Luci,Mai,María,Marti,Paz,Vicky"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E204" type="list">
+      <formula1>"Sí,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -2144,32 +2389,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="H4" s="17" t="n">
         <f aca="false">SUM(D5:D204)</f>
@@ -2181,10 +2426,10 @@
         <v>46315</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D5" s="18" t="n">
         <v>3</v>
@@ -2194,7 +2439,7 @@
         <v>1470</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="H5" s="13" t="n">
         <f aca="false">SUM(E5:E204)</f>
@@ -2211,7 +2456,7 @@
         <v/>
       </c>
       <c r="G6" s="12" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H6" s="20" t="n">
         <v>490</v>
@@ -4237,27 +4482,27 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="F4" s="21" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4268,7 +4513,7 @@
         <v>8</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>12000</v>
@@ -4364,12 +4609,12 @@
       <c r="B12" s="15"/>
       <c r="C12" s="15"/>
       <c r="D12" s="16"/>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G12" s="23" t="n">
-        <f aca="false">SUM(G5:G11)</f>
-        <v>12000</v>
+      <c r="G12" s="22" t="n">
+        <f aca="false">SUMIF($B$5:$B$204,F12,$D$5:$D$204)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4377,6 +4622,13 @@
       <c r="B13" s="15"/>
       <c r="C13" s="15"/>
       <c r="D13" s="16"/>
+      <c r="F13" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="23" t="n">
+        <f aca="false">SUM(G5:G12)</f>
+        <v>12000</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14"/>
@@ -5527,7 +5779,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation allowBlank="true" error="Elegí una categoría de la lista." errorStyle="stop" errorTitle="Categoría inválida" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B5:B204" type="list">
-      <formula1>"Maquillaje,Luces,Escenografía,Utilería,Vestuario,Audio,Comida"</formula1>
+      <formula1>"Maquillaje,Luces,Escenografía,Utilería,Vestuario,Audio,Comida,Extra"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Lo pendiente de la rifa no suma al saldo; firma de Luci
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014cQS814DmisHJYTJthjhHq
</commit_message>
<xml_diff>
--- a/Finanzas_Proyecto.xlsx
+++ b/Finanzas_Proyecto.xlsx
@@ -34,7 +34,7 @@
     <t xml:space="preserve">INGRESOS</t>
   </si>
   <si>
-    <t xml:space="preserve">Rifa del peso</t>
+    <t xml:space="preserve">Rifa del peso (solo pagado)</t>
   </si>
   <si>
     <t xml:space="preserve">Remeras (recaudo)</t>
@@ -730,7 +730,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="5" t="n">
-        <f aca="false">'Rifa del Peso'!H4</f>
+        <f aca="false">'Rifa del Peso'!H5</f>
         <v>25000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Pagado también en remeras: lo pendiente no suma al saldo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014cQS814DmisHJYTJthjhHq
</commit_message>
<xml_diff>
--- a/Finanzas_Proyecto.xlsx
+++ b/Finanzas_Proyecto.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="46">
   <si>
     <t xml:space="preserve">FINANZAS DEL PROYECTO</t>
   </si>
@@ -37,7 +37,7 @@
     <t xml:space="preserve">Rifa del peso (solo pagado)</t>
   </si>
   <si>
-    <t xml:space="preserve">Remeras (recaudo)</t>
+    <t xml:space="preserve">Remeras (solo pagado)</t>
   </si>
   <si>
     <t xml:space="preserve">Remeras vendidas (unidades)</t>
@@ -121,10 +121,10 @@
     <t xml:space="preserve">VENTA DE REMERAS</t>
   </si>
   <si>
-    <t xml:space="preserve">Celdas rosas = para completar. Una fila por venta; elegí el componente y poné las unidades. El recaudo se calcula solo con el precio por unidad. La fila 5 es un ejemplo: reemplazala.</t>
+    <t xml:space="preserve">Celdas rosas = para completar. Una fila por venta; elegí el componente y poné las unidades. El recaudo se calcula solo con el precio por unidad. Marcá Sí en Pagado cuando esté cobrado. La fila 5 es un ejemplo: reemplazala.</t>
   </si>
   <si>
-    <t xml:space="preserve">Detalle (talle, comprador, etc.)</t>
+    <t xml:space="preserve">Detalle (talle, compradora, etc.)</t>
   </si>
   <si>
     <t xml:space="preserve">Cantidad (unidades)</t>
@@ -739,7 +739,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="5" t="n">
-        <f aca="false">Remeras!H5</f>
+        <f aca="false">Remeras!I6</f>
         <v>1470</v>
       </c>
     </row>
@@ -748,7 +748,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="6" t="n">
-        <f aca="false">Remeras!H4</f>
+        <f aca="false">Remeras!I4</f>
         <v>3</v>
       </c>
     </row>
@@ -2375,7 +2375,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H204"/>
+  <dimension ref="A1:I204"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -2383,8 +2383,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2413,10 +2414,13 @@
       <c r="E4" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="F4" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="H4" s="17" t="n">
+      <c r="I4" s="17" t="n">
         <f aca="false">SUM(D5:D204)</f>
         <v>3</v>
       </c>
@@ -2435,13 +2439,16 @@
         <v>3</v>
       </c>
       <c r="E5" s="19" t="n">
-        <f aca="false">IF(D5="","",D5*$H$6)</f>
+        <f aca="false">IF(D5="","",D5*$I$8)</f>
         <v>1470</v>
       </c>
-      <c r="G5" s="12" t="s">
+      <c r="F5" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="H5" s="13" t="n">
+      <c r="I5" s="13" t="n">
         <f aca="false">SUM(E5:E204)</f>
         <v>1470</v>
       </c>
@@ -2452,14 +2459,16 @@
       <c r="C6" s="15"/>
       <c r="D6" s="18"/>
       <c r="E6" s="19" t="str">
-        <f aca="false">IF(D6="","",D6*$H$6)</f>
-        <v/>
-      </c>
-      <c r="G6" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" s="20" t="n">
-        <v>490</v>
+        <f aca="false">IF(D6="","",D6*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F6" s="15"/>
+      <c r="H6" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="I6" s="13" t="n">
+        <f aca="false">SUMIF(F5:F204,"Sí",E5:E204)</f>
+        <v>1470</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2468,8 +2477,16 @@
       <c r="C7" s="15"/>
       <c r="D7" s="18"/>
       <c r="E7" s="19" t="str">
-        <f aca="false">IF(D7="","",D7*$H$6)</f>
-        <v/>
+        <f aca="false">IF(D7="","",D7*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F7" s="15"/>
+      <c r="H7" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="I7" s="13" t="n">
+        <f aca="false">I5-I6</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2478,8 +2495,15 @@
       <c r="C8" s="15"/>
       <c r="D8" s="18"/>
       <c r="E8" s="19" t="str">
-        <f aca="false">IF(D8="","",D8*$H$6)</f>
-        <v/>
+        <f aca="false">IF(D8="","",D8*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="15"/>
+      <c r="H8" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="I8" s="20" t="n">
+        <v>490</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2488,9 +2512,10 @@
       <c r="C9" s="15"/>
       <c r="D9" s="18"/>
       <c r="E9" s="19" t="str">
-        <f aca="false">IF(D9="","",D9*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D9="","",D9*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="15"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14"/>
@@ -2498,9 +2523,10 @@
       <c r="C10" s="15"/>
       <c r="D10" s="18"/>
       <c r="E10" s="19" t="str">
-        <f aca="false">IF(D10="","",D10*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D10="","",D10*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14"/>
@@ -2508,9 +2534,10 @@
       <c r="C11" s="15"/>
       <c r="D11" s="18"/>
       <c r="E11" s="19" t="str">
-        <f aca="false">IF(D11="","",D11*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D11="","",D11*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F11" s="15"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14"/>
@@ -2518,9 +2545,10 @@
       <c r="C12" s="15"/>
       <c r="D12" s="18"/>
       <c r="E12" s="19" t="str">
-        <f aca="false">IF(D12="","",D12*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D12="","",D12*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14"/>
@@ -2528,9 +2556,10 @@
       <c r="C13" s="15"/>
       <c r="D13" s="18"/>
       <c r="E13" s="19" t="str">
-        <f aca="false">IF(D13="","",D13*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D13="","",D13*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F13" s="15"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14"/>
@@ -2538,9 +2567,10 @@
       <c r="C14" s="15"/>
       <c r="D14" s="18"/>
       <c r="E14" s="19" t="str">
-        <f aca="false">IF(D14="","",D14*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D14="","",D14*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F14" s="15"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14"/>
@@ -2548,9 +2578,10 @@
       <c r="C15" s="15"/>
       <c r="D15" s="18"/>
       <c r="E15" s="19" t="str">
-        <f aca="false">IF(D15="","",D15*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D15="","",D15*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F15" s="15"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14"/>
@@ -2558,9 +2589,10 @@
       <c r="C16" s="15"/>
       <c r="D16" s="18"/>
       <c r="E16" s="19" t="str">
-        <f aca="false">IF(D16="","",D16*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D16="","",D16*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F16" s="15"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14"/>
@@ -2568,9 +2600,10 @@
       <c r="C17" s="15"/>
       <c r="D17" s="18"/>
       <c r="E17" s="19" t="str">
-        <f aca="false">IF(D17="","",D17*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D17="","",D17*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F17" s="15"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14"/>
@@ -2578,9 +2611,10 @@
       <c r="C18" s="15"/>
       <c r="D18" s="18"/>
       <c r="E18" s="19" t="str">
-        <f aca="false">IF(D18="","",D18*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D18="","",D18*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F18" s="15"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14"/>
@@ -2588,9 +2622,10 @@
       <c r="C19" s="15"/>
       <c r="D19" s="18"/>
       <c r="E19" s="19" t="str">
-        <f aca="false">IF(D19="","",D19*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D19="","",D19*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F19" s="15"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14"/>
@@ -2598,9 +2633,10 @@
       <c r="C20" s="15"/>
       <c r="D20" s="18"/>
       <c r="E20" s="19" t="str">
-        <f aca="false">IF(D20="","",D20*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D20="","",D20*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F20" s="15"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14"/>
@@ -2608,9 +2644,10 @@
       <c r="C21" s="15"/>
       <c r="D21" s="18"/>
       <c r="E21" s="19" t="str">
-        <f aca="false">IF(D21="","",D21*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D21="","",D21*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F21" s="15"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14"/>
@@ -2618,9 +2655,10 @@
       <c r="C22" s="15"/>
       <c r="D22" s="18"/>
       <c r="E22" s="19" t="str">
-        <f aca="false">IF(D22="","",D22*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D22="","",D22*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F22" s="15"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="14"/>
@@ -2628,9 +2666,10 @@
       <c r="C23" s="15"/>
       <c r="D23" s="18"/>
       <c r="E23" s="19" t="str">
-        <f aca="false">IF(D23="","",D23*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D23="","",D23*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F23" s="15"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14"/>
@@ -2638,9 +2677,10 @@
       <c r="C24" s="15"/>
       <c r="D24" s="18"/>
       <c r="E24" s="19" t="str">
-        <f aca="false">IF(D24="","",D24*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D24="","",D24*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F24" s="15"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14"/>
@@ -2648,9 +2688,10 @@
       <c r="C25" s="15"/>
       <c r="D25" s="18"/>
       <c r="E25" s="19" t="str">
-        <f aca="false">IF(D25="","",D25*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D25="","",D25*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F25" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14"/>
@@ -2658,9 +2699,10 @@
       <c r="C26" s="15"/>
       <c r="D26" s="18"/>
       <c r="E26" s="19" t="str">
-        <f aca="false">IF(D26="","",D26*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D26="","",D26*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F26" s="15"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14"/>
@@ -2668,9 +2710,10 @@
       <c r="C27" s="15"/>
       <c r="D27" s="18"/>
       <c r="E27" s="19" t="str">
-        <f aca="false">IF(D27="","",D27*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D27="","",D27*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F27" s="15"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14"/>
@@ -2678,9 +2721,10 @@
       <c r="C28" s="15"/>
       <c r="D28" s="18"/>
       <c r="E28" s="19" t="str">
-        <f aca="false">IF(D28="","",D28*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D28="","",D28*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F28" s="15"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14"/>
@@ -2688,9 +2732,10 @@
       <c r="C29" s="15"/>
       <c r="D29" s="18"/>
       <c r="E29" s="19" t="str">
-        <f aca="false">IF(D29="","",D29*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D29="","",D29*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F29" s="15"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14"/>
@@ -2698,9 +2743,10 @@
       <c r="C30" s="15"/>
       <c r="D30" s="18"/>
       <c r="E30" s="19" t="str">
-        <f aca="false">IF(D30="","",D30*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D30="","",D30*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F30" s="15"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14"/>
@@ -2708,9 +2754,10 @@
       <c r="C31" s="15"/>
       <c r="D31" s="18"/>
       <c r="E31" s="19" t="str">
-        <f aca="false">IF(D31="","",D31*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D31="","",D31*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F31" s="15"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14"/>
@@ -2718,9 +2765,10 @@
       <c r="C32" s="15"/>
       <c r="D32" s="18"/>
       <c r="E32" s="19" t="str">
-        <f aca="false">IF(D32="","",D32*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D32="","",D32*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14"/>
@@ -2728,9 +2776,10 @@
       <c r="C33" s="15"/>
       <c r="D33" s="18"/>
       <c r="E33" s="19" t="str">
-        <f aca="false">IF(D33="","",D33*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D33="","",D33*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14"/>
@@ -2738,9 +2787,10 @@
       <c r="C34" s="15"/>
       <c r="D34" s="18"/>
       <c r="E34" s="19" t="str">
-        <f aca="false">IF(D34="","",D34*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D34="","",D34*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="14"/>
@@ -2748,9 +2798,10 @@
       <c r="C35" s="15"/>
       <c r="D35" s="18"/>
       <c r="E35" s="19" t="str">
-        <f aca="false">IF(D35="","",D35*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D35="","",D35*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F35" s="15"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="14"/>
@@ -2758,9 +2809,10 @@
       <c r="C36" s="15"/>
       <c r="D36" s="18"/>
       <c r="E36" s="19" t="str">
-        <f aca="false">IF(D36="","",D36*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D36="","",D36*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F36" s="15"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14"/>
@@ -2768,9 +2820,10 @@
       <c r="C37" s="15"/>
       <c r="D37" s="18"/>
       <c r="E37" s="19" t="str">
-        <f aca="false">IF(D37="","",D37*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D37="","",D37*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F37" s="15"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14"/>
@@ -2778,9 +2831,10 @@
       <c r="C38" s="15"/>
       <c r="D38" s="18"/>
       <c r="E38" s="19" t="str">
-        <f aca="false">IF(D38="","",D38*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D38="","",D38*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F38" s="15"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="14"/>
@@ -2788,9 +2842,10 @@
       <c r="C39" s="15"/>
       <c r="D39" s="18"/>
       <c r="E39" s="19" t="str">
-        <f aca="false">IF(D39="","",D39*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D39="","",D39*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F39" s="15"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="14"/>
@@ -2798,9 +2853,10 @@
       <c r="C40" s="15"/>
       <c r="D40" s="18"/>
       <c r="E40" s="19" t="str">
-        <f aca="false">IF(D40="","",D40*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D40="","",D40*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F40" s="15"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="14"/>
@@ -2808,9 +2864,10 @@
       <c r="C41" s="15"/>
       <c r="D41" s="18"/>
       <c r="E41" s="19" t="str">
-        <f aca="false">IF(D41="","",D41*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D41="","",D41*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F41" s="15"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14"/>
@@ -2818,9 +2875,10 @@
       <c r="C42" s="15"/>
       <c r="D42" s="18"/>
       <c r="E42" s="19" t="str">
-        <f aca="false">IF(D42="","",D42*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D42="","",D42*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F42" s="15"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="14"/>
@@ -2828,9 +2886,10 @@
       <c r="C43" s="15"/>
       <c r="D43" s="18"/>
       <c r="E43" s="19" t="str">
-        <f aca="false">IF(D43="","",D43*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D43="","",D43*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F43" s="15"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="14"/>
@@ -2838,9 +2897,10 @@
       <c r="C44" s="15"/>
       <c r="D44" s="18"/>
       <c r="E44" s="19" t="str">
-        <f aca="false">IF(D44="","",D44*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D44="","",D44*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F44" s="15"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="14"/>
@@ -2848,9 +2908,10 @@
       <c r="C45" s="15"/>
       <c r="D45" s="18"/>
       <c r="E45" s="19" t="str">
-        <f aca="false">IF(D45="","",D45*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D45="","",D45*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F45" s="15"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="14"/>
@@ -2858,9 +2919,10 @@
       <c r="C46" s="15"/>
       <c r="D46" s="18"/>
       <c r="E46" s="19" t="str">
-        <f aca="false">IF(D46="","",D46*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D46="","",D46*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F46" s="15"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="14"/>
@@ -2868,9 +2930,10 @@
       <c r="C47" s="15"/>
       <c r="D47" s="18"/>
       <c r="E47" s="19" t="str">
-        <f aca="false">IF(D47="","",D47*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D47="","",D47*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F47" s="15"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="14"/>
@@ -2878,9 +2941,10 @@
       <c r="C48" s="15"/>
       <c r="D48" s="18"/>
       <c r="E48" s="19" t="str">
-        <f aca="false">IF(D48="","",D48*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D48="","",D48*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F48" s="15"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="14"/>
@@ -2888,9 +2952,10 @@
       <c r="C49" s="15"/>
       <c r="D49" s="18"/>
       <c r="E49" s="19" t="str">
-        <f aca="false">IF(D49="","",D49*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D49="","",D49*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F49" s="15"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="14"/>
@@ -2898,9 +2963,10 @@
       <c r="C50" s="15"/>
       <c r="D50" s="18"/>
       <c r="E50" s="19" t="str">
-        <f aca="false">IF(D50="","",D50*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D50="","",D50*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F50" s="15"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="14"/>
@@ -2908,9 +2974,10 @@
       <c r="C51" s="15"/>
       <c r="D51" s="18"/>
       <c r="E51" s="19" t="str">
-        <f aca="false">IF(D51="","",D51*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D51="","",D51*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F51" s="15"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="14"/>
@@ -2918,9 +2985,10 @@
       <c r="C52" s="15"/>
       <c r="D52" s="18"/>
       <c r="E52" s="19" t="str">
-        <f aca="false">IF(D52="","",D52*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D52="","",D52*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F52" s="15"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="14"/>
@@ -2928,9 +2996,10 @@
       <c r="C53" s="15"/>
       <c r="D53" s="18"/>
       <c r="E53" s="19" t="str">
-        <f aca="false">IF(D53="","",D53*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D53="","",D53*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F53" s="15"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="14"/>
@@ -2938,9 +3007,10 @@
       <c r="C54" s="15"/>
       <c r="D54" s="18"/>
       <c r="E54" s="19" t="str">
-        <f aca="false">IF(D54="","",D54*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D54="","",D54*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F54" s="15"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="14"/>
@@ -2948,9 +3018,10 @@
       <c r="C55" s="15"/>
       <c r="D55" s="18"/>
       <c r="E55" s="19" t="str">
-        <f aca="false">IF(D55="","",D55*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D55="","",D55*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F55" s="15"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="14"/>
@@ -2958,9 +3029,10 @@
       <c r="C56" s="15"/>
       <c r="D56" s="18"/>
       <c r="E56" s="19" t="str">
-        <f aca="false">IF(D56="","",D56*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D56="","",D56*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F56" s="15"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="14"/>
@@ -2968,9 +3040,10 @@
       <c r="C57" s="15"/>
       <c r="D57" s="18"/>
       <c r="E57" s="19" t="str">
-        <f aca="false">IF(D57="","",D57*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D57="","",D57*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F57" s="15"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="14"/>
@@ -2978,9 +3051,10 @@
       <c r="C58" s="15"/>
       <c r="D58" s="18"/>
       <c r="E58" s="19" t="str">
-        <f aca="false">IF(D58="","",D58*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D58="","",D58*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F58" s="15"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="14"/>
@@ -2988,9 +3062,10 @@
       <c r="C59" s="15"/>
       <c r="D59" s="18"/>
       <c r="E59" s="19" t="str">
-        <f aca="false">IF(D59="","",D59*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D59="","",D59*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F59" s="15"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="14"/>
@@ -2998,9 +3073,10 @@
       <c r="C60" s="15"/>
       <c r="D60" s="18"/>
       <c r="E60" s="19" t="str">
-        <f aca="false">IF(D60="","",D60*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D60="","",D60*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F60" s="15"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="14"/>
@@ -3008,9 +3084,10 @@
       <c r="C61" s="15"/>
       <c r="D61" s="18"/>
       <c r="E61" s="19" t="str">
-        <f aca="false">IF(D61="","",D61*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D61="","",D61*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F61" s="15"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="14"/>
@@ -3018,9 +3095,10 @@
       <c r="C62" s="15"/>
       <c r="D62" s="18"/>
       <c r="E62" s="19" t="str">
-        <f aca="false">IF(D62="","",D62*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D62="","",D62*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F62" s="15"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="14"/>
@@ -3028,9 +3106,10 @@
       <c r="C63" s="15"/>
       <c r="D63" s="18"/>
       <c r="E63" s="19" t="str">
-        <f aca="false">IF(D63="","",D63*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D63="","",D63*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F63" s="15"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="14"/>
@@ -3038,9 +3117,10 @@
       <c r="C64" s="15"/>
       <c r="D64" s="18"/>
       <c r="E64" s="19" t="str">
-        <f aca="false">IF(D64="","",D64*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D64="","",D64*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F64" s="15"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="14"/>
@@ -3048,9 +3128,10 @@
       <c r="C65" s="15"/>
       <c r="D65" s="18"/>
       <c r="E65" s="19" t="str">
-        <f aca="false">IF(D65="","",D65*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D65="","",D65*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F65" s="15"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="14"/>
@@ -3058,9 +3139,10 @@
       <c r="C66" s="15"/>
       <c r="D66" s="18"/>
       <c r="E66" s="19" t="str">
-        <f aca="false">IF(D66="","",D66*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D66="","",D66*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F66" s="15"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="14"/>
@@ -3068,9 +3150,10 @@
       <c r="C67" s="15"/>
       <c r="D67" s="18"/>
       <c r="E67" s="19" t="str">
-        <f aca="false">IF(D67="","",D67*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D67="","",D67*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F67" s="15"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="14"/>
@@ -3078,9 +3161,10 @@
       <c r="C68" s="15"/>
       <c r="D68" s="18"/>
       <c r="E68" s="19" t="str">
-        <f aca="false">IF(D68="","",D68*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D68="","",D68*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F68" s="15"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="14"/>
@@ -3088,9 +3172,10 @@
       <c r="C69" s="15"/>
       <c r="D69" s="18"/>
       <c r="E69" s="19" t="str">
-        <f aca="false">IF(D69="","",D69*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D69="","",D69*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F69" s="15"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="14"/>
@@ -3098,9 +3183,10 @@
       <c r="C70" s="15"/>
       <c r="D70" s="18"/>
       <c r="E70" s="19" t="str">
-        <f aca="false">IF(D70="","",D70*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D70="","",D70*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F70" s="15"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="14"/>
@@ -3108,9 +3194,10 @@
       <c r="C71" s="15"/>
       <c r="D71" s="18"/>
       <c r="E71" s="19" t="str">
-        <f aca="false">IF(D71="","",D71*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D71="","",D71*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F71" s="15"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="14"/>
@@ -3118,9 +3205,10 @@
       <c r="C72" s="15"/>
       <c r="D72" s="18"/>
       <c r="E72" s="19" t="str">
-        <f aca="false">IF(D72="","",D72*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D72="","",D72*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F72" s="15"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="14"/>
@@ -3128,9 +3216,10 @@
       <c r="C73" s="15"/>
       <c r="D73" s="18"/>
       <c r="E73" s="19" t="str">
-        <f aca="false">IF(D73="","",D73*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D73="","",D73*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F73" s="15"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="14"/>
@@ -3138,9 +3227,10 @@
       <c r="C74" s="15"/>
       <c r="D74" s="18"/>
       <c r="E74" s="19" t="str">
-        <f aca="false">IF(D74="","",D74*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D74="","",D74*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F74" s="15"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="14"/>
@@ -3148,9 +3238,10 @@
       <c r="C75" s="15"/>
       <c r="D75" s="18"/>
       <c r="E75" s="19" t="str">
-        <f aca="false">IF(D75="","",D75*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D75="","",D75*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F75" s="15"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="14"/>
@@ -3158,9 +3249,10 @@
       <c r="C76" s="15"/>
       <c r="D76" s="18"/>
       <c r="E76" s="19" t="str">
-        <f aca="false">IF(D76="","",D76*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D76="","",D76*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F76" s="15"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="14"/>
@@ -3168,9 +3260,10 @@
       <c r="C77" s="15"/>
       <c r="D77" s="18"/>
       <c r="E77" s="19" t="str">
-        <f aca="false">IF(D77="","",D77*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D77="","",D77*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F77" s="15"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="14"/>
@@ -3178,9 +3271,10 @@
       <c r="C78" s="15"/>
       <c r="D78" s="18"/>
       <c r="E78" s="19" t="str">
-        <f aca="false">IF(D78="","",D78*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D78="","",D78*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F78" s="15"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="14"/>
@@ -3188,9 +3282,10 @@
       <c r="C79" s="15"/>
       <c r="D79" s="18"/>
       <c r="E79" s="19" t="str">
-        <f aca="false">IF(D79="","",D79*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D79="","",D79*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F79" s="15"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="14"/>
@@ -3198,9 +3293,10 @@
       <c r="C80" s="15"/>
       <c r="D80" s="18"/>
       <c r="E80" s="19" t="str">
-        <f aca="false">IF(D80="","",D80*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D80="","",D80*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F80" s="15"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="14"/>
@@ -3208,9 +3304,10 @@
       <c r="C81" s="15"/>
       <c r="D81" s="18"/>
       <c r="E81" s="19" t="str">
-        <f aca="false">IF(D81="","",D81*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D81="","",D81*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F81" s="15"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="14"/>
@@ -3218,9 +3315,10 @@
       <c r="C82" s="15"/>
       <c r="D82" s="18"/>
       <c r="E82" s="19" t="str">
-        <f aca="false">IF(D82="","",D82*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D82="","",D82*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F82" s="15"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="14"/>
@@ -3228,9 +3326,10 @@
       <c r="C83" s="15"/>
       <c r="D83" s="18"/>
       <c r="E83" s="19" t="str">
-        <f aca="false">IF(D83="","",D83*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D83="","",D83*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F83" s="15"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="14"/>
@@ -3238,9 +3337,10 @@
       <c r="C84" s="15"/>
       <c r="D84" s="18"/>
       <c r="E84" s="19" t="str">
-        <f aca="false">IF(D84="","",D84*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D84="","",D84*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F84" s="15"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="14"/>
@@ -3248,9 +3348,10 @@
       <c r="C85" s="15"/>
       <c r="D85" s="18"/>
       <c r="E85" s="19" t="str">
-        <f aca="false">IF(D85="","",D85*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D85="","",D85*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F85" s="15"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="14"/>
@@ -3258,9 +3359,10 @@
       <c r="C86" s="15"/>
       <c r="D86" s="18"/>
       <c r="E86" s="19" t="str">
-        <f aca="false">IF(D86="","",D86*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D86="","",D86*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F86" s="15"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="14"/>
@@ -3268,9 +3370,10 @@
       <c r="C87" s="15"/>
       <c r="D87" s="18"/>
       <c r="E87" s="19" t="str">
-        <f aca="false">IF(D87="","",D87*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D87="","",D87*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F87" s="15"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="14"/>
@@ -3278,9 +3381,10 @@
       <c r="C88" s="15"/>
       <c r="D88" s="18"/>
       <c r="E88" s="19" t="str">
-        <f aca="false">IF(D88="","",D88*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D88="","",D88*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F88" s="15"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="14"/>
@@ -3288,9 +3392,10 @@
       <c r="C89" s="15"/>
       <c r="D89" s="18"/>
       <c r="E89" s="19" t="str">
-        <f aca="false">IF(D89="","",D89*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D89="","",D89*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F89" s="15"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="14"/>
@@ -3298,9 +3403,10 @@
       <c r="C90" s="15"/>
       <c r="D90" s="18"/>
       <c r="E90" s="19" t="str">
-        <f aca="false">IF(D90="","",D90*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D90="","",D90*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F90" s="15"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="14"/>
@@ -3308,9 +3414,10 @@
       <c r="C91" s="15"/>
       <c r="D91" s="18"/>
       <c r="E91" s="19" t="str">
-        <f aca="false">IF(D91="","",D91*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D91="","",D91*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F91" s="15"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="14"/>
@@ -3318,9 +3425,10 @@
       <c r="C92" s="15"/>
       <c r="D92" s="18"/>
       <c r="E92" s="19" t="str">
-        <f aca="false">IF(D92="","",D92*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D92="","",D92*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F92" s="15"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="14"/>
@@ -3328,9 +3436,10 @@
       <c r="C93" s="15"/>
       <c r="D93" s="18"/>
       <c r="E93" s="19" t="str">
-        <f aca="false">IF(D93="","",D93*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D93="","",D93*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F93" s="15"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="14"/>
@@ -3338,9 +3447,10 @@
       <c r="C94" s="15"/>
       <c r="D94" s="18"/>
       <c r="E94" s="19" t="str">
-        <f aca="false">IF(D94="","",D94*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D94="","",D94*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F94" s="15"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="14"/>
@@ -3348,9 +3458,10 @@
       <c r="C95" s="15"/>
       <c r="D95" s="18"/>
       <c r="E95" s="19" t="str">
-        <f aca="false">IF(D95="","",D95*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D95="","",D95*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F95" s="15"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="14"/>
@@ -3358,9 +3469,10 @@
       <c r="C96" s="15"/>
       <c r="D96" s="18"/>
       <c r="E96" s="19" t="str">
-        <f aca="false">IF(D96="","",D96*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D96="","",D96*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F96" s="15"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="14"/>
@@ -3368,9 +3480,10 @@
       <c r="C97" s="15"/>
       <c r="D97" s="18"/>
       <c r="E97" s="19" t="str">
-        <f aca="false">IF(D97="","",D97*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D97="","",D97*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F97" s="15"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="14"/>
@@ -3378,9 +3491,10 @@
       <c r="C98" s="15"/>
       <c r="D98" s="18"/>
       <c r="E98" s="19" t="str">
-        <f aca="false">IF(D98="","",D98*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D98="","",D98*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F98" s="15"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="14"/>
@@ -3388,9 +3502,10 @@
       <c r="C99" s="15"/>
       <c r="D99" s="18"/>
       <c r="E99" s="19" t="str">
-        <f aca="false">IF(D99="","",D99*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D99="","",D99*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F99" s="15"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="14"/>
@@ -3398,9 +3513,10 @@
       <c r="C100" s="15"/>
       <c r="D100" s="18"/>
       <c r="E100" s="19" t="str">
-        <f aca="false">IF(D100="","",D100*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D100="","",D100*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F100" s="15"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="14"/>
@@ -3408,9 +3524,10 @@
       <c r="C101" s="15"/>
       <c r="D101" s="18"/>
       <c r="E101" s="19" t="str">
-        <f aca="false">IF(D101="","",D101*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D101="","",D101*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F101" s="15"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="14"/>
@@ -3418,9 +3535,10 @@
       <c r="C102" s="15"/>
       <c r="D102" s="18"/>
       <c r="E102" s="19" t="str">
-        <f aca="false">IF(D102="","",D102*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D102="","",D102*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F102" s="15"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="14"/>
@@ -3428,9 +3546,10 @@
       <c r="C103" s="15"/>
       <c r="D103" s="18"/>
       <c r="E103" s="19" t="str">
-        <f aca="false">IF(D103="","",D103*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D103="","",D103*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F103" s="15"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="14"/>
@@ -3438,9 +3557,10 @@
       <c r="C104" s="15"/>
       <c r="D104" s="18"/>
       <c r="E104" s="19" t="str">
-        <f aca="false">IF(D104="","",D104*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D104="","",D104*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F104" s="15"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="14"/>
@@ -3448,9 +3568,10 @@
       <c r="C105" s="15"/>
       <c r="D105" s="18"/>
       <c r="E105" s="19" t="str">
-        <f aca="false">IF(D105="","",D105*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D105="","",D105*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F105" s="15"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="14"/>
@@ -3458,9 +3579,10 @@
       <c r="C106" s="15"/>
       <c r="D106" s="18"/>
       <c r="E106" s="19" t="str">
-        <f aca="false">IF(D106="","",D106*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D106="","",D106*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F106" s="15"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="14"/>
@@ -3468,9 +3590,10 @@
       <c r="C107" s="15"/>
       <c r="D107" s="18"/>
       <c r="E107" s="19" t="str">
-        <f aca="false">IF(D107="","",D107*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D107="","",D107*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F107" s="15"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="14"/>
@@ -3478,9 +3601,10 @@
       <c r="C108" s="15"/>
       <c r="D108" s="18"/>
       <c r="E108" s="19" t="str">
-        <f aca="false">IF(D108="","",D108*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D108="","",D108*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F108" s="15"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="14"/>
@@ -3488,9 +3612,10 @@
       <c r="C109" s="15"/>
       <c r="D109" s="18"/>
       <c r="E109" s="19" t="str">
-        <f aca="false">IF(D109="","",D109*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D109="","",D109*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F109" s="15"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="14"/>
@@ -3498,9 +3623,10 @@
       <c r="C110" s="15"/>
       <c r="D110" s="18"/>
       <c r="E110" s="19" t="str">
-        <f aca="false">IF(D110="","",D110*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D110="","",D110*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F110" s="15"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="14"/>
@@ -3508,9 +3634,10 @@
       <c r="C111" s="15"/>
       <c r="D111" s="18"/>
       <c r="E111" s="19" t="str">
-        <f aca="false">IF(D111="","",D111*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D111="","",D111*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F111" s="15"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="14"/>
@@ -3518,9 +3645,10 @@
       <c r="C112" s="15"/>
       <c r="D112" s="18"/>
       <c r="E112" s="19" t="str">
-        <f aca="false">IF(D112="","",D112*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D112="","",D112*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F112" s="15"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="14"/>
@@ -3528,9 +3656,10 @@
       <c r="C113" s="15"/>
       <c r="D113" s="18"/>
       <c r="E113" s="19" t="str">
-        <f aca="false">IF(D113="","",D113*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D113="","",D113*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F113" s="15"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="14"/>
@@ -3538,9 +3667,10 @@
       <c r="C114" s="15"/>
       <c r="D114" s="18"/>
       <c r="E114" s="19" t="str">
-        <f aca="false">IF(D114="","",D114*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D114="","",D114*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F114" s="15"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="14"/>
@@ -3548,9 +3678,10 @@
       <c r="C115" s="15"/>
       <c r="D115" s="18"/>
       <c r="E115" s="19" t="str">
-        <f aca="false">IF(D115="","",D115*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D115="","",D115*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F115" s="15"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="14"/>
@@ -3558,9 +3689,10 @@
       <c r="C116" s="15"/>
       <c r="D116" s="18"/>
       <c r="E116" s="19" t="str">
-        <f aca="false">IF(D116="","",D116*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D116="","",D116*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F116" s="15"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="14"/>
@@ -3568,9 +3700,10 @@
       <c r="C117" s="15"/>
       <c r="D117" s="18"/>
       <c r="E117" s="19" t="str">
-        <f aca="false">IF(D117="","",D117*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D117="","",D117*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F117" s="15"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="14"/>
@@ -3578,9 +3711,10 @@
       <c r="C118" s="15"/>
       <c r="D118" s="18"/>
       <c r="E118" s="19" t="str">
-        <f aca="false">IF(D118="","",D118*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D118="","",D118*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F118" s="15"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="14"/>
@@ -3588,9 +3722,10 @@
       <c r="C119" s="15"/>
       <c r="D119" s="18"/>
       <c r="E119" s="19" t="str">
-        <f aca="false">IF(D119="","",D119*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D119="","",D119*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F119" s="15"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="14"/>
@@ -3598,9 +3733,10 @@
       <c r="C120" s="15"/>
       <c r="D120" s="18"/>
       <c r="E120" s="19" t="str">
-        <f aca="false">IF(D120="","",D120*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D120="","",D120*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F120" s="15"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="14"/>
@@ -3608,9 +3744,10 @@
       <c r="C121" s="15"/>
       <c r="D121" s="18"/>
       <c r="E121" s="19" t="str">
-        <f aca="false">IF(D121="","",D121*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D121="","",D121*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F121" s="15"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="14"/>
@@ -3618,9 +3755,10 @@
       <c r="C122" s="15"/>
       <c r="D122" s="18"/>
       <c r="E122" s="19" t="str">
-        <f aca="false">IF(D122="","",D122*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D122="","",D122*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F122" s="15"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="14"/>
@@ -3628,9 +3766,10 @@
       <c r="C123" s="15"/>
       <c r="D123" s="18"/>
       <c r="E123" s="19" t="str">
-        <f aca="false">IF(D123="","",D123*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D123="","",D123*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F123" s="15"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="14"/>
@@ -3638,9 +3777,10 @@
       <c r="C124" s="15"/>
       <c r="D124" s="18"/>
       <c r="E124" s="19" t="str">
-        <f aca="false">IF(D124="","",D124*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D124="","",D124*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F124" s="15"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="14"/>
@@ -3648,9 +3788,10 @@
       <c r="C125" s="15"/>
       <c r="D125" s="18"/>
       <c r="E125" s="19" t="str">
-        <f aca="false">IF(D125="","",D125*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D125="","",D125*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F125" s="15"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="14"/>
@@ -3658,9 +3799,10 @@
       <c r="C126" s="15"/>
       <c r="D126" s="18"/>
       <c r="E126" s="19" t="str">
-        <f aca="false">IF(D126="","",D126*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D126="","",D126*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F126" s="15"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="14"/>
@@ -3668,9 +3810,10 @@
       <c r="C127" s="15"/>
       <c r="D127" s="18"/>
       <c r="E127" s="19" t="str">
-        <f aca="false">IF(D127="","",D127*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D127="","",D127*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F127" s="15"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="14"/>
@@ -3678,9 +3821,10 @@
       <c r="C128" s="15"/>
       <c r="D128" s="18"/>
       <c r="E128" s="19" t="str">
-        <f aca="false">IF(D128="","",D128*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D128="","",D128*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F128" s="15"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="14"/>
@@ -3688,9 +3832,10 @@
       <c r="C129" s="15"/>
       <c r="D129" s="18"/>
       <c r="E129" s="19" t="str">
-        <f aca="false">IF(D129="","",D129*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D129="","",D129*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F129" s="15"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="14"/>
@@ -3698,9 +3843,10 @@
       <c r="C130" s="15"/>
       <c r="D130" s="18"/>
       <c r="E130" s="19" t="str">
-        <f aca="false">IF(D130="","",D130*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D130="","",D130*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F130" s="15"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="14"/>
@@ -3708,9 +3854,10 @@
       <c r="C131" s="15"/>
       <c r="D131" s="18"/>
       <c r="E131" s="19" t="str">
-        <f aca="false">IF(D131="","",D131*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D131="","",D131*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F131" s="15"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="14"/>
@@ -3718,9 +3865,10 @@
       <c r="C132" s="15"/>
       <c r="D132" s="18"/>
       <c r="E132" s="19" t="str">
-        <f aca="false">IF(D132="","",D132*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D132="","",D132*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F132" s="15"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="14"/>
@@ -3728,9 +3876,10 @@
       <c r="C133" s="15"/>
       <c r="D133" s="18"/>
       <c r="E133" s="19" t="str">
-        <f aca="false">IF(D133="","",D133*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D133="","",D133*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F133" s="15"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="14"/>
@@ -3738,9 +3887,10 @@
       <c r="C134" s="15"/>
       <c r="D134" s="18"/>
       <c r="E134" s="19" t="str">
-        <f aca="false">IF(D134="","",D134*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D134="","",D134*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F134" s="15"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="14"/>
@@ -3748,9 +3898,10 @@
       <c r="C135" s="15"/>
       <c r="D135" s="18"/>
       <c r="E135" s="19" t="str">
-        <f aca="false">IF(D135="","",D135*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D135="","",D135*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F135" s="15"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="14"/>
@@ -3758,9 +3909,10 @@
       <c r="C136" s="15"/>
       <c r="D136" s="18"/>
       <c r="E136" s="19" t="str">
-        <f aca="false">IF(D136="","",D136*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D136="","",D136*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F136" s="15"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="14"/>
@@ -3768,9 +3920,10 @@
       <c r="C137" s="15"/>
       <c r="D137" s="18"/>
       <c r="E137" s="19" t="str">
-        <f aca="false">IF(D137="","",D137*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D137="","",D137*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F137" s="15"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="14"/>
@@ -3778,9 +3931,10 @@
       <c r="C138" s="15"/>
       <c r="D138" s="18"/>
       <c r="E138" s="19" t="str">
-        <f aca="false">IF(D138="","",D138*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D138="","",D138*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F138" s="15"/>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="14"/>
@@ -3788,9 +3942,10 @@
       <c r="C139" s="15"/>
       <c r="D139" s="18"/>
       <c r="E139" s="19" t="str">
-        <f aca="false">IF(D139="","",D139*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D139="","",D139*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F139" s="15"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="14"/>
@@ -3798,9 +3953,10 @@
       <c r="C140" s="15"/>
       <c r="D140" s="18"/>
       <c r="E140" s="19" t="str">
-        <f aca="false">IF(D140="","",D140*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D140="","",D140*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F140" s="15"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="14"/>
@@ -3808,9 +3964,10 @@
       <c r="C141" s="15"/>
       <c r="D141" s="18"/>
       <c r="E141" s="19" t="str">
-        <f aca="false">IF(D141="","",D141*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D141="","",D141*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F141" s="15"/>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="14"/>
@@ -3818,9 +3975,10 @@
       <c r="C142" s="15"/>
       <c r="D142" s="18"/>
       <c r="E142" s="19" t="str">
-        <f aca="false">IF(D142="","",D142*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D142="","",D142*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F142" s="15"/>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="14"/>
@@ -3828,9 +3986,10 @@
       <c r="C143" s="15"/>
       <c r="D143" s="18"/>
       <c r="E143" s="19" t="str">
-        <f aca="false">IF(D143="","",D143*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D143="","",D143*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F143" s="15"/>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="14"/>
@@ -3838,9 +3997,10 @@
       <c r="C144" s="15"/>
       <c r="D144" s="18"/>
       <c r="E144" s="19" t="str">
-        <f aca="false">IF(D144="","",D144*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D144="","",D144*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F144" s="15"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="14"/>
@@ -3848,9 +4008,10 @@
       <c r="C145" s="15"/>
       <c r="D145" s="18"/>
       <c r="E145" s="19" t="str">
-        <f aca="false">IF(D145="","",D145*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D145="","",D145*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F145" s="15"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="14"/>
@@ -3858,9 +4019,10 @@
       <c r="C146" s="15"/>
       <c r="D146" s="18"/>
       <c r="E146" s="19" t="str">
-        <f aca="false">IF(D146="","",D146*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D146="","",D146*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F146" s="15"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="14"/>
@@ -3868,9 +4030,10 @@
       <c r="C147" s="15"/>
       <c r="D147" s="18"/>
       <c r="E147" s="19" t="str">
-        <f aca="false">IF(D147="","",D147*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D147="","",D147*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F147" s="15"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="14"/>
@@ -3878,9 +4041,10 @@
       <c r="C148" s="15"/>
       <c r="D148" s="18"/>
       <c r="E148" s="19" t="str">
-        <f aca="false">IF(D148="","",D148*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D148="","",D148*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F148" s="15"/>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="14"/>
@@ -3888,9 +4052,10 @@
       <c r="C149" s="15"/>
       <c r="D149" s="18"/>
       <c r="E149" s="19" t="str">
-        <f aca="false">IF(D149="","",D149*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D149="","",D149*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F149" s="15"/>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="14"/>
@@ -3898,9 +4063,10 @@
       <c r="C150" s="15"/>
       <c r="D150" s="18"/>
       <c r="E150" s="19" t="str">
-        <f aca="false">IF(D150="","",D150*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D150="","",D150*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F150" s="15"/>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="14"/>
@@ -3908,9 +4074,10 @@
       <c r="C151" s="15"/>
       <c r="D151" s="18"/>
       <c r="E151" s="19" t="str">
-        <f aca="false">IF(D151="","",D151*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D151="","",D151*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F151" s="15"/>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="14"/>
@@ -3918,9 +4085,10 @@
       <c r="C152" s="15"/>
       <c r="D152" s="18"/>
       <c r="E152" s="19" t="str">
-        <f aca="false">IF(D152="","",D152*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D152="","",D152*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F152" s="15"/>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="14"/>
@@ -3928,9 +4096,10 @@
       <c r="C153" s="15"/>
       <c r="D153" s="18"/>
       <c r="E153" s="19" t="str">
-        <f aca="false">IF(D153="","",D153*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D153="","",D153*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F153" s="15"/>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="14"/>
@@ -3938,9 +4107,10 @@
       <c r="C154" s="15"/>
       <c r="D154" s="18"/>
       <c r="E154" s="19" t="str">
-        <f aca="false">IF(D154="","",D154*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D154="","",D154*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F154" s="15"/>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="14"/>
@@ -3948,9 +4118,10 @@
       <c r="C155" s="15"/>
       <c r="D155" s="18"/>
       <c r="E155" s="19" t="str">
-        <f aca="false">IF(D155="","",D155*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D155="","",D155*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F155" s="15"/>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="14"/>
@@ -3958,9 +4129,10 @@
       <c r="C156" s="15"/>
       <c r="D156" s="18"/>
       <c r="E156" s="19" t="str">
-        <f aca="false">IF(D156="","",D156*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D156="","",D156*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F156" s="15"/>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="14"/>
@@ -3968,9 +4140,10 @@
       <c r="C157" s="15"/>
       <c r="D157" s="18"/>
       <c r="E157" s="19" t="str">
-        <f aca="false">IF(D157="","",D157*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D157="","",D157*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F157" s="15"/>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="14"/>
@@ -3978,9 +4151,10 @@
       <c r="C158" s="15"/>
       <c r="D158" s="18"/>
       <c r="E158" s="19" t="str">
-        <f aca="false">IF(D158="","",D158*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D158="","",D158*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F158" s="15"/>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="14"/>
@@ -3988,9 +4162,10 @@
       <c r="C159" s="15"/>
       <c r="D159" s="18"/>
       <c r="E159" s="19" t="str">
-        <f aca="false">IF(D159="","",D159*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D159="","",D159*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F159" s="15"/>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="14"/>
@@ -3998,9 +4173,10 @@
       <c r="C160" s="15"/>
       <c r="D160" s="18"/>
       <c r="E160" s="19" t="str">
-        <f aca="false">IF(D160="","",D160*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D160="","",D160*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F160" s="15"/>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="14"/>
@@ -4008,9 +4184,10 @@
       <c r="C161" s="15"/>
       <c r="D161" s="18"/>
       <c r="E161" s="19" t="str">
-        <f aca="false">IF(D161="","",D161*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D161="","",D161*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F161" s="15"/>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="14"/>
@@ -4018,9 +4195,10 @@
       <c r="C162" s="15"/>
       <c r="D162" s="18"/>
       <c r="E162" s="19" t="str">
-        <f aca="false">IF(D162="","",D162*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D162="","",D162*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F162" s="15"/>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="14"/>
@@ -4028,9 +4206,10 @@
       <c r="C163" s="15"/>
       <c r="D163" s="18"/>
       <c r="E163" s="19" t="str">
-        <f aca="false">IF(D163="","",D163*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D163="","",D163*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F163" s="15"/>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="14"/>
@@ -4038,9 +4217,10 @@
       <c r="C164" s="15"/>
       <c r="D164" s="18"/>
       <c r="E164" s="19" t="str">
-        <f aca="false">IF(D164="","",D164*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D164="","",D164*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F164" s="15"/>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="14"/>
@@ -4048,9 +4228,10 @@
       <c r="C165" s="15"/>
       <c r="D165" s="18"/>
       <c r="E165" s="19" t="str">
-        <f aca="false">IF(D165="","",D165*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D165="","",D165*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F165" s="15"/>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="14"/>
@@ -4058,9 +4239,10 @@
       <c r="C166" s="15"/>
       <c r="D166" s="18"/>
       <c r="E166" s="19" t="str">
-        <f aca="false">IF(D166="","",D166*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D166="","",D166*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F166" s="15"/>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="14"/>
@@ -4068,9 +4250,10 @@
       <c r="C167" s="15"/>
       <c r="D167" s="18"/>
       <c r="E167" s="19" t="str">
-        <f aca="false">IF(D167="","",D167*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D167="","",D167*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F167" s="15"/>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="14"/>
@@ -4078,9 +4261,10 @@
       <c r="C168" s="15"/>
       <c r="D168" s="18"/>
       <c r="E168" s="19" t="str">
-        <f aca="false">IF(D168="","",D168*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D168="","",D168*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F168" s="15"/>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="14"/>
@@ -4088,9 +4272,10 @@
       <c r="C169" s="15"/>
       <c r="D169" s="18"/>
       <c r="E169" s="19" t="str">
-        <f aca="false">IF(D169="","",D169*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D169="","",D169*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F169" s="15"/>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="14"/>
@@ -4098,9 +4283,10 @@
       <c r="C170" s="15"/>
       <c r="D170" s="18"/>
       <c r="E170" s="19" t="str">
-        <f aca="false">IF(D170="","",D170*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D170="","",D170*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F170" s="15"/>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="14"/>
@@ -4108,9 +4294,10 @@
       <c r="C171" s="15"/>
       <c r="D171" s="18"/>
       <c r="E171" s="19" t="str">
-        <f aca="false">IF(D171="","",D171*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D171="","",D171*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F171" s="15"/>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="14"/>
@@ -4118,9 +4305,10 @@
       <c r="C172" s="15"/>
       <c r="D172" s="18"/>
       <c r="E172" s="19" t="str">
-        <f aca="false">IF(D172="","",D172*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D172="","",D172*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F172" s="15"/>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="14"/>
@@ -4128,9 +4316,10 @@
       <c r="C173" s="15"/>
       <c r="D173" s="18"/>
       <c r="E173" s="19" t="str">
-        <f aca="false">IF(D173="","",D173*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D173="","",D173*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F173" s="15"/>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="14"/>
@@ -4138,9 +4327,10 @@
       <c r="C174" s="15"/>
       <c r="D174" s="18"/>
       <c r="E174" s="19" t="str">
-        <f aca="false">IF(D174="","",D174*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D174="","",D174*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F174" s="15"/>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="14"/>
@@ -4148,9 +4338,10 @@
       <c r="C175" s="15"/>
       <c r="D175" s="18"/>
       <c r="E175" s="19" t="str">
-        <f aca="false">IF(D175="","",D175*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D175="","",D175*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F175" s="15"/>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="14"/>
@@ -4158,9 +4349,10 @@
       <c r="C176" s="15"/>
       <c r="D176" s="18"/>
       <c r="E176" s="19" t="str">
-        <f aca="false">IF(D176="","",D176*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D176="","",D176*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F176" s="15"/>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="14"/>
@@ -4168,9 +4360,10 @@
       <c r="C177" s="15"/>
       <c r="D177" s="18"/>
       <c r="E177" s="19" t="str">
-        <f aca="false">IF(D177="","",D177*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D177="","",D177*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F177" s="15"/>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="14"/>
@@ -4178,9 +4371,10 @@
       <c r="C178" s="15"/>
       <c r="D178" s="18"/>
       <c r="E178" s="19" t="str">
-        <f aca="false">IF(D178="","",D178*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D178="","",D178*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F178" s="15"/>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="14"/>
@@ -4188,9 +4382,10 @@
       <c r="C179" s="15"/>
       <c r="D179" s="18"/>
       <c r="E179" s="19" t="str">
-        <f aca="false">IF(D179="","",D179*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D179="","",D179*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F179" s="15"/>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="14"/>
@@ -4198,9 +4393,10 @@
       <c r="C180" s="15"/>
       <c r="D180" s="18"/>
       <c r="E180" s="19" t="str">
-        <f aca="false">IF(D180="","",D180*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D180="","",D180*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F180" s="15"/>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="14"/>
@@ -4208,9 +4404,10 @@
       <c r="C181" s="15"/>
       <c r="D181" s="18"/>
       <c r="E181" s="19" t="str">
-        <f aca="false">IF(D181="","",D181*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D181="","",D181*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F181" s="15"/>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="14"/>
@@ -4218,9 +4415,10 @@
       <c r="C182" s="15"/>
       <c r="D182" s="18"/>
       <c r="E182" s="19" t="str">
-        <f aca="false">IF(D182="","",D182*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D182="","",D182*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F182" s="15"/>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="14"/>
@@ -4228,9 +4426,10 @@
       <c r="C183" s="15"/>
       <c r="D183" s="18"/>
       <c r="E183" s="19" t="str">
-        <f aca="false">IF(D183="","",D183*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D183="","",D183*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F183" s="15"/>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="14"/>
@@ -4238,9 +4437,10 @@
       <c r="C184" s="15"/>
       <c r="D184" s="18"/>
       <c r="E184" s="19" t="str">
-        <f aca="false">IF(D184="","",D184*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D184="","",D184*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F184" s="15"/>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="14"/>
@@ -4248,9 +4448,10 @@
       <c r="C185" s="15"/>
       <c r="D185" s="18"/>
       <c r="E185" s="19" t="str">
-        <f aca="false">IF(D185="","",D185*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D185="","",D185*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F185" s="15"/>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="14"/>
@@ -4258,9 +4459,10 @@
       <c r="C186" s="15"/>
       <c r="D186" s="18"/>
       <c r="E186" s="19" t="str">
-        <f aca="false">IF(D186="","",D186*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D186="","",D186*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F186" s="15"/>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="14"/>
@@ -4268,9 +4470,10 @@
       <c r="C187" s="15"/>
       <c r="D187" s="18"/>
       <c r="E187" s="19" t="str">
-        <f aca="false">IF(D187="","",D187*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D187="","",D187*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F187" s="15"/>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="14"/>
@@ -4278,9 +4481,10 @@
       <c r="C188" s="15"/>
       <c r="D188" s="18"/>
       <c r="E188" s="19" t="str">
-        <f aca="false">IF(D188="","",D188*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D188="","",D188*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F188" s="15"/>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="14"/>
@@ -4288,9 +4492,10 @@
       <c r="C189" s="15"/>
       <c r="D189" s="18"/>
       <c r="E189" s="19" t="str">
-        <f aca="false">IF(D189="","",D189*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D189="","",D189*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F189" s="15"/>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="14"/>
@@ -4298,9 +4503,10 @@
       <c r="C190" s="15"/>
       <c r="D190" s="18"/>
       <c r="E190" s="19" t="str">
-        <f aca="false">IF(D190="","",D190*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D190="","",D190*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F190" s="15"/>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="14"/>
@@ -4308,9 +4514,10 @@
       <c r="C191" s="15"/>
       <c r="D191" s="18"/>
       <c r="E191" s="19" t="str">
-        <f aca="false">IF(D191="","",D191*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D191="","",D191*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F191" s="15"/>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="14"/>
@@ -4318,9 +4525,10 @@
       <c r="C192" s="15"/>
       <c r="D192" s="18"/>
       <c r="E192" s="19" t="str">
-        <f aca="false">IF(D192="","",D192*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D192="","",D192*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F192" s="15"/>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="14"/>
@@ -4328,9 +4536,10 @@
       <c r="C193" s="15"/>
       <c r="D193" s="18"/>
       <c r="E193" s="19" t="str">
-        <f aca="false">IF(D193="","",D193*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D193="","",D193*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F193" s="15"/>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="14"/>
@@ -4338,9 +4547,10 @@
       <c r="C194" s="15"/>
       <c r="D194" s="18"/>
       <c r="E194" s="19" t="str">
-        <f aca="false">IF(D194="","",D194*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D194="","",D194*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F194" s="15"/>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="14"/>
@@ -4348,9 +4558,10 @@
       <c r="C195" s="15"/>
       <c r="D195" s="18"/>
       <c r="E195" s="19" t="str">
-        <f aca="false">IF(D195="","",D195*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D195="","",D195*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F195" s="15"/>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="14"/>
@@ -4358,9 +4569,10 @@
       <c r="C196" s="15"/>
       <c r="D196" s="18"/>
       <c r="E196" s="19" t="str">
-        <f aca="false">IF(D196="","",D196*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D196="","",D196*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F196" s="15"/>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="14"/>
@@ -4368,9 +4580,10 @@
       <c r="C197" s="15"/>
       <c r="D197" s="18"/>
       <c r="E197" s="19" t="str">
-        <f aca="false">IF(D197="","",D197*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D197="","",D197*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F197" s="15"/>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="14"/>
@@ -4378,9 +4591,10 @@
       <c r="C198" s="15"/>
       <c r="D198" s="18"/>
       <c r="E198" s="19" t="str">
-        <f aca="false">IF(D198="","",D198*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D198="","",D198*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F198" s="15"/>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="14"/>
@@ -4388,9 +4602,10 @@
       <c r="C199" s="15"/>
       <c r="D199" s="18"/>
       <c r="E199" s="19" t="str">
-        <f aca="false">IF(D199="","",D199*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D199="","",D199*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F199" s="15"/>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="14"/>
@@ -4398,9 +4613,10 @@
       <c r="C200" s="15"/>
       <c r="D200" s="18"/>
       <c r="E200" s="19" t="str">
-        <f aca="false">IF(D200="","",D200*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D200="","",D200*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F200" s="15"/>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="14"/>
@@ -4408,9 +4624,10 @@
       <c r="C201" s="15"/>
       <c r="D201" s="18"/>
       <c r="E201" s="19" t="str">
-        <f aca="false">IF(D201="","",D201*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D201="","",D201*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F201" s="15"/>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="14"/>
@@ -4418,9 +4635,10 @@
       <c r="C202" s="15"/>
       <c r="D202" s="18"/>
       <c r="E202" s="19" t="str">
-        <f aca="false">IF(D202="","",D202*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D202="","",D202*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F202" s="15"/>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="14"/>
@@ -4428,9 +4646,10 @@
       <c r="C203" s="15"/>
       <c r="D203" s="18"/>
       <c r="E203" s="19" t="str">
-        <f aca="false">IF(D203="","",D203*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D203="","",D203*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F203" s="15"/>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="14"/>
@@ -4438,14 +4657,19 @@
       <c r="C204" s="15"/>
       <c r="D204" s="18"/>
       <c r="E204" s="19" t="str">
-        <f aca="false">IF(D204="","",D204*$H$6)</f>
-        <v/>
-      </c>
+        <f aca="false">IF(D204="","",D204*$I$8)</f>
+        <v/>
+      </c>
+      <c r="F204" s="15"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation allowBlank="true" error="Elegí un componente de la lista." errorStyle="stop" errorTitle="Componente inválido" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B5:B204" type="list">
       <formula1>"Agus C.,Agus M.,Boli,Cami,Flopa,Katy,Luci,Mai,María,Marti,Paz,Vicky"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F204" type="list">
+      <formula1>"Sí,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>